<commit_message>
auto update (5 cells, +83, -4)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -7,12 +7,12 @@
     <sheet sheetId="1" name="المتعاقدين الحالين حتى 10-2026" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="الغير متعاقدين حتى 10-2026" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2332" uniqueCount="741">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2502" uniqueCount="911">
   <si>
     <t xml:space="preserve">الاجمالى </t>
   </si>
@@ -2235,6 +2235,516 @@
   </si>
   <si>
     <t>وفاه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد محمد احمد احمد مؤنس (عقد حتى 14-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عبدالعظيم مبروك خميس (عقد حتى 14-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">طارق عباس محمود على (عقد حتى 9-4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ايمن رمزى إبراهيم هيكل (عقد حتى 31-3 )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد صالح محمد الخولى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">خميس محمد محمد جبريل</t>
+  </si>
+  <si>
+    <t xml:space="preserve">التبريد والتهوية خط 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">جمال الدين على محمد عطوه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">هشام محمد بهجت عبدالفتاح</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فنى صيانة</t>
+  </si>
+  <si>
+    <t xml:space="preserve">طلعت احمد السيد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">حرفى مؤقت</t>
+  </si>
+  <si>
+    <t xml:space="preserve">المكتب الفني للهندسة الكهربائية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ماهر سعد مصطفى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">إيرادات الركاب</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد حسين عبد العزيز حسين خاطر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مهندس استشارى قسم الاعطال</t>
+  </si>
+  <si>
+    <t xml:space="preserve">السلامة والجودةلعمليات التشغيل</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 شهر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ابراهيم بخيت عبدالرحيم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اخصائي امن (مدير عام ادارة الامن)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الامن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 شهر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عادل عطيتو عادل احمد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سمير عزيز اسكندر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">وحدات متحركة خط اول</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 شهر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عاطف عبد الستار محمد سلام</t>
+  </si>
+  <si>
+    <t xml:space="preserve">امن بوابات</t>
+  </si>
+  <si>
+    <t xml:space="preserve">إدارة الامن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">احمد صالح عبد الغنى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">احمد احمد سليمان شحاتة</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمود سيد احمد احمد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فنى بالتحكم المركزى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">التحكم المركزى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">لملوم عبدالعزيز عبدالرحمن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عاطف احمد جاد الله</t>
+  </si>
+  <si>
+    <t xml:space="preserve">جرجس فهمى جرجس شنوده</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عادل قمصان مرسى ريحان</t>
+  </si>
+  <si>
+    <t xml:space="preserve">هندسة سكه -جسم النفق</t>
+  </si>
+  <si>
+    <t xml:space="preserve">احمد امين محمد عبدالجواد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">صراف تذاكر مؤقت</t>
+  </si>
+  <si>
+    <t xml:space="preserve">استشارى بالقوى الكهربائية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">القوى الكهربائية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد احمد ابراهيم الغرباوى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اخصائى صيانة مدنية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الصيانة المدنية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد احمد ذكى مرسي</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اخصائي اشارات وتحكم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الإشارات والتحكم خط اول</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رؤوف فايق سلامه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اخصائي ميكانيكا (مدير عام هندسة السكة)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">هندسة السكة</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 شهر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عماد الدين عبد الرؤوف حماد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">طبيب</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الإدارة الطبية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اشرف على مصطفى دبور</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ملاحظ تشغيل</t>
+  </si>
+  <si>
+    <t xml:space="preserve">تشغيل خط اول</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مصطفى دسوقي على عمر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قوى كهربائية - خط اول</t>
+  </si>
+  <si>
+    <t xml:space="preserve">شعبان الوصال على على</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عبد المنعم حمزه جمال الدين</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اخصائي اسعاف</t>
+  </si>
+  <si>
+    <t xml:space="preserve">طارق عبد المجيد محمد السيد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سيد احمد عبدالعزيز عبدالرحمن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">منقطع من يوم 2023/12/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد عبد المجيد نصر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">طبيب اسنان</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سيد عبدالمنعم محمود</t>
+  </si>
+  <si>
+    <t xml:space="preserve">منقطع من يوم 2023/11/11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عبدالناصر نادى احمد ابو المحسن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">انهاء تعاقد بتاريخ 2024/3/27 (لم تاتى موافقة بتجديد العقد )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد احمد سالم خليفه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">انقطاع ولم يجدد العقد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عبدالمقصود عيسى عبدالمقصود عيسى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اعتذار عن استلم العمل</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عادل عبدالمنعم حسنين محمد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">وحدات متحركة - خط اول</t>
+  </si>
+  <si>
+    <t xml:space="preserve">وفاة 2024/4/7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">حازم حسن مصطفى حسن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قائد قطار بالاحواش</t>
+  </si>
+  <si>
+    <t xml:space="preserve">انهاء تعاقد وعدم تجديد العقد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عبدالحميد عبدالفتاح عبدالفتاح حسين</t>
+  </si>
+  <si>
+    <t xml:space="preserve">انهاء تعاقد بتاريخ 2024/2/29 (للانقطاع)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد العبد عوض</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محامى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الشئون القانونية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">انهاء تعاقد بتاريخ 2024/6/27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد عبدالمنعم هاشم احمد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ملاحظ تشغيل السائقين</t>
+  </si>
+  <si>
+    <t xml:space="preserve">التشغيل اول</t>
+  </si>
+  <si>
+    <t xml:space="preserve">انهاء تعاقد للوفاه 4/9/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سالم محمد حسنين ابو عيضه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عاطف محمد الجوهرى عامر عبدالفتاح</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45295</t>
+  </si>
+  <si>
+    <t xml:space="preserve">على احمد على محمد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ميسه مصطفى حسن احمد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 شهر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45485</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ابراهيم عباس السيد على</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اخصائى تحكم المحطات الكهربائية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44581</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد عبدالعال محمد سليم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44957</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سعيد احمد محمد عبدالقادر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44166</t>
+  </si>
+  <si>
+    <t xml:space="preserve">احمد عبدالحافظ عبدالمنعم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اخصائى قوى كهربائية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44921</t>
+  </si>
+  <si>
+    <t xml:space="preserve">القوى الكهربائية - خط ثانى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">احمد عبدالفتاح حسين غنيه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمود عثمان على عثمان زيد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44312</t>
+  </si>
+  <si>
+    <t xml:space="preserve">بدر عبدالنعيم على ابراهيم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44234</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عبدالعزيز عبدالخالق السيد خليفه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">44659</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سلالم ومصاعد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عبدالرحمن عبدالقوى محمدهيكل</t>
+  </si>
+  <si>
+    <t xml:space="preserve">خبيير انظمة (ادارى)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">أنظمة القيادة - ورشة شبرا</t>
+  </si>
+  <si>
+    <t xml:space="preserve">يوسف عبدالحليم محمد سليمان</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 شهر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">حسن محمد عمر خلاف</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فنى تشغيل rs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">على احمد عبدالفتاح قايد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19781</t>
+  </si>
+  <si>
+    <t xml:space="preserve">السعيد ابراهيم رضوان حسن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فنى - اخصائى امن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22364</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ادارة الامن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سويلم عبدالمنعم عباس سويلم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">علاء حسن عطية عيد حسن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22394</t>
+  </si>
+  <si>
+    <t xml:space="preserve">موسى عبدالخالق موسي عفيفى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22145</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد عبدالسلام محمد عبدالعال</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سلطان عبدالرشيد عبدالغنى علي</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عبدالحكيم عبدالحميد أحمد سلطان</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23709</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عدلى يحيى طه سالم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مجدى على عبداللطيف شاهين</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22857</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ياسر محمود فهمى عبدالرحمن</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22943</t>
+  </si>
+  <si>
+    <t xml:space="preserve">احمد ابوالقاسم امين الدرقاوى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23740</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رأفت حسيني عبد الله سليمان</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22465</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 شهر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">حسين عبدالحميد عبدالعال</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23715</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محمد محمد محمود عزب</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22722</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عبدالله زكريا محمود البرعي</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ايرادات الركاب - خط ثان</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46157</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46130</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46145</t>
   </si>
 </sst>
 </file>
@@ -9377,30 +9887,20 @@
       <c r="G119" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="H119" s="10">
-        <v>45139</v>
-      </c>
+      <c r="H119" s="10"/>
       <c r="I119" s="11"/>
       <c r="J119" s="12"/>
       <c r="K119" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="L119" s="11">
-        <v>22510</v>
-      </c>
-      <c r="M119" s="11">
-        <v>45117</v>
-      </c>
+      <c r="L119" s="11"/>
+      <c r="M119" s="11"/>
       <c r="N119" s="13"/>
       <c r="O119" s="7"/>
-      <c r="P119" s="13">
-        <v>26108171301291</v>
-      </c>
+      <c r="P119" s="13"/>
       <c r="Q119" s="16"/>
       <c r="R119" s="15"/>
-      <c r="S119" s="7" t="s">
-        <v>349</v>
-      </c>
+      <c r="S119" s="7"/>
     </row>
     <row r="120" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A120" s="7">
@@ -9424,36 +9924,20 @@
       <c r="G120" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="H120" s="10">
-        <v>45263</v>
-      </c>
-      <c r="I120" s="11">
-        <v>45629</v>
-      </c>
-      <c r="J120" s="12">
-        <v>45720</v>
-      </c>
+      <c r="H120" s="10"/>
+      <c r="I120" s="11"/>
+      <c r="J120" s="12"/>
       <c r="K120" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="L120" s="11">
-        <v>21886</v>
-      </c>
-      <c r="M120" s="11">
-        <v>43801</v>
-      </c>
+      <c r="L120" s="11"/>
+      <c r="M120" s="11"/>
       <c r="N120" s="13"/>
-      <c r="O120" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="P120" s="13">
-        <v>25912021300059</v>
-      </c>
+      <c r="O120" s="7"/>
+      <c r="P120" s="13"/>
       <c r="Q120" s="16"/>
       <c r="R120" s="15"/>
-      <c r="S120" s="7" t="s">
-        <v>349</v>
-      </c>
+      <c r="S120" s="7"/>
     </row>
     <row r="121" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A121" s="7">
@@ -9477,30 +9961,20 @@
       <c r="G121" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="H121" s="10">
-        <v>44805</v>
-      </c>
+      <c r="H121" s="10"/>
       <c r="I121" s="11"/>
       <c r="J121" s="12"/>
       <c r="K121" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="L121" s="11">
-        <v>22944</v>
-      </c>
-      <c r="M121" s="11">
-        <v>44859</v>
-      </c>
+      <c r="L121" s="11"/>
+      <c r="M121" s="11"/>
       <c r="N121" s="13"/>
       <c r="O121" s="7"/>
-      <c r="P121" s="13">
-        <v>26210251400258</v>
-      </c>
+      <c r="P121" s="13"/>
       <c r="Q121" s="16"/>
       <c r="R121" s="15"/>
-      <c r="S121" s="7" t="s">
-        <v>349</v>
-      </c>
+      <c r="S121" s="7"/>
     </row>
     <row r="122" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A122" s="7">
@@ -9524,30 +9998,20 @@
       <c r="G122" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="H122" s="10">
-        <v>44814</v>
-      </c>
+      <c r="H122" s="10"/>
       <c r="I122" s="11"/>
       <c r="J122" s="12"/>
       <c r="K122" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="L122" s="11">
-        <v>21539</v>
-      </c>
-      <c r="M122" s="11">
-        <v>43454</v>
-      </c>
+      <c r="L122" s="11"/>
+      <c r="M122" s="11"/>
       <c r="N122" s="13"/>
       <c r="O122" s="7"/>
-      <c r="P122" s="13">
-        <v>25812208800538</v>
-      </c>
+      <c r="P122" s="13"/>
       <c r="Q122" s="16"/>
       <c r="R122" s="15"/>
-      <c r="S122" s="7" t="s">
-        <v>349</v>
-      </c>
+      <c r="S122" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:S122"/>
@@ -9564,7 +10028,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S189"/>
+  <dimension ref="A1:S268"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -9592,7 +10056,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D189)</f>
-        <v>187</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -11759,7 +12223,7 @@
         <v>121</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>441</v>
+        <v>741</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>20</v>
@@ -11816,7 +12280,7 @@
         <v>125</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>444</v>
+        <v>742</v>
       </c>
       <c r="E40" s="7" t="s">
         <v>20</v>
@@ -12866,7 +13330,7 @@
         <v>103</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>485</v>
+        <v>743</v>
       </c>
       <c r="E58" s="7" t="s">
         <v>20</v>
@@ -15440,7 +15904,7 @@
         <v>191</v>
       </c>
       <c r="D102" s="9" t="s">
-        <v>581</v>
+        <v>744</v>
       </c>
       <c r="E102" s="7" t="s">
         <v>20</v>
@@ -20135,9 +20599,7 @@
       <c r="R185" s="15" t="s">
         <v>732</v>
       </c>
-      <c r="S185" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S185" s="7"/>
     </row>
     <row r="186" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A186" s="7">
@@ -20339,8 +20801,3555 @@
         <v>740</v>
       </c>
     </row>
+    <row r="190" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A190" s="7">
+        <v>188</v>
+      </c>
+      <c r="B190" s="7">
+        <v>20274</v>
+      </c>
+      <c r="C190" s="8">
+        <v>19</v>
+      </c>
+      <c r="D190" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="E190" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F190" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="G190" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H190" s="10">
+        <v>45139</v>
+      </c>
+      <c r="I190" s="11"/>
+      <c r="J190" s="12"/>
+      <c r="K190" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L190" s="11">
+        <v>22510</v>
+      </c>
+      <c r="M190" s="11">
+        <v>45117</v>
+      </c>
+      <c r="N190" s="13"/>
+      <c r="O190" s="7"/>
+      <c r="P190" s="13">
+        <v>26108171301291</v>
+      </c>
+      <c r="Q190" s="14"/>
+      <c r="R190" s="15"/>
+      <c r="S190" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="191" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A191" s="7">
+        <v>189</v>
+      </c>
+      <c r="B191" s="7">
+        <v>20276</v>
+      </c>
+      <c r="C191" s="8">
+        <v>56</v>
+      </c>
+      <c r="D191" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="E191" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F191" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G191" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H191" s="10">
+        <v>45263</v>
+      </c>
+      <c r="I191" s="11">
+        <v>45629</v>
+      </c>
+      <c r="J191" s="12">
+        <v>45720</v>
+      </c>
+      <c r="K191" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L191" s="11">
+        <v>21886</v>
+      </c>
+      <c r="M191" s="11">
+        <v>43801</v>
+      </c>
+      <c r="N191" s="13"/>
+      <c r="O191" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P191" s="13">
+        <v>25912021300059</v>
+      </c>
+      <c r="Q191" s="14"/>
+      <c r="R191" s="15"/>
+      <c r="S191" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="192" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A192" s="7">
+        <v>190</v>
+      </c>
+      <c r="B192" s="7">
+        <v>20211</v>
+      </c>
+      <c r="C192" s="8">
+        <v>151</v>
+      </c>
+      <c r="D192" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="E192" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F192" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G192" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H192" s="10">
+        <v>44805</v>
+      </c>
+      <c r="I192" s="11"/>
+      <c r="J192" s="12"/>
+      <c r="K192" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L192" s="11">
+        <v>22944</v>
+      </c>
+      <c r="M192" s="11">
+        <v>44859</v>
+      </c>
+      <c r="N192" s="13"/>
+      <c r="O192" s="7"/>
+      <c r="P192" s="13">
+        <v>26210251400258</v>
+      </c>
+      <c r="Q192" s="14"/>
+      <c r="R192" s="15"/>
+      <c r="S192" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="193" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A193" s="7">
+        <v>191</v>
+      </c>
+      <c r="B193" s="7">
+        <v>20212</v>
+      </c>
+      <c r="C193" s="8">
+        <v>152</v>
+      </c>
+      <c r="D193" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="E193" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F193" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G193" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H193" s="10">
+        <v>44814</v>
+      </c>
+      <c r="I193" s="11"/>
+      <c r="J193" s="12"/>
+      <c r="K193" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L193" s="11">
+        <v>21539</v>
+      </c>
+      <c r="M193" s="11">
+        <v>43454</v>
+      </c>
+      <c r="N193" s="13"/>
+      <c r="O193" s="7"/>
+      <c r="P193" s="13">
+        <v>25812208800538</v>
+      </c>
+      <c r="Q193" s="14"/>
+      <c r="R193" s="15"/>
+      <c r="S193" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="194" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A194" s="7">
+        <v>192</v>
+      </c>
+      <c r="B194" s="7"/>
+      <c r="C194" s="8"/>
+      <c r="D194" s="9" t="s">
+        <v>745</v>
+      </c>
+      <c r="E194" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F194" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="G194" s="7"/>
+      <c r="H194" s="10">
+        <v>44340</v>
+      </c>
+      <c r="I194" s="11"/>
+      <c r="J194" s="12"/>
+      <c r="K194" s="7"/>
+      <c r="L194" s="11"/>
+      <c r="M194" s="11"/>
+      <c r="N194" s="13"/>
+      <c r="O194" s="7"/>
+      <c r="P194" s="13"/>
+      <c r="Q194" s="14"/>
+      <c r="R194" s="15"/>
+      <c r="S194" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="195" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A195" s="7">
+        <v>193</v>
+      </c>
+      <c r="B195" s="7"/>
+      <c r="C195" s="8"/>
+      <c r="D195" s="9" t="s">
+        <v>746</v>
+      </c>
+      <c r="E195" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F195" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G195" s="7"/>
+      <c r="H195" s="10">
+        <v>44170</v>
+      </c>
+      <c r="I195" s="11">
+        <v>44444</v>
+      </c>
+      <c r="J195" s="12">
+        <v>44534</v>
+      </c>
+      <c r="K195" s="7" t="s">
+        <v>747</v>
+      </c>
+      <c r="L195" s="11"/>
+      <c r="M195" s="11"/>
+      <c r="N195" s="13"/>
+      <c r="O195" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P195" s="13"/>
+      <c r="Q195" s="14"/>
+      <c r="R195" s="15"/>
+      <c r="S195" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="196" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A196" s="7">
+        <v>194</v>
+      </c>
+      <c r="B196" s="7"/>
+      <c r="C196" s="8"/>
+      <c r="D196" s="9" t="s">
+        <v>748</v>
+      </c>
+      <c r="E196" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F196" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G196" s="7"/>
+      <c r="H196" s="10">
+        <v>44348</v>
+      </c>
+      <c r="I196" s="11"/>
+      <c r="J196" s="12"/>
+      <c r="K196" s="7"/>
+      <c r="L196" s="11"/>
+      <c r="M196" s="11"/>
+      <c r="N196" s="13"/>
+      <c r="O196" s="7"/>
+      <c r="P196" s="13"/>
+      <c r="Q196" s="14"/>
+      <c r="R196" s="15"/>
+      <c r="S196" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="197" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A197" s="7">
+        <v>195</v>
+      </c>
+      <c r="B197" s="7"/>
+      <c r="C197" s="8"/>
+      <c r="D197" s="9" t="s">
+        <v>749</v>
+      </c>
+      <c r="E197" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F197" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="G197" s="7"/>
+      <c r="H197" s="10">
+        <v>44272</v>
+      </c>
+      <c r="I197" s="11">
+        <v>44547</v>
+      </c>
+      <c r="J197" s="12">
+        <v>44636</v>
+      </c>
+      <c r="K197" s="7"/>
+      <c r="L197" s="11"/>
+      <c r="M197" s="11"/>
+      <c r="N197" s="13"/>
+      <c r="O197" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P197" s="13"/>
+      <c r="Q197" s="14"/>
+      <c r="R197" s="15"/>
+      <c r="S197" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="198" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A198" s="7">
+        <v>196</v>
+      </c>
+      <c r="B198" s="7"/>
+      <c r="C198" s="8"/>
+      <c r="D198" s="9" t="s">
+        <v>751</v>
+      </c>
+      <c r="E198" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F198" s="7" t="s">
+        <v>752</v>
+      </c>
+      <c r="G198" s="7"/>
+      <c r="H198" s="10">
+        <v>44389</v>
+      </c>
+      <c r="I198" s="11">
+        <v>44756</v>
+      </c>
+      <c r="J198" s="12">
+        <v>44845</v>
+      </c>
+      <c r="K198" s="7" t="s">
+        <v>753</v>
+      </c>
+      <c r="L198" s="11"/>
+      <c r="M198" s="11"/>
+      <c r="N198" s="13"/>
+      <c r="O198" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P198" s="13"/>
+      <c r="Q198" s="14"/>
+      <c r="R198" s="15"/>
+      <c r="S198" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="199" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A199" s="7">
+        <v>197</v>
+      </c>
+      <c r="B199" s="7"/>
+      <c r="C199" s="8"/>
+      <c r="D199" s="9" t="s">
+        <v>754</v>
+      </c>
+      <c r="E199" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F199" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G199" s="7"/>
+      <c r="H199" s="10">
+        <v>43234</v>
+      </c>
+      <c r="I199" s="11">
+        <v>44241</v>
+      </c>
+      <c r="J199" s="12">
+        <v>44329</v>
+      </c>
+      <c r="K199" s="7" t="s">
+        <v>755</v>
+      </c>
+      <c r="L199" s="11"/>
+      <c r="M199" s="11"/>
+      <c r="N199" s="13"/>
+      <c r="O199" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P199" s="13"/>
+      <c r="Q199" s="14"/>
+      <c r="R199" s="15"/>
+      <c r="S199" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="200" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A200" s="7">
+        <v>198</v>
+      </c>
+      <c r="B200" s="7"/>
+      <c r="C200" s="8"/>
+      <c r="D200" s="9" t="s">
+        <v>756</v>
+      </c>
+      <c r="E200" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F200" s="7" t="s">
+        <v>757</v>
+      </c>
+      <c r="G200" s="7"/>
+      <c r="H200" s="10">
+        <v>44621</v>
+      </c>
+      <c r="I200" s="11">
+        <v>44986</v>
+      </c>
+      <c r="J200" s="12">
+        <v>45139</v>
+      </c>
+      <c r="K200" s="7" t="s">
+        <v>758</v>
+      </c>
+      <c r="L200" s="11"/>
+      <c r="M200" s="11"/>
+      <c r="N200" s="13"/>
+      <c r="O200" s="7" t="s">
+        <v>759</v>
+      </c>
+      <c r="P200" s="13"/>
+      <c r="Q200" s="14"/>
+      <c r="R200" s="15"/>
+      <c r="S200" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="201" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A201" s="7">
+        <v>199</v>
+      </c>
+      <c r="B201" s="7"/>
+      <c r="C201" s="8"/>
+      <c r="D201" s="9" t="s">
+        <v>760</v>
+      </c>
+      <c r="E201" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F201" s="7" t="s">
+        <v>761</v>
+      </c>
+      <c r="G201" s="7"/>
+      <c r="H201" s="10">
+        <v>44044</v>
+      </c>
+      <c r="I201" s="11">
+        <v>44777</v>
+      </c>
+      <c r="J201" s="12">
+        <v>44896</v>
+      </c>
+      <c r="K201" s="7" t="s">
+        <v>762</v>
+      </c>
+      <c r="L201" s="11"/>
+      <c r="M201" s="11"/>
+      <c r="N201" s="13"/>
+      <c r="O201" s="7" t="s">
+        <v>763</v>
+      </c>
+      <c r="P201" s="13"/>
+      <c r="Q201" s="14"/>
+      <c r="R201" s="15"/>
+      <c r="S201" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="202" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A202" s="7">
+        <v>200</v>
+      </c>
+      <c r="B202" s="7"/>
+      <c r="C202" s="8"/>
+      <c r="D202" s="9" t="s">
+        <v>764</v>
+      </c>
+      <c r="E202" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F202" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G202" s="7"/>
+      <c r="H202" s="10">
+        <v>44241</v>
+      </c>
+      <c r="I202" s="11">
+        <v>44241</v>
+      </c>
+      <c r="J202" s="12">
+        <v>44329</v>
+      </c>
+      <c r="K202" s="7" t="s">
+        <v>755</v>
+      </c>
+      <c r="L202" s="11"/>
+      <c r="M202" s="11"/>
+      <c r="N202" s="13"/>
+      <c r="O202" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P202" s="13"/>
+      <c r="Q202" s="14"/>
+      <c r="R202" s="15"/>
+      <c r="S202" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="203" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A203" s="7">
+        <v>201</v>
+      </c>
+      <c r="B203" s="7"/>
+      <c r="C203" s="8"/>
+      <c r="D203" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="E203" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F203" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="G203" s="7"/>
+      <c r="H203" s="10">
+        <v>44380</v>
+      </c>
+      <c r="I203" s="11">
+        <v>44837</v>
+      </c>
+      <c r="J203" s="12">
+        <v>44882</v>
+      </c>
+      <c r="K203" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="L203" s="11"/>
+      <c r="M203" s="11"/>
+      <c r="N203" s="13"/>
+      <c r="O203" s="7" t="s">
+        <v>767</v>
+      </c>
+      <c r="P203" s="13"/>
+      <c r="Q203" s="14"/>
+      <c r="R203" s="15"/>
+      <c r="S203" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="204" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A204" s="7">
+        <v>202</v>
+      </c>
+      <c r="B204" s="7"/>
+      <c r="C204" s="8"/>
+      <c r="D204" s="9" t="s">
+        <v>768</v>
+      </c>
+      <c r="E204" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F204" s="7" t="s">
+        <v>769</v>
+      </c>
+      <c r="G204" s="7"/>
+      <c r="H204" s="10">
+        <v>44958</v>
+      </c>
+      <c r="I204" s="11">
+        <v>44958</v>
+      </c>
+      <c r="J204" s="12">
+        <v>44959</v>
+      </c>
+      <c r="K204" s="7" t="s">
+        <v>770</v>
+      </c>
+      <c r="L204" s="11"/>
+      <c r="M204" s="11"/>
+      <c r="N204" s="13"/>
+      <c r="O204" s="7"/>
+      <c r="P204" s="13"/>
+      <c r="Q204" s="14"/>
+      <c r="R204" s="15"/>
+      <c r="S204" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="205" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A205" s="7">
+        <v>203</v>
+      </c>
+      <c r="B205" s="7"/>
+      <c r="C205" s="8"/>
+      <c r="D205" s="9" t="s">
+        <v>771</v>
+      </c>
+      <c r="E205" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F205" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="G205" s="7"/>
+      <c r="H205" s="10">
+        <v>44688</v>
+      </c>
+      <c r="I205" s="11">
+        <v>45053</v>
+      </c>
+      <c r="J205" s="12">
+        <v>45144</v>
+      </c>
+      <c r="K205" s="7" t="s">
+        <v>626</v>
+      </c>
+      <c r="L205" s="11"/>
+      <c r="M205" s="11"/>
+      <c r="N205" s="13"/>
+      <c r="O205" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P205" s="13"/>
+      <c r="Q205" s="14"/>
+      <c r="R205" s="15"/>
+      <c r="S205" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="206" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A206" s="7">
+        <v>204</v>
+      </c>
+      <c r="B206" s="7"/>
+      <c r="C206" s="8"/>
+      <c r="D206" s="9" t="s">
+        <v>772</v>
+      </c>
+      <c r="E206" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F206" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G206" s="7"/>
+      <c r="H206" s="10">
+        <v>43694</v>
+      </c>
+      <c r="I206" s="11">
+        <v>45007</v>
+      </c>
+      <c r="J206" s="12">
+        <v>45098</v>
+      </c>
+      <c r="K206" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="L206" s="11"/>
+      <c r="M206" s="11"/>
+      <c r="N206" s="13"/>
+      <c r="O206" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P206" s="13"/>
+      <c r="Q206" s="14"/>
+      <c r="R206" s="15"/>
+      <c r="S206" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="207" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A207" s="7">
+        <v>205</v>
+      </c>
+      <c r="B207" s="7"/>
+      <c r="C207" s="8"/>
+      <c r="D207" s="9" t="s">
+        <v>773</v>
+      </c>
+      <c r="E207" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F207" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="G207" s="7"/>
+      <c r="H207" s="10">
+        <v>44661</v>
+      </c>
+      <c r="I207" s="11">
+        <v>44846</v>
+      </c>
+      <c r="J207" s="12">
+        <v>44935</v>
+      </c>
+      <c r="K207" s="7" t="s">
+        <v>775</v>
+      </c>
+      <c r="L207" s="11"/>
+      <c r="M207" s="11"/>
+      <c r="N207" s="13"/>
+      <c r="O207" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P207" s="13"/>
+      <c r="Q207" s="14"/>
+      <c r="R207" s="15"/>
+      <c r="S207" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="208" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A208" s="7">
+        <v>206</v>
+      </c>
+      <c r="B208" s="7"/>
+      <c r="C208" s="8"/>
+      <c r="D208" s="9" t="s">
+        <v>776</v>
+      </c>
+      <c r="E208" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F208" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G208" s="7"/>
+      <c r="H208" s="10">
+        <v>44202</v>
+      </c>
+      <c r="I208" s="11">
+        <v>45022</v>
+      </c>
+      <c r="J208" s="12">
+        <v>45112</v>
+      </c>
+      <c r="K208" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="L208" s="11"/>
+      <c r="M208" s="11"/>
+      <c r="N208" s="13"/>
+      <c r="O208" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P208" s="13"/>
+      <c r="Q208" s="14"/>
+      <c r="R208" s="15"/>
+      <c r="S208" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="209" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A209" s="7">
+        <v>207</v>
+      </c>
+      <c r="B209" s="7"/>
+      <c r="C209" s="8"/>
+      <c r="D209" s="9" t="s">
+        <v>777</v>
+      </c>
+      <c r="E209" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F209" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="G209" s="7"/>
+      <c r="H209" s="10">
+        <v>43884</v>
+      </c>
+      <c r="I209" s="11"/>
+      <c r="J209" s="12"/>
+      <c r="K209" s="7"/>
+      <c r="L209" s="11"/>
+      <c r="M209" s="11"/>
+      <c r="N209" s="13"/>
+      <c r="O209" s="7"/>
+      <c r="P209" s="13"/>
+      <c r="Q209" s="14"/>
+      <c r="R209" s="15"/>
+      <c r="S209" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="210" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A210" s="7">
+        <v>208</v>
+      </c>
+      <c r="B210" s="7"/>
+      <c r="C210" s="8"/>
+      <c r="D210" s="9" t="s">
+        <v>778</v>
+      </c>
+      <c r="E210" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F210" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="G210" s="7"/>
+      <c r="H210" s="10">
+        <v>44791</v>
+      </c>
+      <c r="I210" s="11">
+        <v>44885</v>
+      </c>
+      <c r="J210" s="12">
+        <v>44974</v>
+      </c>
+      <c r="K210" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="L210" s="11"/>
+      <c r="M210" s="11"/>
+      <c r="N210" s="13"/>
+      <c r="O210" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P210" s="13"/>
+      <c r="Q210" s="14"/>
+      <c r="R210" s="15"/>
+      <c r="S210" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="211" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A211" s="7">
+        <v>209</v>
+      </c>
+      <c r="B211" s="7"/>
+      <c r="C211" s="8"/>
+      <c r="D211" s="9" t="s">
+        <v>779</v>
+      </c>
+      <c r="E211" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F211" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="G211" s="7"/>
+      <c r="H211" s="10">
+        <v>44836</v>
+      </c>
+      <c r="I211" s="11">
+        <v>45108</v>
+      </c>
+      <c r="J211" s="12">
+        <v>45158</v>
+      </c>
+      <c r="K211" s="7" t="s">
+        <v>780</v>
+      </c>
+      <c r="L211" s="11"/>
+      <c r="M211" s="11"/>
+      <c r="N211" s="13"/>
+      <c r="O211" s="7" t="s">
+        <v>767</v>
+      </c>
+      <c r="P211" s="13"/>
+      <c r="Q211" s="14"/>
+      <c r="R211" s="15"/>
+      <c r="S211" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="212" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A212" s="7">
+        <v>210</v>
+      </c>
+      <c r="B212" s="7"/>
+      <c r="C212" s="8"/>
+      <c r="D212" s="9" t="s">
+        <v>781</v>
+      </c>
+      <c r="E212" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F212" s="7" t="s">
+        <v>782</v>
+      </c>
+      <c r="G212" s="7"/>
+      <c r="H212" s="10">
+        <v>44896</v>
+      </c>
+      <c r="I212" s="11">
+        <v>44896</v>
+      </c>
+      <c r="J212" s="12">
+        <v>44985</v>
+      </c>
+      <c r="K212" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="L212" s="11"/>
+      <c r="M212" s="11"/>
+      <c r="N212" s="13"/>
+      <c r="O212" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P212" s="13"/>
+      <c r="Q212" s="14"/>
+      <c r="R212" s="15"/>
+      <c r="S212" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="213" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A213" s="7">
+        <v>211</v>
+      </c>
+      <c r="B213" s="7"/>
+      <c r="C213" s="8"/>
+      <c r="D213" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="E213" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F213" s="7" t="s">
+        <v>783</v>
+      </c>
+      <c r="G213" s="7"/>
+      <c r="H213" s="10">
+        <v>44827</v>
+      </c>
+      <c r="I213" s="11">
+        <v>45169</v>
+      </c>
+      <c r="J213" s="12">
+        <v>45169</v>
+      </c>
+      <c r="K213" s="7" t="s">
+        <v>784</v>
+      </c>
+      <c r="L213" s="11"/>
+      <c r="M213" s="11"/>
+      <c r="N213" s="13"/>
+      <c r="O213" s="7"/>
+      <c r="P213" s="13"/>
+      <c r="Q213" s="14"/>
+      <c r="R213" s="15"/>
+      <c r="S213" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="214" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A214" s="7">
+        <v>212</v>
+      </c>
+      <c r="B214" s="7"/>
+      <c r="C214" s="8"/>
+      <c r="D214" s="9" t="s">
+        <v>785</v>
+      </c>
+      <c r="E214" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F214" s="7" t="s">
+        <v>786</v>
+      </c>
+      <c r="G214" s="7"/>
+      <c r="H214" s="10">
+        <v>44927</v>
+      </c>
+      <c r="I214" s="11">
+        <v>45108</v>
+      </c>
+      <c r="J214" s="12">
+        <v>45199</v>
+      </c>
+      <c r="K214" s="7" t="s">
+        <v>787</v>
+      </c>
+      <c r="L214" s="11"/>
+      <c r="M214" s="11"/>
+      <c r="N214" s="13"/>
+      <c r="O214" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P214" s="13"/>
+      <c r="Q214" s="14"/>
+      <c r="R214" s="15"/>
+      <c r="S214" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="215" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A215" s="7">
+        <v>213</v>
+      </c>
+      <c r="B215" s="7"/>
+      <c r="C215" s="8"/>
+      <c r="D215" s="9" t="s">
+        <v>788</v>
+      </c>
+      <c r="E215" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F215" s="7" t="s">
+        <v>789</v>
+      </c>
+      <c r="G215" s="7"/>
+      <c r="H215" s="10">
+        <v>45029</v>
+      </c>
+      <c r="I215" s="11">
+        <v>44968</v>
+      </c>
+      <c r="J215" s="12">
+        <v>44968</v>
+      </c>
+      <c r="K215" s="7" t="s">
+        <v>790</v>
+      </c>
+      <c r="L215" s="11"/>
+      <c r="M215" s="11"/>
+      <c r="N215" s="13"/>
+      <c r="O215" s="7"/>
+      <c r="P215" s="13"/>
+      <c r="Q215" s="14"/>
+      <c r="R215" s="15"/>
+      <c r="S215" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="216" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A216" s="7">
+        <v>214</v>
+      </c>
+      <c r="B216" s="7"/>
+      <c r="C216" s="8"/>
+      <c r="D216" s="9" t="s">
+        <v>791</v>
+      </c>
+      <c r="E216" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F216" s="7" t="s">
+        <v>792</v>
+      </c>
+      <c r="G216" s="7"/>
+      <c r="H216" s="10">
+        <v>41640</v>
+      </c>
+      <c r="I216" s="11">
+        <v>44927</v>
+      </c>
+      <c r="J216" s="12">
+        <v>45138</v>
+      </c>
+      <c r="K216" s="7" t="s">
+        <v>793</v>
+      </c>
+      <c r="L216" s="11"/>
+      <c r="M216" s="11"/>
+      <c r="N216" s="13"/>
+      <c r="O216" s="7" t="s">
+        <v>794</v>
+      </c>
+      <c r="P216" s="13"/>
+      <c r="Q216" s="14"/>
+      <c r="R216" s="15"/>
+      <c r="S216" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="217" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A217" s="7">
+        <v>215</v>
+      </c>
+      <c r="B217" s="7"/>
+      <c r="C217" s="8"/>
+      <c r="D217" s="9" t="s">
+        <v>795</v>
+      </c>
+      <c r="E217" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F217" s="7" t="s">
+        <v>796</v>
+      </c>
+      <c r="G217" s="7"/>
+      <c r="H217" s="10">
+        <v>44206</v>
+      </c>
+      <c r="I217" s="11">
+        <v>45170</v>
+      </c>
+      <c r="J217" s="12">
+        <v>45170</v>
+      </c>
+      <c r="K217" s="7" t="s">
+        <v>797</v>
+      </c>
+      <c r="L217" s="11"/>
+      <c r="M217" s="11"/>
+      <c r="N217" s="13"/>
+      <c r="O217" s="7"/>
+      <c r="P217" s="13"/>
+      <c r="Q217" s="14"/>
+      <c r="R217" s="15"/>
+      <c r="S217" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="218" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A218" s="7">
+        <v>216</v>
+      </c>
+      <c r="B218" s="7"/>
+      <c r="C218" s="8"/>
+      <c r="D218" s="9" t="s">
+        <v>798</v>
+      </c>
+      <c r="E218" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F218" s="7" t="s">
+        <v>799</v>
+      </c>
+      <c r="G218" s="7"/>
+      <c r="H218" s="10">
+        <v>44571</v>
+      </c>
+      <c r="I218" s="11">
+        <v>44844</v>
+      </c>
+      <c r="J218" s="12">
+        <v>44955</v>
+      </c>
+      <c r="K218" s="7" t="s">
+        <v>800</v>
+      </c>
+      <c r="L218" s="11"/>
+      <c r="M218" s="11"/>
+      <c r="N218" s="13"/>
+      <c r="O218" s="7" t="s">
+        <v>763</v>
+      </c>
+      <c r="P218" s="13"/>
+      <c r="Q218" s="14"/>
+      <c r="R218" s="15"/>
+      <c r="S218" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="219" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A219" s="7">
+        <v>217</v>
+      </c>
+      <c r="B219" s="7"/>
+      <c r="C219" s="8"/>
+      <c r="D219" s="9" t="s">
+        <v>801</v>
+      </c>
+      <c r="E219" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F219" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G219" s="7"/>
+      <c r="H219" s="10">
+        <v>44632</v>
+      </c>
+      <c r="I219" s="11">
+        <v>44997</v>
+      </c>
+      <c r="J219" s="12">
+        <v>45088</v>
+      </c>
+      <c r="K219" s="7" t="s">
+        <v>802</v>
+      </c>
+      <c r="L219" s="11"/>
+      <c r="M219" s="11"/>
+      <c r="N219" s="13"/>
+      <c r="O219" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P219" s="13"/>
+      <c r="Q219" s="14"/>
+      <c r="R219" s="15"/>
+      <c r="S219" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="220" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A220" s="7">
+        <v>218</v>
+      </c>
+      <c r="B220" s="7"/>
+      <c r="C220" s="8"/>
+      <c r="D220" s="9" t="s">
+        <v>803</v>
+      </c>
+      <c r="E220" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F220" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="G220" s="7"/>
+      <c r="H220" s="10">
+        <v>44629</v>
+      </c>
+      <c r="I220" s="11">
+        <v>45086</v>
+      </c>
+      <c r="J220" s="12">
+        <v>45177</v>
+      </c>
+      <c r="K220" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="L220" s="11"/>
+      <c r="M220" s="11"/>
+      <c r="N220" s="13"/>
+      <c r="O220" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P220" s="13"/>
+      <c r="Q220" s="14"/>
+      <c r="R220" s="15"/>
+      <c r="S220" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="221" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A221" s="7">
+        <v>219</v>
+      </c>
+      <c r="B221" s="7"/>
+      <c r="C221" s="8"/>
+      <c r="D221" s="9" t="s">
+        <v>804</v>
+      </c>
+      <c r="E221" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F221" s="7" t="s">
+        <v>805</v>
+      </c>
+      <c r="G221" s="7"/>
+      <c r="H221" s="10">
+        <v>42102</v>
+      </c>
+      <c r="I221" s="11">
+        <v>45115</v>
+      </c>
+      <c r="J221" s="12">
+        <v>45206</v>
+      </c>
+      <c r="K221" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="L221" s="11"/>
+      <c r="M221" s="11"/>
+      <c r="N221" s="13"/>
+      <c r="O221" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P221" s="13"/>
+      <c r="Q221" s="14"/>
+      <c r="R221" s="15"/>
+      <c r="S221" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="222" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A222" s="7">
+        <v>220</v>
+      </c>
+      <c r="B222" s="7"/>
+      <c r="C222" s="8"/>
+      <c r="D222" s="9" t="s">
+        <v>806</v>
+      </c>
+      <c r="E222" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F222" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G222" s="7"/>
+      <c r="H222" s="10">
+        <v>43234</v>
+      </c>
+      <c r="I222" s="11">
+        <v>45152</v>
+      </c>
+      <c r="J222" s="12">
+        <v>45243</v>
+      </c>
+      <c r="K222" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="L222" s="11"/>
+      <c r="M222" s="11"/>
+      <c r="N222" s="13"/>
+      <c r="O222" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P222" s="13"/>
+      <c r="Q222" s="14"/>
+      <c r="R222" s="15"/>
+      <c r="S222" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="223" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A223" s="7">
+        <v>221</v>
+      </c>
+      <c r="B223" s="7"/>
+      <c r="C223" s="8"/>
+      <c r="D223" s="9" t="s">
+        <v>807</v>
+      </c>
+      <c r="E223" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F223" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G223" s="7"/>
+      <c r="H223" s="10">
+        <v>44625</v>
+      </c>
+      <c r="I223" s="11">
+        <v>45174</v>
+      </c>
+      <c r="J223" s="12">
+        <v>45264</v>
+      </c>
+      <c r="K223" s="7"/>
+      <c r="L223" s="11"/>
+      <c r="M223" s="11"/>
+      <c r="N223" s="13"/>
+      <c r="O223" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P223" s="13"/>
+      <c r="Q223" s="14"/>
+      <c r="R223" s="15"/>
+      <c r="S223" s="7" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="224" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A224" s="7">
+        <v>222</v>
+      </c>
+      <c r="B224" s="7"/>
+      <c r="C224" s="8"/>
+      <c r="D224" s="9" t="s">
+        <v>809</v>
+      </c>
+      <c r="E224" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F224" s="7" t="s">
+        <v>810</v>
+      </c>
+      <c r="G224" s="7"/>
+      <c r="H224" s="10">
+        <v>40124</v>
+      </c>
+      <c r="I224" s="11">
+        <v>44927</v>
+      </c>
+      <c r="J224" s="12">
+        <v>45291</v>
+      </c>
+      <c r="K224" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="L224" s="11"/>
+      <c r="M224" s="11"/>
+      <c r="N224" s="13"/>
+      <c r="O224" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P224" s="13"/>
+      <c r="Q224" s="14"/>
+      <c r="R224" s="15"/>
+      <c r="S224" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="225" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A225" s="7">
+        <v>223</v>
+      </c>
+      <c r="B225" s="7"/>
+      <c r="C225" s="8"/>
+      <c r="D225" s="9" t="s">
+        <v>811</v>
+      </c>
+      <c r="E225" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F225" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="G225" s="7"/>
+      <c r="H225" s="10">
+        <v>44238</v>
+      </c>
+      <c r="I225" s="11">
+        <v>45241</v>
+      </c>
+      <c r="J225" s="12">
+        <v>45332</v>
+      </c>
+      <c r="K225" s="7"/>
+      <c r="L225" s="11"/>
+      <c r="M225" s="11"/>
+      <c r="N225" s="13"/>
+      <c r="O225" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P225" s="13"/>
+      <c r="Q225" s="14"/>
+      <c r="R225" s="15"/>
+      <c r="S225" s="7" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="226" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A226" s="7">
+        <v>224</v>
+      </c>
+      <c r="B226" s="7"/>
+      <c r="C226" s="8"/>
+      <c r="D226" s="9" t="s">
+        <v>813</v>
+      </c>
+      <c r="E226" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F226" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="G226" s="7"/>
+      <c r="H226" s="10">
+        <v>44832</v>
+      </c>
+      <c r="I226" s="11">
+        <v>45288</v>
+      </c>
+      <c r="J226" s="12">
+        <v>45378</v>
+      </c>
+      <c r="K226" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="L226" s="11"/>
+      <c r="M226" s="11"/>
+      <c r="N226" s="13"/>
+      <c r="O226" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P226" s="13"/>
+      <c r="Q226" s="14"/>
+      <c r="R226" s="15"/>
+      <c r="S226" s="7" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="227" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A227" s="7">
+        <v>225</v>
+      </c>
+      <c r="B227" s="7">
+        <v>44</v>
+      </c>
+      <c r="C227" s="8"/>
+      <c r="D227" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="E227" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F227" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G227" s="7"/>
+      <c r="H227" s="10">
+        <v>44311</v>
+      </c>
+      <c r="I227" s="11">
+        <v>45316</v>
+      </c>
+      <c r="J227" s="12">
+        <v>45406</v>
+      </c>
+      <c r="K227" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="L227" s="11">
+        <v>22362</v>
+      </c>
+      <c r="M227" s="11">
+        <v>44277</v>
+      </c>
+      <c r="N227" s="13"/>
+      <c r="O227" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P227" s="13">
+        <v>26103221701013</v>
+      </c>
+      <c r="Q227" s="14">
+        <v>1228894728</v>
+      </c>
+      <c r="R227" s="15"/>
+      <c r="S227" s="7" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="228" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A228" s="7">
+        <v>226</v>
+      </c>
+      <c r="B228" s="7">
+        <v>209</v>
+      </c>
+      <c r="C228" s="8"/>
+      <c r="D228" s="9" t="s">
+        <v>817</v>
+      </c>
+      <c r="E228" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F228" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="G228" s="7"/>
+      <c r="H228" s="10"/>
+      <c r="I228" s="11"/>
+      <c r="J228" s="12"/>
+      <c r="K228" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="L228" s="11">
+        <v>23460</v>
+      </c>
+      <c r="M228" s="11">
+        <v>45375</v>
+      </c>
+      <c r="N228" s="13"/>
+      <c r="O228" s="7"/>
+      <c r="P228" s="13">
+        <v>26403241301899</v>
+      </c>
+      <c r="Q228" s="14"/>
+      <c r="R228" s="15"/>
+      <c r="S228" s="7" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="229" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A229" s="7">
+        <v>227</v>
+      </c>
+      <c r="B229" s="7">
+        <v>179</v>
+      </c>
+      <c r="C229" s="8"/>
+      <c r="D229" s="9" t="s">
+        <v>819</v>
+      </c>
+      <c r="E229" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F229" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G229" s="7"/>
+      <c r="H229" s="10">
+        <v>44954</v>
+      </c>
+      <c r="I229" s="11">
+        <v>45319</v>
+      </c>
+      <c r="J229" s="12">
+        <v>45409</v>
+      </c>
+      <c r="K229" s="7" t="s">
+        <v>820</v>
+      </c>
+      <c r="L229" s="11">
+        <v>23017</v>
+      </c>
+      <c r="M229" s="11">
+        <v>44932</v>
+      </c>
+      <c r="N229" s="13"/>
+      <c r="O229" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P229" s="13">
+        <v>26301061701735</v>
+      </c>
+      <c r="Q229" s="14">
+        <v>1225942643</v>
+      </c>
+      <c r="R229" s="15"/>
+      <c r="S229" s="7" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="230" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A230" s="7">
+        <v>228</v>
+      </c>
+      <c r="B230" s="7">
+        <v>183</v>
+      </c>
+      <c r="C230" s="8"/>
+      <c r="D230" s="9" t="s">
+        <v>822</v>
+      </c>
+      <c r="E230" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F230" s="7" t="s">
+        <v>823</v>
+      </c>
+      <c r="G230" s="7"/>
+      <c r="H230" s="10">
+        <v>45073</v>
+      </c>
+      <c r="I230" s="11">
+        <v>45073</v>
+      </c>
+      <c r="J230" s="12">
+        <v>45438</v>
+      </c>
+      <c r="K230" s="7"/>
+      <c r="L230" s="11"/>
+      <c r="M230" s="11"/>
+      <c r="N230" s="13"/>
+      <c r="O230" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P230" s="13"/>
+      <c r="Q230" s="14"/>
+      <c r="R230" s="15"/>
+      <c r="S230" s="7" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="231" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A231" s="7">
+        <v>229</v>
+      </c>
+      <c r="B231" s="7">
+        <v>131</v>
+      </c>
+      <c r="C231" s="8"/>
+      <c r="D231" s="9" t="s">
+        <v>825</v>
+      </c>
+      <c r="E231" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F231" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G231" s="7"/>
+      <c r="H231" s="10">
+        <v>44567</v>
+      </c>
+      <c r="I231" s="11">
+        <v>45297</v>
+      </c>
+      <c r="J231" s="12">
+        <v>45478</v>
+      </c>
+      <c r="K231" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="L231" s="11"/>
+      <c r="M231" s="11"/>
+      <c r="N231" s="13"/>
+      <c r="O231" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="P231" s="13"/>
+      <c r="Q231" s="14"/>
+      <c r="R231" s="15"/>
+      <c r="S231" s="7" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="232" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A232" s="7">
+        <v>230</v>
+      </c>
+      <c r="B232" s="7">
+        <v>124</v>
+      </c>
+      <c r="C232" s="8"/>
+      <c r="D232" s="9" t="s">
+        <v>827</v>
+      </c>
+      <c r="E232" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F232" s="7" t="s">
+        <v>828</v>
+      </c>
+      <c r="G232" s="7"/>
+      <c r="H232" s="10">
+        <v>40776</v>
+      </c>
+      <c r="I232" s="11">
+        <v>45105</v>
+      </c>
+      <c r="J232" s="12">
+        <v>45470</v>
+      </c>
+      <c r="K232" s="7" t="s">
+        <v>829</v>
+      </c>
+      <c r="L232" s="11"/>
+      <c r="M232" s="11"/>
+      <c r="N232" s="13"/>
+      <c r="O232" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P232" s="13"/>
+      <c r="Q232" s="14"/>
+      <c r="R232" s="15"/>
+      <c r="S232" s="7" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="233" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A233" s="7">
+        <v>231</v>
+      </c>
+      <c r="B233" s="7">
+        <v>63</v>
+      </c>
+      <c r="C233" s="8"/>
+      <c r="D233" s="9" t="s">
+        <v>831</v>
+      </c>
+      <c r="E233" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F233" s="7" t="s">
+        <v>832</v>
+      </c>
+      <c r="G233" s="7"/>
+      <c r="H233" s="10">
+        <v>44409</v>
+      </c>
+      <c r="I233" s="11">
+        <v>45505</v>
+      </c>
+      <c r="J233" s="12">
+        <v>45596</v>
+      </c>
+      <c r="K233" s="7" t="s">
+        <v>833</v>
+      </c>
+      <c r="L233" s="11">
+        <v>20885</v>
+      </c>
+      <c r="M233" s="11">
+        <v>42800</v>
+      </c>
+      <c r="N233" s="13"/>
+      <c r="O233" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P233" s="13">
+        <v>25703062201377</v>
+      </c>
+      <c r="Q233" s="14">
+        <v>1201992554</v>
+      </c>
+      <c r="R233" s="15"/>
+      <c r="S233" s="7" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="234" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A234" s="7">
+        <v>232</v>
+      </c>
+      <c r="B234" s="7">
+        <v>20119</v>
+      </c>
+      <c r="C234" s="8"/>
+      <c r="D234" s="9" t="s">
+        <v>835</v>
+      </c>
+      <c r="E234" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F234" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G234" s="7"/>
+      <c r="H234" s="10">
+        <v>43740</v>
+      </c>
+      <c r="I234" s="11">
+        <v>45475</v>
+      </c>
+      <c r="J234" s="12">
+        <v>45566</v>
+      </c>
+      <c r="K234" s="7" t="s">
+        <v>836</v>
+      </c>
+      <c r="L234" s="11">
+        <v>21095</v>
+      </c>
+      <c r="M234" s="11">
+        <v>43010</v>
+      </c>
+      <c r="N234" s="13"/>
+      <c r="O234" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P234" s="13">
+        <v>25710020102391</v>
+      </c>
+      <c r="Q234" s="14">
+        <v>1282057201</v>
+      </c>
+      <c r="R234" s="15"/>
+      <c r="S234" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="235" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A235" s="7">
+        <v>233</v>
+      </c>
+      <c r="B235" s="7">
+        <v>20270</v>
+      </c>
+      <c r="C235" s="8"/>
+      <c r="D235" s="9" t="s">
+        <v>837</v>
+      </c>
+      <c r="E235" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F235" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G235" s="7"/>
+      <c r="H235" s="10">
+        <v>45383</v>
+      </c>
+      <c r="I235" s="11">
+        <v>45383</v>
+      </c>
+      <c r="J235" s="12">
+        <v>45473</v>
+      </c>
+      <c r="K235" s="7" t="s">
+        <v>838</v>
+      </c>
+      <c r="L235" s="11">
+        <v>23380</v>
+      </c>
+      <c r="M235" s="11">
+        <v>45295</v>
+      </c>
+      <c r="N235" s="13"/>
+      <c r="O235" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P235" s="13">
+        <v>26401041400717</v>
+      </c>
+      <c r="Q235" s="14">
+        <v>1141614868</v>
+      </c>
+      <c r="R235" s="15"/>
+      <c r="S235" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="236" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A236" s="7">
+        <v>234</v>
+      </c>
+      <c r="B236" s="7">
+        <v>73</v>
+      </c>
+      <c r="C236" s="8"/>
+      <c r="D236" s="9" t="s">
+        <v>839</v>
+      </c>
+      <c r="E236" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F236" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G236" s="7"/>
+      <c r="H236" s="10">
+        <v>42054</v>
+      </c>
+      <c r="I236" s="11">
+        <v>45431</v>
+      </c>
+      <c r="J236" s="12">
+        <v>45522</v>
+      </c>
+      <c r="K236" s="7" t="s">
+        <v>840</v>
+      </c>
+      <c r="L236" s="11">
+        <v>20136</v>
+      </c>
+      <c r="M236" s="11">
+        <v>42051</v>
+      </c>
+      <c r="N236" s="13"/>
+      <c r="O236" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P236" s="13">
+        <v>25502160102454</v>
+      </c>
+      <c r="Q236" s="14"/>
+      <c r="R236" s="15"/>
+      <c r="S236" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="237" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A237" s="7">
+        <v>235</v>
+      </c>
+      <c r="B237" s="7">
+        <v>159</v>
+      </c>
+      <c r="C237" s="8"/>
+      <c r="D237" s="9" t="s">
+        <v>841</v>
+      </c>
+      <c r="E237" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F237" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G237" s="7"/>
+      <c r="H237" s="10">
+        <v>44847</v>
+      </c>
+      <c r="I237" s="11">
+        <v>44847</v>
+      </c>
+      <c r="J237" s="12">
+        <v>45395</v>
+      </c>
+      <c r="K237" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="L237" s="11">
+        <v>22915</v>
+      </c>
+      <c r="M237" s="11">
+        <v>44830</v>
+      </c>
+      <c r="N237" s="13"/>
+      <c r="O237" s="7" t="s">
+        <v>842</v>
+      </c>
+      <c r="P237" s="13">
+        <v>26209260101905</v>
+      </c>
+      <c r="Q237" s="14">
+        <v>1270942558</v>
+      </c>
+      <c r="R237" s="15"/>
+      <c r="S237" s="7" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="238" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A238" s="7">
+        <v>236</v>
+      </c>
+      <c r="B238" s="7">
+        <v>130</v>
+      </c>
+      <c r="C238" s="8"/>
+      <c r="D238" s="9" t="s">
+        <v>844</v>
+      </c>
+      <c r="E238" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F238" s="7" t="s">
+        <v>845</v>
+      </c>
+      <c r="G238" s="7"/>
+      <c r="H238" s="10">
+        <v>44946</v>
+      </c>
+      <c r="I238" s="11">
+        <v>45311</v>
+      </c>
+      <c r="J238" s="12">
+        <v>45676</v>
+      </c>
+      <c r="K238" s="7" t="s">
+        <v>846</v>
+      </c>
+      <c r="L238" s="11">
+        <v>22666</v>
+      </c>
+      <c r="M238" s="11">
+        <v>44581</v>
+      </c>
+      <c r="N238" s="13"/>
+      <c r="O238" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P238" s="13">
+        <v>26201200102537</v>
+      </c>
+      <c r="Q238" s="14"/>
+      <c r="R238" s="15"/>
+      <c r="S238" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="239" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A239" s="7">
+        <v>237</v>
+      </c>
+      <c r="B239" s="7">
+        <v>180</v>
+      </c>
+      <c r="C239" s="8"/>
+      <c r="D239" s="9" t="s">
+        <v>847</v>
+      </c>
+      <c r="E239" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F239" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G239" s="7"/>
+      <c r="H239" s="10">
+        <v>44957</v>
+      </c>
+      <c r="I239" s="11">
+        <v>44957</v>
+      </c>
+      <c r="J239" s="12">
+        <v>45321</v>
+      </c>
+      <c r="K239" s="7" t="s">
+        <v>848</v>
+      </c>
+      <c r="L239" s="11"/>
+      <c r="M239" s="11"/>
+      <c r="N239" s="13"/>
+      <c r="O239" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P239" s="13"/>
+      <c r="Q239" s="14"/>
+      <c r="R239" s="15"/>
+      <c r="S239" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="240" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A240" s="7">
+        <v>238</v>
+      </c>
+      <c r="B240" s="7">
+        <v>20098</v>
+      </c>
+      <c r="C240" s="8"/>
+      <c r="D240" s="9" t="s">
+        <v>849</v>
+      </c>
+      <c r="E240" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F240" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="G240" s="7"/>
+      <c r="H240" s="10">
+        <v>44235</v>
+      </c>
+      <c r="I240" s="11">
+        <v>45420</v>
+      </c>
+      <c r="J240" s="12">
+        <v>45511</v>
+      </c>
+      <c r="K240" s="7" t="s">
+        <v>850</v>
+      </c>
+      <c r="L240" s="11">
+        <v>22251</v>
+      </c>
+      <c r="M240" s="11">
+        <v>44166</v>
+      </c>
+      <c r="N240" s="13"/>
+      <c r="O240" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P240" s="13">
+        <v>26012012200893</v>
+      </c>
+      <c r="Q240" s="14"/>
+      <c r="R240" s="15"/>
+      <c r="S240" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="241" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A241" s="7">
+        <v>239</v>
+      </c>
+      <c r="B241" s="7">
+        <v>169</v>
+      </c>
+      <c r="C241" s="8"/>
+      <c r="D241" s="9" t="s">
+        <v>851</v>
+      </c>
+      <c r="E241" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F241" s="7" t="s">
+        <v>852</v>
+      </c>
+      <c r="G241" s="7"/>
+      <c r="H241" s="10">
+        <v>44927</v>
+      </c>
+      <c r="I241" s="11">
+        <v>45474</v>
+      </c>
+      <c r="J241" s="12">
+        <v>45565</v>
+      </c>
+      <c r="K241" s="7" t="s">
+        <v>853</v>
+      </c>
+      <c r="L241" s="11">
+        <v>23008</v>
+      </c>
+      <c r="M241" s="11">
+        <v>44923</v>
+      </c>
+      <c r="N241" s="13"/>
+      <c r="O241" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P241" s="13">
+        <v>26212280104839</v>
+      </c>
+      <c r="Q241" s="14"/>
+      <c r="R241" s="15"/>
+      <c r="S241" s="7" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="242" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A242" s="7">
+        <v>240</v>
+      </c>
+      <c r="B242" s="7">
+        <v>20122</v>
+      </c>
+      <c r="C242" s="8"/>
+      <c r="D242" s="9" t="s">
+        <v>855</v>
+      </c>
+      <c r="E242" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F242" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G242" s="7"/>
+      <c r="H242" s="10">
+        <v>45363</v>
+      </c>
+      <c r="I242" s="11">
+        <v>45363</v>
+      </c>
+      <c r="J242" s="12"/>
+      <c r="K242" s="7" t="s">
+        <v>856</v>
+      </c>
+      <c r="L242" s="11">
+        <v>22414</v>
+      </c>
+      <c r="M242" s="11">
+        <v>44329</v>
+      </c>
+      <c r="N242" s="13"/>
+      <c r="O242" s="7"/>
+      <c r="P242" s="13">
+        <v>26105131401234</v>
+      </c>
+      <c r="Q242" s="14">
+        <v>1062087284</v>
+      </c>
+      <c r="R242" s="15"/>
+      <c r="S242" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="243" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A243" s="7">
+        <v>241</v>
+      </c>
+      <c r="B243" s="7">
+        <v>20170</v>
+      </c>
+      <c r="C243" s="8"/>
+      <c r="D243" s="9" t="s">
+        <v>857</v>
+      </c>
+      <c r="E243" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F243" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G243" s="7"/>
+      <c r="H243" s="10">
+        <v>44325</v>
+      </c>
+      <c r="I243" s="11">
+        <v>45421</v>
+      </c>
+      <c r="J243" s="12">
+        <v>45512</v>
+      </c>
+      <c r="K243" s="7" t="s">
+        <v>858</v>
+      </c>
+      <c r="L243" s="11">
+        <v>22397</v>
+      </c>
+      <c r="M243" s="11">
+        <v>44312</v>
+      </c>
+      <c r="N243" s="13"/>
+      <c r="O243" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P243" s="13">
+        <v>26104261701055</v>
+      </c>
+      <c r="Q243" s="14"/>
+      <c r="R243" s="15"/>
+      <c r="S243" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="244" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A244" s="7">
+        <v>242</v>
+      </c>
+      <c r="B244" s="7">
+        <v>20162</v>
+      </c>
+      <c r="C244" s="8">
+        <v>98</v>
+      </c>
+      <c r="D244" s="9" t="s">
+        <v>859</v>
+      </c>
+      <c r="E244" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F244" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G244" s="7"/>
+      <c r="H244" s="10">
+        <v>44368</v>
+      </c>
+      <c r="I244" s="11">
+        <v>45372</v>
+      </c>
+      <c r="J244" s="12">
+        <v>45463</v>
+      </c>
+      <c r="K244" s="7" t="s">
+        <v>860</v>
+      </c>
+      <c r="L244" s="11">
+        <v>22319</v>
+      </c>
+      <c r="M244" s="11">
+        <v>44234</v>
+      </c>
+      <c r="N244" s="13"/>
+      <c r="O244" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P244" s="13">
+        <v>26102071302313</v>
+      </c>
+      <c r="Q244" s="14"/>
+      <c r="R244" s="15"/>
+      <c r="S244" s="7" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="245" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A245" s="7">
+        <v>243</v>
+      </c>
+      <c r="B245" s="7">
+        <v>20201</v>
+      </c>
+      <c r="C245" s="8">
+        <v>141</v>
+      </c>
+      <c r="D245" s="9" t="s">
+        <v>861</v>
+      </c>
+      <c r="E245" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F245" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G245" s="7"/>
+      <c r="H245" s="10">
+        <v>44691</v>
+      </c>
+      <c r="I245" s="11">
+        <v>45698</v>
+      </c>
+      <c r="J245" s="12">
+        <v>45786</v>
+      </c>
+      <c r="K245" s="7" t="s">
+        <v>862</v>
+      </c>
+      <c r="L245" s="11">
+        <v>22744</v>
+      </c>
+      <c r="M245" s="11">
+        <v>44659</v>
+      </c>
+      <c r="N245" s="13"/>
+      <c r="O245" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P245" s="13">
+        <v>26204081400736</v>
+      </c>
+      <c r="Q245" s="14">
+        <v>1280523610</v>
+      </c>
+      <c r="R245" s="15"/>
+      <c r="S245" s="7" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="246" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A246" s="7">
+        <v>244</v>
+      </c>
+      <c r="B246" s="7">
+        <v>20244</v>
+      </c>
+      <c r="C246" s="8">
+        <v>182</v>
+      </c>
+      <c r="D246" s="9" t="s">
+        <v>864</v>
+      </c>
+      <c r="E246" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F246" s="7" t="s">
+        <v>865</v>
+      </c>
+      <c r="G246" s="7"/>
+      <c r="H246" s="10">
+        <v>45047</v>
+      </c>
+      <c r="I246" s="11">
+        <v>45413</v>
+      </c>
+      <c r="J246" s="12">
+        <v>45777</v>
+      </c>
+      <c r="K246" s="7" t="s">
+        <v>866</v>
+      </c>
+      <c r="L246" s="11">
+        <v>23102</v>
+      </c>
+      <c r="M246" s="11">
+        <v>45017</v>
+      </c>
+      <c r="N246" s="13"/>
+      <c r="O246" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P246" s="13">
+        <v>26304011400776</v>
+      </c>
+      <c r="Q246" s="14"/>
+      <c r="R246" s="15"/>
+      <c r="S246" s="7" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="247" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A247" s="7">
+        <v>245</v>
+      </c>
+      <c r="B247" s="7">
+        <v>20157</v>
+      </c>
+      <c r="C247" s="8">
+        <v>93</v>
+      </c>
+      <c r="D247" s="9" t="s">
+        <v>868</v>
+      </c>
+      <c r="E247" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F247" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G247" s="7"/>
+      <c r="H247" s="10">
+        <v>43832</v>
+      </c>
+      <c r="I247" s="11">
+        <v>45384</v>
+      </c>
+      <c r="J247" s="12">
+        <v>45809</v>
+      </c>
+      <c r="K247" s="7"/>
+      <c r="L247" s="11">
+        <v>21451</v>
+      </c>
+      <c r="M247" s="11">
+        <v>43366</v>
+      </c>
+      <c r="N247" s="13"/>
+      <c r="O247" s="7" t="s">
+        <v>869</v>
+      </c>
+      <c r="P247" s="13">
+        <v>25809230101238</v>
+      </c>
+      <c r="Q247" s="14">
+        <v>1148141435</v>
+      </c>
+      <c r="R247" s="15"/>
+      <c r="S247" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="248" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A248" s="7">
+        <v>246</v>
+      </c>
+      <c r="B248" s="7">
+        <v>20265</v>
+      </c>
+      <c r="C248" s="8">
+        <v>208</v>
+      </c>
+      <c r="D248" s="9" t="s">
+        <v>870</v>
+      </c>
+      <c r="E248" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F248" s="7" t="s">
+        <v>871</v>
+      </c>
+      <c r="G248" s="7"/>
+      <c r="H248" s="10">
+        <v>45374</v>
+      </c>
+      <c r="I248" s="11">
+        <v>45739</v>
+      </c>
+      <c r="J248" s="12">
+        <v>45830</v>
+      </c>
+      <c r="K248" s="7"/>
+      <c r="L248" s="11">
+        <v>23408</v>
+      </c>
+      <c r="M248" s="11">
+        <v>45323</v>
+      </c>
+      <c r="N248" s="13"/>
+      <c r="O248" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P248" s="13">
+        <v>26402011701018</v>
+      </c>
+      <c r="Q248" s="14">
+        <v>1202825386</v>
+      </c>
+      <c r="R248" s="15"/>
+      <c r="S248" s="7" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="249" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A249" s="7">
+        <v>247</v>
+      </c>
+      <c r="B249" s="7">
+        <v>20034</v>
+      </c>
+      <c r="C249" s="8">
+        <v>38</v>
+      </c>
+      <c r="D249" s="9" t="s">
+        <v>872</v>
+      </c>
+      <c r="E249" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F249" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G249" s="7"/>
+      <c r="H249" s="10">
+        <v>43312</v>
+      </c>
+      <c r="I249" s="11">
+        <v>45778</v>
+      </c>
+      <c r="J249" s="12">
+        <v>45868</v>
+      </c>
+      <c r="K249" s="7" t="s">
+        <v>873</v>
+      </c>
+      <c r="L249" s="11">
+        <v>20084</v>
+      </c>
+      <c r="M249" s="11">
+        <v>41999</v>
+      </c>
+      <c r="N249" s="13"/>
+      <c r="O249" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P249" s="13">
+        <v>25412261300231</v>
+      </c>
+      <c r="Q249" s="14">
+        <v>1220128618</v>
+      </c>
+      <c r="R249" s="15"/>
+      <c r="S249" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="250" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A250" s="7">
+        <v>248</v>
+      </c>
+      <c r="B250" s="7">
+        <v>20179</v>
+      </c>
+      <c r="C250" s="8">
+        <v>115</v>
+      </c>
+      <c r="D250" s="9" t="s">
+        <v>874</v>
+      </c>
+      <c r="E250" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F250" s="7" t="s">
+        <v>875</v>
+      </c>
+      <c r="G250" s="7"/>
+      <c r="H250" s="10">
+        <v>44333</v>
+      </c>
+      <c r="I250" s="11">
+        <v>45613</v>
+      </c>
+      <c r="J250" s="12">
+        <v>45977</v>
+      </c>
+      <c r="K250" s="7" t="s">
+        <v>876</v>
+      </c>
+      <c r="L250" s="11">
+        <v>22364</v>
+      </c>
+      <c r="M250" s="11">
+        <v>44279</v>
+      </c>
+      <c r="N250" s="13"/>
+      <c r="O250" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P250" s="13">
+        <v>26103240100659</v>
+      </c>
+      <c r="Q250" s="14"/>
+      <c r="R250" s="15"/>
+      <c r="S250" s="7" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="251" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A251" s="7">
+        <v>249</v>
+      </c>
+      <c r="B251" s="7">
+        <v>20109</v>
+      </c>
+      <c r="C251" s="8">
+        <v>25</v>
+      </c>
+      <c r="D251" s="9" t="s">
+        <v>878</v>
+      </c>
+      <c r="E251" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F251" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="G251" s="7"/>
+      <c r="H251" s="10">
+        <v>44454</v>
+      </c>
+      <c r="I251" s="11">
+        <v>45731</v>
+      </c>
+      <c r="J251" s="12">
+        <v>45822</v>
+      </c>
+      <c r="K251" s="7" t="s">
+        <v>879</v>
+      </c>
+      <c r="L251" s="11">
+        <v>22503</v>
+      </c>
+      <c r="M251" s="11">
+        <v>44418</v>
+      </c>
+      <c r="N251" s="13"/>
+      <c r="O251" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P251" s="13">
+        <v>26108102200792</v>
+      </c>
+      <c r="Q251" s="14">
+        <v>1142996504</v>
+      </c>
+      <c r="R251" s="15"/>
+      <c r="S251" s="7" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="252" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A252" s="7">
+        <v>250</v>
+      </c>
+      <c r="B252" s="7">
+        <v>20113</v>
+      </c>
+      <c r="C252" s="8">
+        <v>31</v>
+      </c>
+      <c r="D252" s="9" t="s">
+        <v>880</v>
+      </c>
+      <c r="E252" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F252" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G252" s="7"/>
+      <c r="H252" s="10">
+        <v>44376</v>
+      </c>
+      <c r="I252" s="11">
+        <v>45745</v>
+      </c>
+      <c r="J252" s="12">
+        <v>45836</v>
+      </c>
+      <c r="K252" s="7" t="s">
+        <v>881</v>
+      </c>
+      <c r="L252" s="11">
+        <v>22394</v>
+      </c>
+      <c r="M252" s="11">
+        <v>44309</v>
+      </c>
+      <c r="N252" s="13"/>
+      <c r="O252" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P252" s="13">
+        <v>26104231600971</v>
+      </c>
+      <c r="Q252" s="14">
+        <v>1270907591</v>
+      </c>
+      <c r="R252" s="15"/>
+      <c r="S252" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="253" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A253" s="7">
+        <v>251</v>
+      </c>
+      <c r="B253" s="7">
+        <v>20124</v>
+      </c>
+      <c r="C253" s="8">
+        <v>48</v>
+      </c>
+      <c r="D253" s="9" t="s">
+        <v>882</v>
+      </c>
+      <c r="E253" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F253" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G253" s="7"/>
+      <c r="H253" s="10">
+        <v>44335</v>
+      </c>
+      <c r="I253" s="11">
+        <v>45796</v>
+      </c>
+      <c r="J253" s="12">
+        <v>45887</v>
+      </c>
+      <c r="K253" s="7" t="s">
+        <v>883</v>
+      </c>
+      <c r="L253" s="11">
+        <v>22145</v>
+      </c>
+      <c r="M253" s="11">
+        <v>44060</v>
+      </c>
+      <c r="N253" s="13"/>
+      <c r="O253" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P253" s="13">
+        <v>26008170101595</v>
+      </c>
+      <c r="Q253" s="14"/>
+      <c r="R253" s="15"/>
+      <c r="S253" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="254" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A254" s="7">
+        <v>252</v>
+      </c>
+      <c r="B254" s="7">
+        <v>20343</v>
+      </c>
+      <c r="C254" s="8">
+        <v>278</v>
+      </c>
+      <c r="D254" s="9" t="s">
+        <v>884</v>
+      </c>
+      <c r="E254" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F254" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G254" s="7"/>
+      <c r="H254" s="10">
+        <v>45875</v>
+      </c>
+      <c r="I254" s="11">
+        <v>45875</v>
+      </c>
+      <c r="J254" s="12">
+        <v>45966</v>
+      </c>
+      <c r="K254" s="7" t="s">
+        <v>885</v>
+      </c>
+      <c r="L254" s="11"/>
+      <c r="M254" s="11"/>
+      <c r="N254" s="13"/>
+      <c r="O254" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P254" s="13"/>
+      <c r="Q254" s="14"/>
+      <c r="R254" s="15"/>
+      <c r="S254" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="255" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A255" s="7">
+        <v>253</v>
+      </c>
+      <c r="B255" s="7">
+        <v>20284</v>
+      </c>
+      <c r="C255" s="8">
+        <v>218</v>
+      </c>
+      <c r="D255" s="9" t="s">
+        <v>886</v>
+      </c>
+      <c r="E255" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F255" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="G255" s="7"/>
+      <c r="H255" s="10">
+        <v>45752</v>
+      </c>
+      <c r="I255" s="11">
+        <v>45752</v>
+      </c>
+      <c r="J255" s="12">
+        <v>45842</v>
+      </c>
+      <c r="K255" s="7" t="s">
+        <v>887</v>
+      </c>
+      <c r="L255" s="11">
+        <v>23090</v>
+      </c>
+      <c r="M255" s="11">
+        <v>45005</v>
+      </c>
+      <c r="N255" s="13"/>
+      <c r="O255" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P255" s="13">
+        <v>26303201701016</v>
+      </c>
+      <c r="Q255" s="14">
+        <v>1002976808</v>
+      </c>
+      <c r="R255" s="15"/>
+      <c r="S255" s="7" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="256" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A256" s="7">
+        <v>254</v>
+      </c>
+      <c r="B256" s="7">
+        <v>20292</v>
+      </c>
+      <c r="C256" s="8">
+        <v>226</v>
+      </c>
+      <c r="D256" s="9" t="s">
+        <v>888</v>
+      </c>
+      <c r="E256" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F256" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G256" s="7"/>
+      <c r="H256" s="10">
+        <v>45716</v>
+      </c>
+      <c r="I256" s="11">
+        <v>45715</v>
+      </c>
+      <c r="J256" s="12">
+        <v>45803</v>
+      </c>
+      <c r="K256" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="L256" s="11">
+        <v>23709</v>
+      </c>
+      <c r="M256" s="11">
+        <v>45624</v>
+      </c>
+      <c r="N256" s="13"/>
+      <c r="O256" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P256" s="13">
+        <v>26411281701094</v>
+      </c>
+      <c r="Q256" s="14">
+        <v>1062830905</v>
+      </c>
+      <c r="R256" s="15"/>
+      <c r="S256" s="7" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="257" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A257" s="7">
+        <v>255</v>
+      </c>
+      <c r="B257" s="7">
+        <v>20269</v>
+      </c>
+      <c r="C257" s="8">
+        <v>205</v>
+      </c>
+      <c r="D257" s="9" t="s">
+        <v>890</v>
+      </c>
+      <c r="E257" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F257" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G257" s="7"/>
+      <c r="H257" s="10">
+        <v>45383</v>
+      </c>
+      <c r="I257" s="11">
+        <v>45748</v>
+      </c>
+      <c r="J257" s="12">
+        <v>45838</v>
+      </c>
+      <c r="K257" s="7" t="s">
+        <v>891</v>
+      </c>
+      <c r="L257" s="11">
+        <v>23021</v>
+      </c>
+      <c r="M257" s="11">
+        <v>44936</v>
+      </c>
+      <c r="N257" s="13"/>
+      <c r="O257" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P257" s="13">
+        <v>26301100104472</v>
+      </c>
+      <c r="Q257" s="14">
+        <v>1270115952</v>
+      </c>
+      <c r="R257" s="15"/>
+      <c r="S257" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="258" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A258" s="7">
+        <v>256</v>
+      </c>
+      <c r="B258" s="7">
+        <v>20238</v>
+      </c>
+      <c r="C258" s="8">
+        <v>178</v>
+      </c>
+      <c r="D258" s="9" t="s">
+        <v>892</v>
+      </c>
+      <c r="E258" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F258" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G258" s="7"/>
+      <c r="H258" s="10">
+        <v>44961</v>
+      </c>
+      <c r="I258" s="11">
+        <v>45781</v>
+      </c>
+      <c r="J258" s="12">
+        <v>45872</v>
+      </c>
+      <c r="K258" s="7" t="s">
+        <v>893</v>
+      </c>
+      <c r="L258" s="11">
+        <v>22857</v>
+      </c>
+      <c r="M258" s="11">
+        <v>44772</v>
+      </c>
+      <c r="N258" s="13"/>
+      <c r="O258" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P258" s="13">
+        <v>26207302100359</v>
+      </c>
+      <c r="Q258" s="14"/>
+      <c r="R258" s="15"/>
+      <c r="S258" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="259" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A259" s="7">
+        <v>257</v>
+      </c>
+      <c r="B259" s="7">
+        <v>20221</v>
+      </c>
+      <c r="C259" s="8">
+        <v>161</v>
+      </c>
+      <c r="D259" s="9" t="s">
+        <v>894</v>
+      </c>
+      <c r="E259" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F259" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G259" s="7"/>
+      <c r="H259" s="10">
+        <v>44878</v>
+      </c>
+      <c r="I259" s="11">
+        <v>45882</v>
+      </c>
+      <c r="J259" s="12">
+        <v>45942</v>
+      </c>
+      <c r="K259" s="7" t="s">
+        <v>895</v>
+      </c>
+      <c r="L259" s="11">
+        <v>22943</v>
+      </c>
+      <c r="M259" s="11">
+        <v>44858</v>
+      </c>
+      <c r="N259" s="13"/>
+      <c r="O259" s="7" t="s">
+        <v>767</v>
+      </c>
+      <c r="P259" s="13">
+        <v>26210241400258</v>
+      </c>
+      <c r="Q259" s="14">
+        <v>1004279367</v>
+      </c>
+      <c r="R259" s="15"/>
+      <c r="S259" s="7" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="260" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A260" s="7">
+        <v>258</v>
+      </c>
+      <c r="B260" s="7">
+        <v>20285</v>
+      </c>
+      <c r="C260" s="8">
+        <v>219</v>
+      </c>
+      <c r="D260" s="9" t="s">
+        <v>896</v>
+      </c>
+      <c r="E260" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F260" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G260" s="7"/>
+      <c r="H260" s="10">
+        <v>45715</v>
+      </c>
+      <c r="I260" s="11">
+        <v>45715</v>
+      </c>
+      <c r="J260" s="12">
+        <v>45803</v>
+      </c>
+      <c r="K260" s="7" t="s">
+        <v>897</v>
+      </c>
+      <c r="L260" s="11">
+        <v>23740</v>
+      </c>
+      <c r="M260" s="11">
+        <v>45655</v>
+      </c>
+      <c r="N260" s="13"/>
+      <c r="O260" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P260" s="13">
+        <v>26412291402717</v>
+      </c>
+      <c r="Q260" s="14">
+        <v>1004348133</v>
+      </c>
+      <c r="R260" s="15"/>
+      <c r="S260" s="7" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="261" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A261" s="7">
+        <v>259</v>
+      </c>
+      <c r="B261" s="7">
+        <v>20126</v>
+      </c>
+      <c r="C261" s="8">
+        <v>50</v>
+      </c>
+      <c r="D261" s="9" t="s">
+        <v>898</v>
+      </c>
+      <c r="E261" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F261" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G261" s="7"/>
+      <c r="H261" s="10">
+        <v>44555</v>
+      </c>
+      <c r="I261" s="11">
+        <v>45741</v>
+      </c>
+      <c r="J261" s="12">
+        <v>46015</v>
+      </c>
+      <c r="K261" s="7" t="s">
+        <v>899</v>
+      </c>
+      <c r="L261" s="11">
+        <v>22465</v>
+      </c>
+      <c r="M261" s="11">
+        <v>44380</v>
+      </c>
+      <c r="N261" s="13"/>
+      <c r="O261" s="7" t="s">
+        <v>900</v>
+      </c>
+      <c r="P261" s="13">
+        <v>26107031300271</v>
+      </c>
+      <c r="Q261" s="14">
+        <v>1063238105</v>
+      </c>
+      <c r="R261" s="15"/>
+      <c r="S261" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="262" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A262" s="7">
+        <v>260</v>
+      </c>
+      <c r="B262" s="7">
+        <v>20377</v>
+      </c>
+      <c r="C262" s="8">
+        <v>312</v>
+      </c>
+      <c r="D262" s="9" t="s">
+        <v>901</v>
+      </c>
+      <c r="E262" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F262" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G262" s="7"/>
+      <c r="H262" s="10">
+        <v>45963</v>
+      </c>
+      <c r="I262" s="11">
+        <v>45963</v>
+      </c>
+      <c r="J262" s="12">
+        <v>46054</v>
+      </c>
+      <c r="K262" s="7" t="s">
+        <v>902</v>
+      </c>
+      <c r="L262" s="11"/>
+      <c r="M262" s="11"/>
+      <c r="N262" s="13"/>
+      <c r="O262" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P262" s="13"/>
+      <c r="Q262" s="14"/>
+      <c r="R262" s="15"/>
+      <c r="S262" s="7" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="263" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A263" s="7">
+        <v>261</v>
+      </c>
+      <c r="B263" s="7">
+        <v>306</v>
+      </c>
+      <c r="C263" s="8" t="s">
+        <v>903</v>
+      </c>
+      <c r="D263" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E263" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F263" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="G263" s="7"/>
+      <c r="H263" s="10">
+        <v>45952</v>
+      </c>
+      <c r="I263" s="11">
+        <v>45952</v>
+      </c>
+      <c r="J263" s="12">
+        <v>46043</v>
+      </c>
+      <c r="K263" s="7" t="s">
+        <v>904</v>
+      </c>
+      <c r="L263" s="11"/>
+      <c r="M263" s="11"/>
+      <c r="N263" s="13"/>
+      <c r="O263" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P263" s="13"/>
+      <c r="Q263" s="14"/>
+      <c r="R263" s="15"/>
+      <c r="S263" s="7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="264" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A264" s="7">
+        <v>262</v>
+      </c>
+      <c r="B264" s="7">
+        <v>20368</v>
+      </c>
+      <c r="C264" s="8">
+        <v>303</v>
+      </c>
+      <c r="D264" s="9" t="s">
+        <v>662</v>
+      </c>
+      <c r="E264" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F264" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G264" s="7"/>
+      <c r="H264" s="10">
+        <v>45931</v>
+      </c>
+      <c r="I264" s="11">
+        <v>45931</v>
+      </c>
+      <c r="J264" s="12">
+        <v>45931</v>
+      </c>
+      <c r="K264" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="L264" s="11"/>
+      <c r="M264" s="11"/>
+      <c r="N264" s="13"/>
+      <c r="O264" s="7"/>
+      <c r="P264" s="13"/>
+      <c r="Q264" s="14"/>
+      <c r="R264" s="15"/>
+      <c r="S264" s="7" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="265" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A265" s="7">
+        <v>263</v>
+      </c>
+      <c r="B265" s="7">
+        <v>20416</v>
+      </c>
+      <c r="C265" s="8">
+        <v>351</v>
+      </c>
+      <c r="D265" s="9" t="s">
+        <v>906</v>
+      </c>
+      <c r="E265" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F265" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G265" s="7"/>
+      <c r="H265" s="10"/>
+      <c r="I265" s="11"/>
+      <c r="J265" s="12"/>
+      <c r="K265" s="7" t="s">
+        <v>907</v>
+      </c>
+      <c r="L265" s="11"/>
+      <c r="M265" s="11"/>
+      <c r="N265" s="13"/>
+      <c r="O265" s="7"/>
+      <c r="P265" s="13"/>
+      <c r="Q265" s="14"/>
+      <c r="R265" s="15"/>
+      <c r="S265" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="266" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A266" s="7">
+        <v>264</v>
+      </c>
+      <c r="B266" s="7">
+        <v>20411</v>
+      </c>
+      <c r="C266" s="8">
+        <v>346</v>
+      </c>
+      <c r="D266" s="9" t="s">
+        <v>694</v>
+      </c>
+      <c r="E266" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F266" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G266" s="7"/>
+      <c r="H266" s="10">
+        <v>46069</v>
+      </c>
+      <c r="I266" s="11">
+        <v>46069</v>
+      </c>
+      <c r="J266" s="12">
+        <v>46069</v>
+      </c>
+      <c r="K266" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="L266" s="11"/>
+      <c r="M266" s="11"/>
+      <c r="N266" s="13"/>
+      <c r="O266" s="7"/>
+      <c r="P266" s="13"/>
+      <c r="Q266" s="14"/>
+      <c r="R266" s="15"/>
+      <c r="S266" s="7" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="267" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A267" s="7">
+        <v>265</v>
+      </c>
+      <c r="B267" s="7">
+        <v>20398</v>
+      </c>
+      <c r="C267" s="8">
+        <v>333</v>
+      </c>
+      <c r="D267" s="9" t="s">
+        <v>669</v>
+      </c>
+      <c r="E267" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F267" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G267" s="7"/>
+      <c r="H267" s="10">
+        <v>46041</v>
+      </c>
+      <c r="I267" s="11">
+        <v>46041</v>
+      </c>
+      <c r="J267" s="12">
+        <v>46041</v>
+      </c>
+      <c r="K267" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="L267" s="11"/>
+      <c r="M267" s="11"/>
+      <c r="N267" s="13"/>
+      <c r="O267" s="7"/>
+      <c r="P267" s="13"/>
+      <c r="Q267" s="14"/>
+      <c r="R267" s="15"/>
+      <c r="S267" s="7" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="268" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A268" s="7">
+        <v>266</v>
+      </c>
+      <c r="B268" s="7">
+        <v>342</v>
+      </c>
+      <c r="C268" s="8"/>
+      <c r="D268" s="9" t="s">
+        <v>677</v>
+      </c>
+      <c r="E268" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F268" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G268" s="7"/>
+      <c r="H268" s="10">
+        <v>46057</v>
+      </c>
+      <c r="I268" s="11">
+        <v>46057</v>
+      </c>
+      <c r="J268" s="12">
+        <v>46057</v>
+      </c>
+      <c r="K268" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="L268" s="11"/>
+      <c r="M268" s="11"/>
+      <c r="N268" s="13"/>
+      <c r="O268" s="7"/>
+      <c r="P268" s="13"/>
+      <c r="Q268" s="14"/>
+      <c r="R268" s="15"/>
+      <c r="S268" s="7" t="s">
+        <v>910</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S189"/>
+  <autoFilter ref="A2:S268"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
auto update (32 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -10056,7 +10056,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D189)</f>
-        <v>238</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -21024,9 +21024,7 @@
       <c r="P194" s="13"/>
       <c r="Q194" s="14"/>
       <c r="R194" s="15"/>
-      <c r="S194" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S194" s="7"/>
     </row>
     <row r="195" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A195" s="7">
@@ -21065,9 +21063,7 @@
       <c r="P195" s="13"/>
       <c r="Q195" s="14"/>
       <c r="R195" s="15"/>
-      <c r="S195" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S195" s="7"/>
     </row>
     <row r="196" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A196" s="7">
@@ -21098,9 +21094,7 @@
       <c r="P196" s="13"/>
       <c r="Q196" s="14"/>
       <c r="R196" s="15"/>
-      <c r="S196" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S196" s="7"/>
     </row>
     <row r="197" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A197" s="7">
@@ -21137,9 +21131,7 @@
       <c r="P197" s="13"/>
       <c r="Q197" s="14"/>
       <c r="R197" s="15"/>
-      <c r="S197" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S197" s="7"/>
     </row>
     <row r="198" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A198" s="7">
@@ -21178,9 +21170,7 @@
       <c r="P198" s="13"/>
       <c r="Q198" s="14"/>
       <c r="R198" s="15"/>
-      <c r="S198" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S198" s="7"/>
     </row>
     <row r="199" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A199" s="7">
@@ -21219,9 +21209,7 @@
       <c r="P199" s="13"/>
       <c r="Q199" s="14"/>
       <c r="R199" s="15"/>
-      <c r="S199" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S199" s="7"/>
     </row>
     <row r="200" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A200" s="7">
@@ -21260,9 +21248,7 @@
       <c r="P200" s="13"/>
       <c r="Q200" s="14"/>
       <c r="R200" s="15"/>
-      <c r="S200" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S200" s="7"/>
     </row>
     <row r="201" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A201" s="7">
@@ -21301,9 +21287,7 @@
       <c r="P201" s="13"/>
       <c r="Q201" s="14"/>
       <c r="R201" s="15"/>
-      <c r="S201" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S201" s="7"/>
     </row>
     <row r="202" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A202" s="7">
@@ -21342,9 +21326,7 @@
       <c r="P202" s="13"/>
       <c r="Q202" s="14"/>
       <c r="R202" s="15"/>
-      <c r="S202" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S202" s="7"/>
     </row>
     <row r="203" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A203" s="7">
@@ -21383,9 +21365,7 @@
       <c r="P203" s="13"/>
       <c r="Q203" s="14"/>
       <c r="R203" s="15"/>
-      <c r="S203" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S203" s="7"/>
     </row>
     <row r="204" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A204" s="7">
@@ -21422,9 +21402,7 @@
       <c r="P204" s="13"/>
       <c r="Q204" s="14"/>
       <c r="R204" s="15"/>
-      <c r="S204" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S204" s="7"/>
     </row>
     <row r="205" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A205" s="7">
@@ -21463,9 +21441,7 @@
       <c r="P205" s="13"/>
       <c r="Q205" s="14"/>
       <c r="R205" s="15"/>
-      <c r="S205" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S205" s="7"/>
     </row>
     <row r="206" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A206" s="7">
@@ -21504,9 +21480,7 @@
       <c r="P206" s="13"/>
       <c r="Q206" s="14"/>
       <c r="R206" s="15"/>
-      <c r="S206" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S206" s="7"/>
     </row>
     <row r="207" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A207" s="7">
@@ -21545,9 +21519,7 @@
       <c r="P207" s="13"/>
       <c r="Q207" s="14"/>
       <c r="R207" s="15"/>
-      <c r="S207" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S207" s="7"/>
     </row>
     <row r="208" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A208" s="7">
@@ -21586,9 +21558,7 @@
       <c r="P208" s="13"/>
       <c r="Q208" s="14"/>
       <c r="R208" s="15"/>
-      <c r="S208" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S208" s="7"/>
     </row>
     <row r="209" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A209" s="7">
@@ -21619,9 +21589,7 @@
       <c r="P209" s="13"/>
       <c r="Q209" s="14"/>
       <c r="R209" s="15"/>
-      <c r="S209" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S209" s="7"/>
     </row>
     <row r="210" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A210" s="7">
@@ -21660,9 +21628,7 @@
       <c r="P210" s="13"/>
       <c r="Q210" s="14"/>
       <c r="R210" s="15"/>
-      <c r="S210" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S210" s="7"/>
     </row>
     <row r="211" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A211" s="7">
@@ -21701,9 +21667,7 @@
       <c r="P211" s="13"/>
       <c r="Q211" s="14"/>
       <c r="R211" s="15"/>
-      <c r="S211" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S211" s="7"/>
     </row>
     <row r="212" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A212" s="7">
@@ -21742,9 +21706,7 @@
       <c r="P212" s="13"/>
       <c r="Q212" s="14"/>
       <c r="R212" s="15"/>
-      <c r="S212" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S212" s="7"/>
     </row>
     <row r="213" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A213" s="7">
@@ -21781,9 +21743,7 @@
       <c r="P213" s="13"/>
       <c r="Q213" s="14"/>
       <c r="R213" s="15"/>
-      <c r="S213" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S213" s="7"/>
     </row>
     <row r="214" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A214" s="7">
@@ -21822,9 +21782,7 @@
       <c r="P214" s="13"/>
       <c r="Q214" s="14"/>
       <c r="R214" s="15"/>
-      <c r="S214" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S214" s="7"/>
     </row>
     <row r="215" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A215" s="7">
@@ -21861,9 +21819,7 @@
       <c r="P215" s="13"/>
       <c r="Q215" s="14"/>
       <c r="R215" s="15"/>
-      <c r="S215" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S215" s="7"/>
     </row>
     <row r="216" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A216" s="7">
@@ -21902,9 +21858,7 @@
       <c r="P216" s="13"/>
       <c r="Q216" s="14"/>
       <c r="R216" s="15"/>
-      <c r="S216" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S216" s="7"/>
     </row>
     <row r="217" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A217" s="7">
@@ -21941,9 +21895,7 @@
       <c r="P217" s="13"/>
       <c r="Q217" s="14"/>
       <c r="R217" s="15"/>
-      <c r="S217" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S217" s="7"/>
     </row>
     <row r="218" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A218" s="7">
@@ -21982,9 +21934,7 @@
       <c r="P218" s="13"/>
       <c r="Q218" s="14"/>
       <c r="R218" s="15"/>
-      <c r="S218" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S218" s="7"/>
     </row>
     <row r="219" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A219" s="7">
@@ -22023,9 +21973,7 @@
       <c r="P219" s="13"/>
       <c r="Q219" s="14"/>
       <c r="R219" s="15"/>
-      <c r="S219" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S219" s="7"/>
     </row>
     <row r="220" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A220" s="7">
@@ -22064,9 +22012,7 @@
       <c r="P220" s="13"/>
       <c r="Q220" s="14"/>
       <c r="R220" s="15"/>
-      <c r="S220" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S220" s="7"/>
     </row>
     <row r="221" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A221" s="7">
@@ -22105,9 +22051,7 @@
       <c r="P221" s="13"/>
       <c r="Q221" s="14"/>
       <c r="R221" s="15"/>
-      <c r="S221" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S221" s="7"/>
     </row>
     <row r="222" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A222" s="7">
@@ -22146,9 +22090,7 @@
       <c r="P222" s="13"/>
       <c r="Q222" s="14"/>
       <c r="R222" s="15"/>
-      <c r="S222" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S222" s="7"/>
     </row>
     <row r="223" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A223" s="7">
@@ -22226,9 +22168,7 @@
       <c r="P224" s="13"/>
       <c r="Q224" s="14"/>
       <c r="R224" s="15"/>
-      <c r="S224" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S224" s="7"/>
     </row>
     <row r="225" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A225" s="7">
@@ -22921,9 +22861,7 @@
       <c r="P239" s="13"/>
       <c r="Q239" s="14"/>
       <c r="R239" s="15"/>
-      <c r="S239" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S239" s="7"/>
     </row>
     <row r="240" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A240" s="7">
@@ -24217,9 +24155,7 @@
       <c r="P265" s="13"/>
       <c r="Q265" s="14"/>
       <c r="R265" s="15"/>
-      <c r="S265" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S265" s="7"/>
     </row>
     <row r="266" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A266" s="7">

</xml_diff>

<commit_message>
auto update (1 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -24298,9 +24298,7 @@
       <c r="R265" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="S265" s="7" t="s">
-        <v>356</v>
-      </c>
+      <c r="S265" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:S265"/>

</xml_diff>

<commit_message>
auto update (2 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3483,10 +3483,10 @@
         <v>41730</v>
       </c>
       <c r="I5" s="11">
-        <v>46204</v>
+        <v>46316</v>
       </c>
       <c r="J5" s="12">
-        <v>46295</v>
+        <v>46407</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
auto update (0 cells, +0, -2)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3255,7 +3255,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S125"/>
+  <dimension ref="A1:S123"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -3283,7 +3283,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D122)</f>
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -9615,19 +9615,19 @@
         <v>112</v>
       </c>
       <c r="B114" s="7">
-        <v>20274</v>
+        <v>20211</v>
       </c>
       <c r="C114" s="8">
-        <v>19</v>
+        <v>151</v>
       </c>
       <c r="D114" s="9" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E114" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F114" s="7" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="G114" s="7" t="s">
         <v>180</v>
@@ -9652,19 +9652,19 @@
         <v>113</v>
       </c>
       <c r="B115" s="7">
-        <v>20276</v>
+        <v>20212</v>
       </c>
       <c r="C115" s="8">
-        <v>56</v>
+        <v>152</v>
       </c>
       <c r="D115" s="9" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="E115" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F115" s="7" t="s">
-        <v>180</v>
+        <v>352</v>
       </c>
       <c r="G115" s="7" t="s">
         <v>180</v>
@@ -9686,90 +9686,126 @@
     </row>
     <row r="116" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A116" s="7">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B116" s="7">
-        <v>20211</v>
+        <v>20422</v>
       </c>
       <c r="C116" s="8">
-        <v>151</v>
+        <v>357</v>
       </c>
       <c r="D116" s="9" t="s">
-        <v>351</v>
+        <v>155</v>
       </c>
       <c r="E116" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F116" s="7" t="s">
-        <v>352</v>
+        <v>68</v>
       </c>
       <c r="G116" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H116" s="10"/>
+        <v>68</v>
+      </c>
+      <c r="H116" s="10">
+        <v>46204</v>
+      </c>
       <c r="I116" s="11"/>
-      <c r="J116" s="12"/>
+      <c r="J116" s="12">
+        <v>46387</v>
+      </c>
       <c r="K116" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L116" s="11"/>
-      <c r="M116" s="11"/>
-      <c r="N116" s="13"/>
-      <c r="O116" s="7"/>
-      <c r="P116" s="13"/>
+        <v>153</v>
+      </c>
+      <c r="L116" s="11">
+        <v>24274</v>
+      </c>
+      <c r="M116" s="11">
+        <v>46189</v>
+      </c>
+      <c r="N116" s="13">
+        <v>3000</v>
+      </c>
+      <c r="O116" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="P116" s="13">
+        <v>26606161701631</v>
+      </c>
       <c r="Q116" s="16"/>
-      <c r="R116" s="15"/>
+      <c r="R116" s="15" t="s">
+        <v>156</v>
+      </c>
       <c r="S116" s="7"/>
     </row>
     <row r="117" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A117" s="7">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B117" s="7">
-        <v>20212</v>
+        <v>20427</v>
       </c>
       <c r="C117" s="8">
-        <v>152</v>
+        <v>362</v>
       </c>
       <c r="D117" s="9" t="s">
-        <v>353</v>
+        <v>273</v>
       </c>
       <c r="E117" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F117" s="7" t="s">
-        <v>352</v>
+        <v>22</v>
       </c>
       <c r="G117" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H117" s="10"/>
-      <c r="I117" s="11"/>
-      <c r="J117" s="12"/>
+        <v>22</v>
+      </c>
+      <c r="H117" s="10">
+        <v>46245</v>
+      </c>
+      <c r="I117" s="11">
+        <v>46337</v>
+      </c>
+      <c r="J117" s="12">
+        <v>46428</v>
+      </c>
       <c r="K117" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L117" s="11"/>
-      <c r="M117" s="11"/>
-      <c r="N117" s="13"/>
-      <c r="O117" s="7"/>
-      <c r="P117" s="13"/>
-      <c r="Q117" s="16"/>
-      <c r="R117" s="15"/>
+        <v>227</v>
+      </c>
+      <c r="L117" s="11">
+        <v>24264</v>
+      </c>
+      <c r="M117" s="11">
+        <v>46179</v>
+      </c>
+      <c r="N117" s="13">
+        <v>3000</v>
+      </c>
+      <c r="O117" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="P117" s="13">
+        <v>26606061701196</v>
+      </c>
+      <c r="Q117" s="16">
+        <v>1201261848</v>
+      </c>
+      <c r="R117" s="15" t="s">
+        <v>274</v>
+      </c>
       <c r="S117" s="7"/>
     </row>
     <row r="118" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A118" s="7">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B118" s="7">
-        <v>20422</v>
+        <v>20432</v>
       </c>
       <c r="C118" s="8">
-        <v>357</v>
+        <v>367</v>
       </c>
       <c r="D118" s="9" t="s">
-        <v>155</v>
+        <v>94</v>
       </c>
       <c r="E118" s="7" t="s">
         <v>20</v>
@@ -9778,23 +9814,25 @@
         <v>68</v>
       </c>
       <c r="G118" s="7" t="s">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="H118" s="10">
-        <v>46204</v>
-      </c>
-      <c r="I118" s="11"/>
+        <v>46285</v>
+      </c>
+      <c r="I118" s="11">
+        <v>46285</v>
+      </c>
       <c r="J118" s="12">
-        <v>46387</v>
+        <v>46375</v>
       </c>
       <c r="K118" s="7" t="s">
-        <v>153</v>
+        <v>95</v>
       </c>
       <c r="L118" s="11">
-        <v>24274</v>
+        <v>24355</v>
       </c>
       <c r="M118" s="11">
-        <v>46189</v>
+        <v>46270</v>
       </c>
       <c r="N118" s="13">
         <v>3000</v>
@@ -9803,207 +9841,191 @@
         <v>96</v>
       </c>
       <c r="P118" s="13">
-        <v>26606161701631</v>
-      </c>
-      <c r="Q118" s="16"/>
+        <v>26609050103873</v>
+      </c>
+      <c r="Q118" s="16">
+        <v>1200869587</v>
+      </c>
       <c r="R118" s="15" t="s">
-        <v>156</v>
+        <v>97</v>
       </c>
       <c r="S118" s="7"/>
     </row>
     <row r="119" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A119" s="7">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B119" s="7">
-        <v>20427</v>
-      </c>
-      <c r="C119" s="8">
-        <v>362</v>
+        <v>20440</v>
+      </c>
+      <c r="C119" s="8" t="s">
+        <v>233</v>
       </c>
       <c r="D119" s="9" t="s">
-        <v>273</v>
+        <v>234</v>
       </c>
       <c r="E119" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F119" s="7" t="s">
-        <v>22</v>
+        <v>235</v>
       </c>
       <c r="G119" s="7" t="s">
-        <v>22</v>
+        <v>236</v>
       </c>
       <c r="H119" s="10">
-        <v>46245</v>
+        <v>46327</v>
       </c>
       <c r="I119" s="11">
-        <v>46337</v>
+        <v>46327</v>
       </c>
       <c r="J119" s="12">
-        <v>46428</v>
+        <v>46418</v>
       </c>
       <c r="K119" s="7" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="L119" s="11">
-        <v>24264</v>
+        <v>24316</v>
       </c>
       <c r="M119" s="11">
-        <v>46179</v>
-      </c>
-      <c r="N119" s="13">
-        <v>3000</v>
-      </c>
+        <v>46231</v>
+      </c>
+      <c r="N119" s="13"/>
       <c r="O119" s="7" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="P119" s="13">
-        <v>26606061701196</v>
+        <v>26609161301038</v>
       </c>
       <c r="Q119" s="16">
-        <v>1201261848</v>
+        <v>1223226004</v>
       </c>
       <c r="R119" s="15" t="s">
-        <v>274</v>
+        <v>912</v>
       </c>
       <c r="S119" s="7"/>
     </row>
     <row r="120" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A120" s="7">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B120" s="7">
-        <v>20432</v>
+        <v>20274</v>
       </c>
       <c r="C120" s="8">
-        <v>367</v>
+        <v>19</v>
       </c>
       <c r="D120" s="9" t="s">
-        <v>94</v>
+        <v>348</v>
       </c>
       <c r="E120" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F120" s="7" t="s">
-        <v>68</v>
+        <v>347</v>
       </c>
       <c r="G120" s="7" t="s">
-        <v>22</v>
+        <v>180</v>
       </c>
       <c r="H120" s="10">
-        <v>46285</v>
-      </c>
-      <c r="I120" s="11">
-        <v>46285</v>
-      </c>
-      <c r="J120" s="12">
-        <v>46375</v>
-      </c>
+        <v>45139</v>
+      </c>
+      <c r="I120" s="11"/>
+      <c r="J120" s="12"/>
       <c r="K120" s="7" t="s">
-        <v>95</v>
+        <v>345</v>
       </c>
       <c r="L120" s="11">
-        <v>24355</v>
+        <v>22510</v>
       </c>
       <c r="M120" s="11">
-        <v>46270</v>
-      </c>
-      <c r="N120" s="13">
-        <v>3000</v>
-      </c>
-      <c r="O120" s="7" t="s">
-        <v>96</v>
-      </c>
+        <v>45117</v>
+      </c>
+      <c r="N120" s="13"/>
+      <c r="O120" s="7"/>
       <c r="P120" s="13">
-        <v>26609050103873</v>
-      </c>
-      <c r="Q120" s="16">
-        <v>1200869587</v>
-      </c>
-      <c r="R120" s="15" t="s">
-        <v>97</v>
-      </c>
+        <v>26108171301291</v>
+      </c>
+      <c r="Q120" s="16"/>
+      <c r="R120" s="15"/>
       <c r="S120" s="7"/>
     </row>
     <row r="121" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A121" s="7">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B121" s="7">
-        <v>20440</v>
-      </c>
-      <c r="C121" s="8" t="s">
-        <v>233</v>
+        <v>20276</v>
+      </c>
+      <c r="C121" s="8">
+        <v>56</v>
       </c>
       <c r="D121" s="9" t="s">
-        <v>234</v>
+        <v>350</v>
       </c>
       <c r="E121" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F121" s="7" t="s">
-        <v>235</v>
+        <v>180</v>
       </c>
       <c r="G121" s="7" t="s">
-        <v>236</v>
+        <v>180</v>
       </c>
       <c r="H121" s="10">
-        <v>46327</v>
+        <v>45263</v>
       </c>
       <c r="I121" s="11">
-        <v>46327</v>
+        <v>45721</v>
       </c>
       <c r="J121" s="12">
-        <v>46418</v>
+        <v>46085</v>
       </c>
       <c r="K121" s="7" t="s">
-        <v>237</v>
+        <v>345</v>
       </c>
       <c r="L121" s="11">
-        <v>24316</v>
+        <v>21886</v>
       </c>
       <c r="M121" s="11">
-        <v>46231</v>
+        <v>43801</v>
       </c>
       <c r="N121" s="13"/>
       <c r="O121" s="7" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="P121" s="13">
-        <v>26609161301038</v>
-      </c>
-      <c r="Q121" s="16">
-        <v>1223226004</v>
-      </c>
-      <c r="R121" s="15" t="s">
-        <v>912</v>
-      </c>
+        <v>25912021300059</v>
+      </c>
+      <c r="Q121" s="16"/>
+      <c r="R121" s="15"/>
       <c r="S121" s="7"/>
     </row>
     <row r="122" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A122" s="7">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B122" s="7">
-        <v>20274</v>
+        <v>20211</v>
       </c>
       <c r="C122" s="8">
-        <v>19</v>
+        <v>151</v>
       </c>
       <c r="D122" s="9" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E122" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F122" s="7" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="G122" s="7" t="s">
         <v>180</v>
       </c>
       <c r="H122" s="10">
-        <v>45139</v>
+        <v>44805</v>
       </c>
       <c r="I122" s="11"/>
       <c r="J122" s="12"/>
@@ -10011,15 +10033,15 @@
         <v>345</v>
       </c>
       <c r="L122" s="11">
-        <v>22510</v>
+        <v>22944</v>
       </c>
       <c r="M122" s="11">
-        <v>45117</v>
+        <v>44859</v>
       </c>
       <c r="N122" s="13"/>
       <c r="O122" s="7"/>
       <c r="P122" s="13">
-        <v>26108171301291</v>
+        <v>26210251400258</v>
       </c>
       <c r="Q122" s="16"/>
       <c r="R122" s="15"/>
@@ -10027,147 +10049,51 @@
     </row>
     <row r="123" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A123" s="7">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B123" s="7">
-        <v>20276</v>
+        <v>20212</v>
       </c>
       <c r="C123" s="8">
-        <v>56</v>
+        <v>152</v>
       </c>
       <c r="D123" s="9" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="E123" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F123" s="7" t="s">
-        <v>180</v>
+        <v>352</v>
       </c>
       <c r="G123" s="7" t="s">
         <v>180</v>
       </c>
       <c r="H123" s="10">
-        <v>45263</v>
-      </c>
-      <c r="I123" s="11">
-        <v>45721</v>
-      </c>
-      <c r="J123" s="12">
-        <v>46085</v>
-      </c>
+        <v>44814</v>
+      </c>
+      <c r="I123" s="11"/>
+      <c r="J123" s="12"/>
       <c r="K123" s="7" t="s">
         <v>345</v>
       </c>
       <c r="L123" s="11">
-        <v>21886</v>
+        <v>21539</v>
       </c>
       <c r="M123" s="11">
-        <v>43801</v>
+        <v>43454</v>
       </c>
       <c r="N123" s="13"/>
-      <c r="O123" s="7" t="s">
-        <v>56</v>
-      </c>
+      <c r="O123" s="7"/>
       <c r="P123" s="13">
-        <v>25912021300059</v>
+        <v>25812208800538</v>
       </c>
       <c r="Q123" s="16"/>
       <c r="R123" s="15"/>
       <c r="S123" s="7"/>
     </row>
-    <row r="124" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A124" s="7">
-        <v>127</v>
-      </c>
-      <c r="B124" s="7">
-        <v>20211</v>
-      </c>
-      <c r="C124" s="8">
-        <v>151</v>
-      </c>
-      <c r="D124" s="9" t="s">
-        <v>351</v>
-      </c>
-      <c r="E124" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F124" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G124" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H124" s="10">
-        <v>44805</v>
-      </c>
-      <c r="I124" s="11"/>
-      <c r="J124" s="12"/>
-      <c r="K124" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L124" s="11">
-        <v>22944</v>
-      </c>
-      <c r="M124" s="11">
-        <v>44859</v>
-      </c>
-      <c r="N124" s="13"/>
-      <c r="O124" s="7"/>
-      <c r="P124" s="13">
-        <v>26210251400258</v>
-      </c>
-      <c r="Q124" s="16"/>
-      <c r="R124" s="15"/>
-      <c r="S124" s="7"/>
-    </row>
-    <row r="125" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A125" s="7">
-        <v>128</v>
-      </c>
-      <c r="B125" s="7">
-        <v>20212</v>
-      </c>
-      <c r="C125" s="8">
-        <v>152</v>
-      </c>
-      <c r="D125" s="9" t="s">
-        <v>353</v>
-      </c>
-      <c r="E125" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F125" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G125" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H125" s="10">
-        <v>44814</v>
-      </c>
-      <c r="I125" s="11"/>
-      <c r="J125" s="12"/>
-      <c r="K125" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L125" s="11">
-        <v>21539</v>
-      </c>
-      <c r="M125" s="11">
-        <v>43454</v>
-      </c>
-      <c r="N125" s="13"/>
-      <c r="O125" s="7"/>
-      <c r="P125" s="13">
-        <v>25812208800538</v>
-      </c>
-      <c r="Q125" s="16"/>
-      <c r="R125" s="15"/>
-      <c r="S125" s="7"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:S125"/>
+  <autoFilter ref="A2:S123"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
auto update (0 cells, +1, -1)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3255,7 +3255,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S123"/>
+  <dimension ref="A1:S124"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -3283,7 +3283,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D122)</f>
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -10092,8 +10092,65 @@
       <c r="R123" s="15"/>
       <c r="S123" s="7"/>
     </row>
+    <row r="124" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A124" s="7">
+        <v>129</v>
+      </c>
+      <c r="B124" s="7">
+        <v>20078</v>
+      </c>
+      <c r="C124" s="8">
+        <v>71</v>
+      </c>
+      <c r="D124" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E124" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F124" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G124" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H124" s="10">
+        <v>40063</v>
+      </c>
+      <c r="I124" s="11">
+        <v>46174</v>
+      </c>
+      <c r="J124" s="12">
+        <v>46265</v>
+      </c>
+      <c r="K124" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="L124" s="11">
+        <v>17467</v>
+      </c>
+      <c r="M124" s="11">
+        <v>35730</v>
+      </c>
+      <c r="N124" s="13">
+        <v>3500</v>
+      </c>
+      <c r="O124" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P124" s="13">
+        <v>24710270101052</v>
+      </c>
+      <c r="Q124" s="16">
+        <v>1221545221</v>
+      </c>
+      <c r="R124" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="S124" s="7"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S123"/>
+  <autoFilter ref="A2:S124"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>
@@ -10107,7 +10164,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S265"/>
+  <dimension ref="A1:S264"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -10135,7 +10192,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D189)</f>
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -24169,65 +24226,8 @@
         <v>910</v>
       </c>
     </row>
-    <row r="265" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A265" s="7">
-        <v>267</v>
-      </c>
-      <c r="B265" s="7">
-        <v>20078</v>
-      </c>
-      <c r="C265" s="8">
-        <v>71</v>
-      </c>
-      <c r="D265" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E265" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F265" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G265" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H265" s="10">
-        <v>40063</v>
-      </c>
-      <c r="I265" s="11">
-        <v>46174</v>
-      </c>
-      <c r="J265" s="12">
-        <v>46265</v>
-      </c>
-      <c r="K265" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="L265" s="11">
-        <v>17467</v>
-      </c>
-      <c r="M265" s="11">
-        <v>35730</v>
-      </c>
-      <c r="N265" s="13">
-        <v>3500</v>
-      </c>
-      <c r="O265" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="P265" s="13">
-        <v>24710270101052</v>
-      </c>
-      <c r="Q265" s="14">
-        <v>1221545221</v>
-      </c>
-      <c r="R265" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="S265" s="7"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:S265"/>
+  <autoFilter ref="A2:S264"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
auto update (0 cells, +0, -1)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -10164,7 +10164,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S264"/>
+  <dimension ref="A1:S263"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -10192,7 +10192,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D189)</f>
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -21657,31 +21657,33 @@
       <c r="B209" s="7"/>
       <c r="C209" s="8"/>
       <c r="D209" s="9" t="s">
-        <v>305</v>
+        <v>785</v>
       </c>
       <c r="E209" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F209" s="7" t="s">
-        <v>783</v>
+        <v>786</v>
       </c>
       <c r="G209" s="7"/>
       <c r="H209" s="10">
-        <v>44827</v>
+        <v>44927</v>
       </c>
       <c r="I209" s="11">
-        <v>45169</v>
+        <v>45108</v>
       </c>
       <c r="J209" s="12">
-        <v>45169</v>
+        <v>45199</v>
       </c>
       <c r="K209" s="7" t="s">
-        <v>784</v>
+        <v>787</v>
       </c>
       <c r="L209" s="11"/>
       <c r="M209" s="11"/>
       <c r="N209" s="13"/>
-      <c r="O209" s="7"/>
+      <c r="O209" s="7" t="s">
+        <v>24</v>
+      </c>
       <c r="P209" s="13"/>
       <c r="Q209" s="14"/>
       <c r="R209" s="15"/>
@@ -21694,33 +21696,31 @@
       <c r="B210" s="7"/>
       <c r="C210" s="8"/>
       <c r="D210" s="9" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
       <c r="E210" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F210" s="7" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="G210" s="7"/>
       <c r="H210" s="10">
-        <v>44927</v>
+        <v>45029</v>
       </c>
       <c r="I210" s="11">
-        <v>45108</v>
+        <v>44968</v>
       </c>
       <c r="J210" s="12">
-        <v>45199</v>
+        <v>44968</v>
       </c>
       <c r="K210" s="7" t="s">
-        <v>787</v>
+        <v>790</v>
       </c>
       <c r="L210" s="11"/>
       <c r="M210" s="11"/>
       <c r="N210" s="13"/>
-      <c r="O210" s="7" t="s">
-        <v>24</v>
-      </c>
+      <c r="O210" s="7"/>
       <c r="P210" s="13"/>
       <c r="Q210" s="14"/>
       <c r="R210" s="15"/>
@@ -21733,31 +21733,33 @@
       <c r="B211" s="7"/>
       <c r="C211" s="8"/>
       <c r="D211" s="9" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="E211" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F211" s="7" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="G211" s="7"/>
       <c r="H211" s="10">
-        <v>45029</v>
+        <v>41640</v>
       </c>
       <c r="I211" s="11">
-        <v>44968</v>
+        <v>44927</v>
       </c>
       <c r="J211" s="12">
-        <v>44968</v>
+        <v>45138</v>
       </c>
       <c r="K211" s="7" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="L211" s="11"/>
       <c r="M211" s="11"/>
       <c r="N211" s="13"/>
-      <c r="O211" s="7"/>
+      <c r="O211" s="7" t="s">
+        <v>794</v>
+      </c>
       <c r="P211" s="13"/>
       <c r="Q211" s="14"/>
       <c r="R211" s="15"/>
@@ -21770,33 +21772,31 @@
       <c r="B212" s="7"/>
       <c r="C212" s="8"/>
       <c r="D212" s="9" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="E212" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F212" s="7" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="G212" s="7"/>
       <c r="H212" s="10">
-        <v>41640</v>
+        <v>44206</v>
       </c>
       <c r="I212" s="11">
-        <v>44927</v>
+        <v>45170</v>
       </c>
       <c r="J212" s="12">
-        <v>45138</v>
+        <v>45170</v>
       </c>
       <c r="K212" s="7" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="L212" s="11"/>
       <c r="M212" s="11"/>
       <c r="N212" s="13"/>
-      <c r="O212" s="7" t="s">
-        <v>794</v>
-      </c>
+      <c r="O212" s="7"/>
       <c r="P212" s="13"/>
       <c r="Q212" s="14"/>
       <c r="R212" s="15"/>
@@ -21809,31 +21809,33 @@
       <c r="B213" s="7"/>
       <c r="C213" s="8"/>
       <c r="D213" s="9" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="E213" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F213" s="7" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="G213" s="7"/>
       <c r="H213" s="10">
-        <v>44206</v>
+        <v>44571</v>
       </c>
       <c r="I213" s="11">
-        <v>45170</v>
+        <v>44844</v>
       </c>
       <c r="J213" s="12">
-        <v>45170</v>
+        <v>44955</v>
       </c>
       <c r="K213" s="7" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="L213" s="11"/>
       <c r="M213" s="11"/>
       <c r="N213" s="13"/>
-      <c r="O213" s="7"/>
+      <c r="O213" s="7" t="s">
+        <v>763</v>
+      </c>
       <c r="P213" s="13"/>
       <c r="Q213" s="14"/>
       <c r="R213" s="15"/>
@@ -21846,32 +21848,32 @@
       <c r="B214" s="7"/>
       <c r="C214" s="8"/>
       <c r="D214" s="9" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="E214" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F214" s="7" t="s">
-        <v>799</v>
+        <v>68</v>
       </c>
       <c r="G214" s="7"/>
       <c r="H214" s="10">
-        <v>44571</v>
+        <v>44632</v>
       </c>
       <c r="I214" s="11">
-        <v>44844</v>
+        <v>44997</v>
       </c>
       <c r="J214" s="12">
-        <v>44955</v>
+        <v>45088</v>
       </c>
       <c r="K214" s="7" t="s">
-        <v>800</v>
+        <v>802</v>
       </c>
       <c r="L214" s="11"/>
       <c r="M214" s="11"/>
       <c r="N214" s="13"/>
       <c r="O214" s="7" t="s">
-        <v>763</v>
+        <v>24</v>
       </c>
       <c r="P214" s="13"/>
       <c r="Q214" s="14"/>
@@ -21885,26 +21887,26 @@
       <c r="B215" s="7"/>
       <c r="C215" s="8"/>
       <c r="D215" s="9" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="E215" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F215" s="7" t="s">
-        <v>68</v>
+        <v>750</v>
       </c>
       <c r="G215" s="7"/>
       <c r="H215" s="10">
-        <v>44632</v>
+        <v>44629</v>
       </c>
       <c r="I215" s="11">
-        <v>44997</v>
+        <v>45086</v>
       </c>
       <c r="J215" s="12">
-        <v>45088</v>
+        <v>45177</v>
       </c>
       <c r="K215" s="7" t="s">
-        <v>802</v>
+        <v>766</v>
       </c>
       <c r="L215" s="11"/>
       <c r="M215" s="11"/>
@@ -21924,26 +21926,26 @@
       <c r="B216" s="7"/>
       <c r="C216" s="8"/>
       <c r="D216" s="9" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="E216" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F216" s="7" t="s">
-        <v>750</v>
+        <v>805</v>
       </c>
       <c r="G216" s="7"/>
       <c r="H216" s="10">
-        <v>44629</v>
+        <v>42102</v>
       </c>
       <c r="I216" s="11">
-        <v>45086</v>
+        <v>45115</v>
       </c>
       <c r="J216" s="12">
-        <v>45177</v>
+        <v>45206</v>
       </c>
       <c r="K216" s="7" t="s">
-        <v>766</v>
+        <v>321</v>
       </c>
       <c r="L216" s="11"/>
       <c r="M216" s="11"/>
@@ -21963,26 +21965,26 @@
       <c r="B217" s="7"/>
       <c r="C217" s="8"/>
       <c r="D217" s="9" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="E217" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F217" s="7" t="s">
-        <v>805</v>
+        <v>27</v>
       </c>
       <c r="G217" s="7"/>
       <c r="H217" s="10">
-        <v>42102</v>
+        <v>43234</v>
       </c>
       <c r="I217" s="11">
-        <v>45115</v>
+        <v>45152</v>
       </c>
       <c r="J217" s="12">
-        <v>45206</v>
+        <v>45243</v>
       </c>
       <c r="K217" s="7" t="s">
-        <v>321</v>
+        <v>32</v>
       </c>
       <c r="L217" s="11"/>
       <c r="M217" s="11"/>
@@ -22002,7 +22004,7 @@
       <c r="B218" s="7"/>
       <c r="C218" s="8"/>
       <c r="D218" s="9" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="E218" s="7" t="s">
         <v>20</v>
@@ -22012,17 +22014,15 @@
       </c>
       <c r="G218" s="7"/>
       <c r="H218" s="10">
-        <v>43234</v>
+        <v>44625</v>
       </c>
       <c r="I218" s="11">
-        <v>45152</v>
+        <v>45174</v>
       </c>
       <c r="J218" s="12">
-        <v>45243</v>
-      </c>
-      <c r="K218" s="7" t="s">
-        <v>32</v>
-      </c>
+        <v>45264</v>
+      </c>
+      <c r="K218" s="7"/>
       <c r="L218" s="11"/>
       <c r="M218" s="11"/>
       <c r="N218" s="13"/>
@@ -22032,7 +22032,9 @@
       <c r="P218" s="13"/>
       <c r="Q218" s="14"/>
       <c r="R218" s="15"/>
-      <c r="S218" s="7"/>
+      <c r="S218" s="7" t="s">
+        <v>808</v>
+      </c>
     </row>
     <row r="219" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A219" s="7">
@@ -22041,37 +22043,37 @@
       <c r="B219" s="7"/>
       <c r="C219" s="8"/>
       <c r="D219" s="9" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="E219" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F219" s="7" t="s">
-        <v>27</v>
+        <v>810</v>
       </c>
       <c r="G219" s="7"/>
       <c r="H219" s="10">
-        <v>44625</v>
+        <v>40124</v>
       </c>
       <c r="I219" s="11">
-        <v>45174</v>
+        <v>44927</v>
       </c>
       <c r="J219" s="12">
-        <v>45264</v>
-      </c>
-      <c r="K219" s="7"/>
+        <v>45291</v>
+      </c>
+      <c r="K219" s="7" t="s">
+        <v>321</v>
+      </c>
       <c r="L219" s="11"/>
       <c r="M219" s="11"/>
       <c r="N219" s="13"/>
       <c r="O219" s="7" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="P219" s="13"/>
       <c r="Q219" s="14"/>
       <c r="R219" s="15"/>
-      <c r="S219" s="7" t="s">
-        <v>808</v>
-      </c>
+      <c r="S219" s="7"/>
     </row>
     <row r="220" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A220" s="7">
@@ -22080,37 +22082,37 @@
       <c r="B220" s="7"/>
       <c r="C220" s="8"/>
       <c r="D220" s="9" t="s">
-        <v>809</v>
+        <v>811</v>
       </c>
       <c r="E220" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F220" s="7" t="s">
-        <v>810</v>
+        <v>750</v>
       </c>
       <c r="G220" s="7"/>
       <c r="H220" s="10">
-        <v>40124</v>
+        <v>44238</v>
       </c>
       <c r="I220" s="11">
-        <v>44927</v>
+        <v>45241</v>
       </c>
       <c r="J220" s="12">
-        <v>45291</v>
-      </c>
-      <c r="K220" s="7" t="s">
-        <v>321</v>
-      </c>
+        <v>45332</v>
+      </c>
+      <c r="K220" s="7"/>
       <c r="L220" s="11"/>
       <c r="M220" s="11"/>
       <c r="N220" s="13"/>
       <c r="O220" s="7" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="P220" s="13"/>
       <c r="Q220" s="14"/>
       <c r="R220" s="15"/>
-      <c r="S220" s="7"/>
+      <c r="S220" s="7" t="s">
+        <v>812</v>
+      </c>
     </row>
     <row r="221" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A221" s="7">
@@ -22119,25 +22121,27 @@
       <c r="B221" s="7"/>
       <c r="C221" s="8"/>
       <c r="D221" s="9" t="s">
-        <v>811</v>
+        <v>813</v>
       </c>
       <c r="E221" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F221" s="7" t="s">
-        <v>750</v>
+        <v>417</v>
       </c>
       <c r="G221" s="7"/>
       <c r="H221" s="10">
-        <v>44238</v>
+        <v>44832</v>
       </c>
       <c r="I221" s="11">
-        <v>45241</v>
+        <v>45288</v>
       </c>
       <c r="J221" s="12">
-        <v>45332</v>
-      </c>
-      <c r="K221" s="7"/>
+        <v>45378</v>
+      </c>
+      <c r="K221" s="7" t="s">
+        <v>373</v>
+      </c>
       <c r="L221" s="11"/>
       <c r="M221" s="11"/>
       <c r="N221" s="13"/>
@@ -22148,48 +22152,58 @@
       <c r="Q221" s="14"/>
       <c r="R221" s="15"/>
       <c r="S221" s="7" t="s">
-        <v>812</v>
+        <v>814</v>
       </c>
     </row>
     <row r="222" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A222" s="7">
         <v>220</v>
       </c>
-      <c r="B222" s="7"/>
+      <c r="B222" s="7">
+        <v>44</v>
+      </c>
       <c r="C222" s="8"/>
       <c r="D222" s="9" t="s">
-        <v>813</v>
+        <v>815</v>
       </c>
       <c r="E222" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F222" s="7" t="s">
-        <v>417</v>
+        <v>27</v>
       </c>
       <c r="G222" s="7"/>
       <c r="H222" s="10">
-        <v>44832</v>
+        <v>44311</v>
       </c>
       <c r="I222" s="11">
-        <v>45288</v>
+        <v>45316</v>
       </c>
       <c r="J222" s="12">
-        <v>45378</v>
+        <v>45406</v>
       </c>
       <c r="K222" s="7" t="s">
-        <v>373</v>
-      </c>
-      <c r="L222" s="11"/>
-      <c r="M222" s="11"/>
+        <v>32</v>
+      </c>
+      <c r="L222" s="11">
+        <v>22362</v>
+      </c>
+      <c r="M222" s="11">
+        <v>44277</v>
+      </c>
       <c r="N222" s="13"/>
       <c r="O222" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="P222" s="13"/>
-      <c r="Q222" s="14"/>
+      <c r="P222" s="13">
+        <v>26103221701013</v>
+      </c>
+      <c r="Q222" s="14">
+        <v>1228894728</v>
+      </c>
       <c r="R222" s="15"/>
       <c r="S222" s="7" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
     </row>
     <row r="223" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22197,50 +22211,40 @@
         <v>221</v>
       </c>
       <c r="B223" s="7">
-        <v>44</v>
+        <v>209</v>
       </c>
       <c r="C223" s="8"/>
       <c r="D223" s="9" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="E223" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F223" s="7" t="s">
-        <v>27</v>
+        <v>256</v>
       </c>
       <c r="G223" s="7"/>
-      <c r="H223" s="10">
-        <v>44311</v>
-      </c>
-      <c r="I223" s="11">
-        <v>45316</v>
-      </c>
-      <c r="J223" s="12">
-        <v>45406</v>
-      </c>
+      <c r="H223" s="10"/>
+      <c r="I223" s="11"/>
+      <c r="J223" s="12"/>
       <c r="K223" s="7" t="s">
-        <v>32</v>
+        <v>224</v>
       </c>
       <c r="L223" s="11">
-        <v>22362</v>
+        <v>23460</v>
       </c>
       <c r="M223" s="11">
-        <v>44277</v>
+        <v>45375</v>
       </c>
       <c r="N223" s="13"/>
-      <c r="O223" s="7" t="s">
-        <v>24</v>
-      </c>
+      <c r="O223" s="7"/>
       <c r="P223" s="13">
-        <v>26103221701013</v>
-      </c>
-      <c r="Q223" s="14">
-        <v>1228894728</v>
-      </c>
+        <v>26403241301899</v>
+      </c>
+      <c r="Q223" s="14"/>
       <c r="R223" s="15"/>
       <c r="S223" s="7" t="s">
-        <v>816</v>
+        <v>818</v>
       </c>
     </row>
     <row r="224" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22248,40 +22252,50 @@
         <v>222</v>
       </c>
       <c r="B224" s="7">
-        <v>209</v>
+        <v>179</v>
       </c>
       <c r="C224" s="8"/>
       <c r="D224" s="9" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
       <c r="E224" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F224" s="7" t="s">
-        <v>256</v>
+        <v>21</v>
       </c>
       <c r="G224" s="7"/>
-      <c r="H224" s="10"/>
-      <c r="I224" s="11"/>
-      <c r="J224" s="12"/>
+      <c r="H224" s="10">
+        <v>44954</v>
+      </c>
+      <c r="I224" s="11">
+        <v>45319</v>
+      </c>
+      <c r="J224" s="12">
+        <v>45409</v>
+      </c>
       <c r="K224" s="7" t="s">
-        <v>224</v>
+        <v>820</v>
       </c>
       <c r="L224" s="11">
-        <v>23460</v>
+        <v>23017</v>
       </c>
       <c r="M224" s="11">
-        <v>45375</v>
+        <v>44932</v>
       </c>
       <c r="N224" s="13"/>
-      <c r="O224" s="7"/>
+      <c r="O224" s="7" t="s">
+        <v>24</v>
+      </c>
       <c r="P224" s="13">
-        <v>26403241301899</v>
-      </c>
-      <c r="Q224" s="14"/>
+        <v>26301061701735</v>
+      </c>
+      <c r="Q224" s="14">
+        <v>1225942643</v>
+      </c>
       <c r="R224" s="15"/>
       <c r="S224" s="7" t="s">
-        <v>818</v>
+        <v>821</v>
       </c>
     </row>
     <row r="225" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22289,50 +22303,40 @@
         <v>223</v>
       </c>
       <c r="B225" s="7">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C225" s="8"/>
       <c r="D225" s="9" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="E225" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F225" s="7" t="s">
-        <v>21</v>
+        <v>823</v>
       </c>
       <c r="G225" s="7"/>
       <c r="H225" s="10">
-        <v>44954</v>
+        <v>45073</v>
       </c>
       <c r="I225" s="11">
-        <v>45319</v>
+        <v>45073</v>
       </c>
       <c r="J225" s="12">
-        <v>45409</v>
-      </c>
-      <c r="K225" s="7" t="s">
-        <v>820</v>
-      </c>
-      <c r="L225" s="11">
-        <v>23017</v>
-      </c>
-      <c r="M225" s="11">
-        <v>44932</v>
-      </c>
+        <v>45438</v>
+      </c>
+      <c r="K225" s="7"/>
+      <c r="L225" s="11"/>
+      <c r="M225" s="11"/>
       <c r="N225" s="13"/>
       <c r="O225" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="P225" s="13">
-        <v>26301061701735</v>
-      </c>
-      <c r="Q225" s="14">
-        <v>1225942643</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="P225" s="13"/>
+      <c r="Q225" s="14"/>
       <c r="R225" s="15"/>
       <c r="S225" s="7" t="s">
-        <v>821</v>
+        <v>824</v>
       </c>
     </row>
     <row r="226" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22340,40 +22344,42 @@
         <v>224</v>
       </c>
       <c r="B226" s="7">
-        <v>183</v>
+        <v>131</v>
       </c>
       <c r="C226" s="8"/>
       <c r="D226" s="9" t="s">
-        <v>822</v>
+        <v>825</v>
       </c>
       <c r="E226" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F226" s="7" t="s">
-        <v>823</v>
+        <v>302</v>
       </c>
       <c r="G226" s="7"/>
       <c r="H226" s="10">
-        <v>45073</v>
+        <v>44567</v>
       </c>
       <c r="I226" s="11">
-        <v>45073</v>
+        <v>45297</v>
       </c>
       <c r="J226" s="12">
-        <v>45438</v>
-      </c>
-      <c r="K226" s="7"/>
+        <v>45478</v>
+      </c>
+      <c r="K226" s="7" t="s">
+        <v>137</v>
+      </c>
       <c r="L226" s="11"/>
       <c r="M226" s="11"/>
       <c r="N226" s="13"/>
       <c r="O226" s="7" t="s">
-        <v>56</v>
+        <v>583</v>
       </c>
       <c r="P226" s="13"/>
       <c r="Q226" s="14"/>
       <c r="R226" s="15"/>
       <c r="S226" s="7" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
     </row>
     <row r="227" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22381,42 +22387,42 @@
         <v>225</v>
       </c>
       <c r="B227" s="7">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C227" s="8"/>
       <c r="D227" s="9" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="E227" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F227" s="7" t="s">
-        <v>302</v>
+        <v>828</v>
       </c>
       <c r="G227" s="7"/>
       <c r="H227" s="10">
-        <v>44567</v>
+        <v>40776</v>
       </c>
       <c r="I227" s="11">
-        <v>45297</v>
+        <v>45105</v>
       </c>
       <c r="J227" s="12">
-        <v>45478</v>
+        <v>45470</v>
       </c>
       <c r="K227" s="7" t="s">
-        <v>137</v>
+        <v>829</v>
       </c>
       <c r="L227" s="11"/>
       <c r="M227" s="11"/>
       <c r="N227" s="13"/>
       <c r="O227" s="7" t="s">
-        <v>583</v>
+        <v>56</v>
       </c>
       <c r="P227" s="13"/>
       <c r="Q227" s="14"/>
       <c r="R227" s="15"/>
       <c r="S227" s="7" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
     </row>
     <row r="228" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22424,42 +22430,50 @@
         <v>226</v>
       </c>
       <c r="B228" s="7">
-        <v>124</v>
+        <v>63</v>
       </c>
       <c r="C228" s="8"/>
       <c r="D228" s="9" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="E228" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F228" s="7" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
       <c r="G228" s="7"/>
       <c r="H228" s="10">
-        <v>40776</v>
+        <v>44409</v>
       </c>
       <c r="I228" s="11">
-        <v>45105</v>
+        <v>45505</v>
       </c>
       <c r="J228" s="12">
-        <v>45470</v>
+        <v>45596</v>
       </c>
       <c r="K228" s="7" t="s">
-        <v>829</v>
-      </c>
-      <c r="L228" s="11"/>
-      <c r="M228" s="11"/>
+        <v>833</v>
+      </c>
+      <c r="L228" s="11">
+        <v>20885</v>
+      </c>
+      <c r="M228" s="11">
+        <v>42800</v>
+      </c>
       <c r="N228" s="13"/>
       <c r="O228" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="P228" s="13"/>
-      <c r="Q228" s="14"/>
+        <v>24</v>
+      </c>
+      <c r="P228" s="13">
+        <v>25703062201377</v>
+      </c>
+      <c r="Q228" s="14">
+        <v>1201992554</v>
+      </c>
       <c r="R228" s="15"/>
       <c r="S228" s="7" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
     </row>
     <row r="229" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22467,50 +22481,50 @@
         <v>227</v>
       </c>
       <c r="B229" s="7">
-        <v>63</v>
+        <v>20119</v>
       </c>
       <c r="C229" s="8"/>
       <c r="D229" s="9" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="E229" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F229" s="7" t="s">
-        <v>832</v>
+        <v>27</v>
       </c>
       <c r="G229" s="7"/>
       <c r="H229" s="10">
-        <v>44409</v>
+        <v>43740</v>
       </c>
       <c r="I229" s="11">
-        <v>45505</v>
+        <v>45475</v>
       </c>
       <c r="J229" s="12">
-        <v>45596</v>
+        <v>45566</v>
       </c>
       <c r="K229" s="7" t="s">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="L229" s="11">
-        <v>20885</v>
+        <v>21095</v>
       </c>
       <c r="M229" s="11">
-        <v>42800</v>
+        <v>43010</v>
       </c>
       <c r="N229" s="13"/>
       <c r="O229" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P229" s="13">
-        <v>25703062201377</v>
+        <v>25710020102391</v>
       </c>
       <c r="Q229" s="14">
-        <v>1201992554</v>
+        <v>1282057201</v>
       </c>
       <c r="R229" s="15"/>
       <c r="S229" s="7" t="s">
-        <v>834</v>
+        <v>29</v>
       </c>
     </row>
     <row r="230" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22518,11 +22532,11 @@
         <v>228</v>
       </c>
       <c r="B230" s="7">
-        <v>20119</v>
+        <v>20270</v>
       </c>
       <c r="C230" s="8"/>
       <c r="D230" s="9" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="E230" s="7" t="s">
         <v>20</v>
@@ -22532,32 +22546,32 @@
       </c>
       <c r="G230" s="7"/>
       <c r="H230" s="10">
-        <v>43740</v>
+        <v>45383</v>
       </c>
       <c r="I230" s="11">
-        <v>45475</v>
+        <v>45383</v>
       </c>
       <c r="J230" s="12">
-        <v>45566</v>
+        <v>45473</v>
       </c>
       <c r="K230" s="7" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="L230" s="11">
-        <v>21095</v>
+        <v>23380</v>
       </c>
       <c r="M230" s="11">
-        <v>43010</v>
+        <v>45295</v>
       </c>
       <c r="N230" s="13"/>
       <c r="O230" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P230" s="13">
-        <v>25710020102391</v>
+        <v>26401041400717</v>
       </c>
       <c r="Q230" s="14">
-        <v>1282057201</v>
+        <v>1141614868</v>
       </c>
       <c r="R230" s="15"/>
       <c r="S230" s="7" t="s">
@@ -22569,50 +22583,48 @@
         <v>229</v>
       </c>
       <c r="B231" s="7">
-        <v>20270</v>
+        <v>73</v>
       </c>
       <c r="C231" s="8"/>
       <c r="D231" s="9" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
       <c r="E231" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F231" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G231" s="7"/>
       <c r="H231" s="10">
-        <v>45383</v>
+        <v>42054</v>
       </c>
       <c r="I231" s="11">
-        <v>45383</v>
+        <v>45431</v>
       </c>
       <c r="J231" s="12">
-        <v>45473</v>
+        <v>45522</v>
       </c>
       <c r="K231" s="7" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="L231" s="11">
-        <v>23380</v>
+        <v>20136</v>
       </c>
       <c r="M231" s="11">
-        <v>45295</v>
+        <v>42051</v>
       </c>
       <c r="N231" s="13"/>
       <c r="O231" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P231" s="13">
-        <v>26401041400717</v>
-      </c>
-      <c r="Q231" s="14">
-        <v>1141614868</v>
-      </c>
+        <v>25502160102454</v>
+      </c>
+      <c r="Q231" s="14"/>
       <c r="R231" s="15"/>
       <c r="S231" s="7" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
     </row>
     <row r="232" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22620,48 +22632,50 @@
         <v>230</v>
       </c>
       <c r="B232" s="7">
-        <v>73</v>
+        <v>159</v>
       </c>
       <c r="C232" s="8"/>
       <c r="D232" s="9" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
       <c r="E232" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F232" s="7" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G232" s="7"/>
       <c r="H232" s="10">
-        <v>42054</v>
+        <v>44847</v>
       </c>
       <c r="I232" s="11">
-        <v>45431</v>
+        <v>44847</v>
       </c>
       <c r="J232" s="12">
-        <v>45522</v>
+        <v>45395</v>
       </c>
       <c r="K232" s="7" t="s">
-        <v>840</v>
+        <v>29</v>
       </c>
       <c r="L232" s="11">
-        <v>20136</v>
+        <v>22915</v>
       </c>
       <c r="M232" s="11">
-        <v>42051</v>
+        <v>44830</v>
       </c>
       <c r="N232" s="13"/>
       <c r="O232" s="7" t="s">
-        <v>24</v>
+        <v>842</v>
       </c>
       <c r="P232" s="13">
-        <v>25502160102454</v>
-      </c>
-      <c r="Q232" s="14"/>
+        <v>26209260101905</v>
+      </c>
+      <c r="Q232" s="14">
+        <v>1270942558</v>
+      </c>
       <c r="R232" s="15"/>
       <c r="S232" s="7" t="s">
-        <v>44</v>
+        <v>843</v>
       </c>
     </row>
     <row r="233" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22669,50 +22683,48 @@
         <v>231</v>
       </c>
       <c r="B233" s="7">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C233" s="8"/>
       <c r="D233" s="9" t="s">
-        <v>841</v>
+        <v>844</v>
       </c>
       <c r="E233" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F233" s="7" t="s">
-        <v>27</v>
+        <v>845</v>
       </c>
       <c r="G233" s="7"/>
       <c r="H233" s="10">
-        <v>44847</v>
+        <v>44946</v>
       </c>
       <c r="I233" s="11">
-        <v>44847</v>
+        <v>45311</v>
       </c>
       <c r="J233" s="12">
-        <v>45395</v>
+        <v>45676</v>
       </c>
       <c r="K233" s="7" t="s">
-        <v>29</v>
+        <v>846</v>
       </c>
       <c r="L233" s="11">
-        <v>22915</v>
+        <v>22666</v>
       </c>
       <c r="M233" s="11">
-        <v>44830</v>
+        <v>44581</v>
       </c>
       <c r="N233" s="13"/>
       <c r="O233" s="7" t="s">
-        <v>842</v>
+        <v>56</v>
       </c>
       <c r="P233" s="13">
-        <v>26209260101905</v>
-      </c>
-      <c r="Q233" s="14">
-        <v>1270942558</v>
-      </c>
+        <v>26201200102537</v>
+      </c>
+      <c r="Q233" s="14"/>
       <c r="R233" s="15"/>
       <c r="S233" s="7" t="s">
-        <v>843</v>
+        <v>314</v>
       </c>
     </row>
     <row r="234" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22720,138 +22732,138 @@
         <v>232</v>
       </c>
       <c r="B234" s="7">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="C234" s="8"/>
       <c r="D234" s="9" t="s">
-        <v>844</v>
+        <v>847</v>
       </c>
       <c r="E234" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F234" s="7" t="s">
-        <v>845</v>
+        <v>180</v>
       </c>
       <c r="G234" s="7"/>
       <c r="H234" s="10">
-        <v>44946</v>
+        <v>44957</v>
       </c>
       <c r="I234" s="11">
-        <v>45311</v>
+        <v>44957</v>
       </c>
       <c r="J234" s="12">
-        <v>45676</v>
+        <v>45321</v>
       </c>
       <c r="K234" s="7" t="s">
-        <v>846</v>
-      </c>
-      <c r="L234" s="11">
-        <v>22666</v>
-      </c>
-      <c r="M234" s="11">
-        <v>44581</v>
-      </c>
+        <v>848</v>
+      </c>
+      <c r="L234" s="11"/>
+      <c r="M234" s="11"/>
       <c r="N234" s="13"/>
       <c r="O234" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="P234" s="13">
-        <v>26201200102537</v>
-      </c>
+      <c r="P234" s="13"/>
       <c r="Q234" s="14"/>
       <c r="R234" s="15"/>
-      <c r="S234" s="7" t="s">
-        <v>314</v>
-      </c>
+      <c r="S234" s="7"/>
     </row>
     <row r="235" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A235" s="7">
         <v>233</v>
       </c>
       <c r="B235" s="7">
-        <v>180</v>
+        <v>20098</v>
       </c>
       <c r="C235" s="8"/>
       <c r="D235" s="9" t="s">
-        <v>847</v>
+        <v>849</v>
       </c>
       <c r="E235" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F235" s="7" t="s">
-        <v>180</v>
+        <v>256</v>
       </c>
       <c r="G235" s="7"/>
       <c r="H235" s="10">
-        <v>44957</v>
+        <v>44235</v>
       </c>
       <c r="I235" s="11">
-        <v>44957</v>
+        <v>45420</v>
       </c>
       <c r="J235" s="12">
-        <v>45321</v>
+        <v>45511</v>
       </c>
       <c r="K235" s="7" t="s">
-        <v>848</v>
-      </c>
-      <c r="L235" s="11"/>
-      <c r="M235" s="11"/>
+        <v>850</v>
+      </c>
+      <c r="L235" s="11">
+        <v>22251</v>
+      </c>
+      <c r="M235" s="11">
+        <v>44166</v>
+      </c>
       <c r="N235" s="13"/>
       <c r="O235" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="P235" s="13"/>
+        <v>24</v>
+      </c>
+      <c r="P235" s="13">
+        <v>26012012200893</v>
+      </c>
       <c r="Q235" s="14"/>
       <c r="R235" s="15"/>
-      <c r="S235" s="7"/>
+      <c r="S235" s="7" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="236" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A236" s="7">
         <v>234</v>
       </c>
       <c r="B236" s="7">
-        <v>20098</v>
+        <v>169</v>
       </c>
       <c r="C236" s="8"/>
       <c r="D236" s="9" t="s">
-        <v>849</v>
+        <v>851</v>
       </c>
       <c r="E236" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F236" s="7" t="s">
-        <v>256</v>
+        <v>852</v>
       </c>
       <c r="G236" s="7"/>
       <c r="H236" s="10">
-        <v>44235</v>
+        <v>44927</v>
       </c>
       <c r="I236" s="11">
-        <v>45420</v>
+        <v>45474</v>
       </c>
       <c r="J236" s="12">
-        <v>45511</v>
+        <v>45565</v>
       </c>
       <c r="K236" s="7" t="s">
-        <v>850</v>
+        <v>853</v>
       </c>
       <c r="L236" s="11">
-        <v>22251</v>
+        <v>23008</v>
       </c>
       <c r="M236" s="11">
-        <v>44166</v>
+        <v>44923</v>
       </c>
       <c r="N236" s="13"/>
       <c r="O236" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P236" s="13">
-        <v>26012012200893</v>
+        <v>26212280104839</v>
       </c>
       <c r="Q236" s="14"/>
       <c r="R236" s="15"/>
       <c r="S236" s="7" t="s">
-        <v>44</v>
+        <v>854</v>
       </c>
     </row>
     <row r="237" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22859,48 +22871,46 @@
         <v>235</v>
       </c>
       <c r="B237" s="7">
-        <v>169</v>
+        <v>20122</v>
       </c>
       <c r="C237" s="8"/>
       <c r="D237" s="9" t="s">
-        <v>851</v>
+        <v>855</v>
       </c>
       <c r="E237" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F237" s="7" t="s">
-        <v>852</v>
+        <v>27</v>
       </c>
       <c r="G237" s="7"/>
       <c r="H237" s="10">
-        <v>44927</v>
+        <v>45363</v>
       </c>
       <c r="I237" s="11">
-        <v>45474</v>
-      </c>
-      <c r="J237" s="12">
-        <v>45565</v>
-      </c>
+        <v>45363</v>
+      </c>
+      <c r="J237" s="12"/>
       <c r="K237" s="7" t="s">
-        <v>853</v>
+        <v>856</v>
       </c>
       <c r="L237" s="11">
-        <v>23008</v>
+        <v>22414</v>
       </c>
       <c r="M237" s="11">
-        <v>44923</v>
+        <v>44329</v>
       </c>
       <c r="N237" s="13"/>
-      <c r="O237" s="7" t="s">
-        <v>24</v>
-      </c>
+      <c r="O237" s="7"/>
       <c r="P237" s="13">
-        <v>26212280104839</v>
-      </c>
-      <c r="Q237" s="14"/>
+        <v>26105131401234</v>
+      </c>
+      <c r="Q237" s="14">
+        <v>1062087284</v>
+      </c>
       <c r="R237" s="15"/>
       <c r="S237" s="7" t="s">
-        <v>854</v>
+        <v>29</v>
       </c>
     </row>
     <row r="238" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22908,46 +22918,48 @@
         <v>236</v>
       </c>
       <c r="B238" s="7">
-        <v>20122</v>
+        <v>20170</v>
       </c>
       <c r="C238" s="8"/>
       <c r="D238" s="9" t="s">
-        <v>855</v>
+        <v>857</v>
       </c>
       <c r="E238" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F238" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G238" s="7"/>
       <c r="H238" s="10">
-        <v>45363</v>
+        <v>44325</v>
       </c>
       <c r="I238" s="11">
-        <v>45363</v>
-      </c>
-      <c r="J238" s="12"/>
+        <v>45421</v>
+      </c>
+      <c r="J238" s="12">
+        <v>45512</v>
+      </c>
       <c r="K238" s="7" t="s">
-        <v>856</v>
+        <v>858</v>
       </c>
       <c r="L238" s="11">
-        <v>22414</v>
+        <v>22397</v>
       </c>
       <c r="M238" s="11">
-        <v>44329</v>
+        <v>44312</v>
       </c>
       <c r="N238" s="13"/>
-      <c r="O238" s="7"/>
+      <c r="O238" s="7" t="s">
+        <v>24</v>
+      </c>
       <c r="P238" s="13">
-        <v>26105131401234</v>
-      </c>
-      <c r="Q238" s="14">
-        <v>1062087284</v>
-      </c>
+        <v>26104261701055</v>
+      </c>
+      <c r="Q238" s="14"/>
       <c r="R238" s="15"/>
       <c r="S238" s="7" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
     </row>
     <row r="239" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -22955,11 +22967,13 @@
         <v>237</v>
       </c>
       <c r="B239" s="7">
-        <v>20170</v>
-      </c>
-      <c r="C239" s="8"/>
+        <v>20162</v>
+      </c>
+      <c r="C239" s="8">
+        <v>98</v>
+      </c>
       <c r="D239" s="9" t="s">
-        <v>857</v>
+        <v>859</v>
       </c>
       <c r="E239" s="7" t="s">
         <v>20</v>
@@ -22969,34 +22983,34 @@
       </c>
       <c r="G239" s="7"/>
       <c r="H239" s="10">
-        <v>44325</v>
+        <v>44368</v>
       </c>
       <c r="I239" s="11">
-        <v>45421</v>
+        <v>45372</v>
       </c>
       <c r="J239" s="12">
-        <v>45512</v>
+        <v>45463</v>
       </c>
       <c r="K239" s="7" t="s">
-        <v>858</v>
+        <v>860</v>
       </c>
       <c r="L239" s="11">
-        <v>22397</v>
+        <v>22319</v>
       </c>
       <c r="M239" s="11">
-        <v>44312</v>
+        <v>44234</v>
       </c>
       <c r="N239" s="13"/>
       <c r="O239" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P239" s="13">
-        <v>26104261701055</v>
+        <v>26102071302313</v>
       </c>
       <c r="Q239" s="14"/>
       <c r="R239" s="15"/>
       <c r="S239" s="7" t="s">
-        <v>44</v>
+        <v>854</v>
       </c>
     </row>
     <row r="240" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23004,13 +23018,13 @@
         <v>238</v>
       </c>
       <c r="B240" s="7">
-        <v>20162</v>
+        <v>20201</v>
       </c>
       <c r="C240" s="8">
-        <v>98</v>
+        <v>141</v>
       </c>
       <c r="D240" s="9" t="s">
-        <v>859</v>
+        <v>861</v>
       </c>
       <c r="E240" s="7" t="s">
         <v>20</v>
@@ -23020,34 +23034,36 @@
       </c>
       <c r="G240" s="7"/>
       <c r="H240" s="10">
-        <v>44368</v>
+        <v>44691</v>
       </c>
       <c r="I240" s="11">
-        <v>45372</v>
+        <v>45698</v>
       </c>
       <c r="J240" s="12">
-        <v>45463</v>
+        <v>45786</v>
       </c>
       <c r="K240" s="7" t="s">
-        <v>860</v>
+        <v>862</v>
       </c>
       <c r="L240" s="11">
-        <v>22319</v>
+        <v>22744</v>
       </c>
       <c r="M240" s="11">
-        <v>44234</v>
+        <v>44659</v>
       </c>
       <c r="N240" s="13"/>
       <c r="O240" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P240" s="13">
-        <v>26102071302313</v>
-      </c>
-      <c r="Q240" s="14"/>
+        <v>26204081400736</v>
+      </c>
+      <c r="Q240" s="14">
+        <v>1280523610</v>
+      </c>
       <c r="R240" s="15"/>
       <c r="S240" s="7" t="s">
-        <v>854</v>
+        <v>863</v>
       </c>
     </row>
     <row r="241" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23055,52 +23071,50 @@
         <v>239</v>
       </c>
       <c r="B241" s="7">
-        <v>20201</v>
+        <v>20244</v>
       </c>
       <c r="C241" s="8">
-        <v>141</v>
+        <v>182</v>
       </c>
       <c r="D241" s="9" t="s">
-        <v>861</v>
+        <v>864</v>
       </c>
       <c r="E241" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F241" s="7" t="s">
-        <v>21</v>
+        <v>865</v>
       </c>
       <c r="G241" s="7"/>
       <c r="H241" s="10">
-        <v>44691</v>
+        <v>45047</v>
       </c>
       <c r="I241" s="11">
-        <v>45698</v>
+        <v>45413</v>
       </c>
       <c r="J241" s="12">
-        <v>45786</v>
+        <v>45777</v>
       </c>
       <c r="K241" s="7" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
       <c r="L241" s="11">
-        <v>22744</v>
+        <v>23102</v>
       </c>
       <c r="M241" s="11">
-        <v>44659</v>
+        <v>45017</v>
       </c>
       <c r="N241" s="13"/>
       <c r="O241" s="7" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="P241" s="13">
-        <v>26204081400736</v>
-      </c>
-      <c r="Q241" s="14">
-        <v>1280523610</v>
-      </c>
+        <v>26304011400776</v>
+      </c>
+      <c r="Q241" s="14"/>
       <c r="R241" s="15"/>
       <c r="S241" s="7" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
     </row>
     <row r="242" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23108,50 +23122,50 @@
         <v>240</v>
       </c>
       <c r="B242" s="7">
-        <v>20244</v>
+        <v>20157</v>
       </c>
       <c r="C242" s="8">
-        <v>182</v>
+        <v>93</v>
       </c>
       <c r="D242" s="9" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="E242" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F242" s="7" t="s">
-        <v>865</v>
+        <v>21</v>
       </c>
       <c r="G242" s="7"/>
       <c r="H242" s="10">
-        <v>45047</v>
+        <v>43832</v>
       </c>
       <c r="I242" s="11">
-        <v>45413</v>
+        <v>45384</v>
       </c>
       <c r="J242" s="12">
-        <v>45777</v>
-      </c>
-      <c r="K242" s="7" t="s">
-        <v>866</v>
-      </c>
+        <v>45809</v>
+      </c>
+      <c r="K242" s="7"/>
       <c r="L242" s="11">
-        <v>23102</v>
+        <v>21451</v>
       </c>
       <c r="M242" s="11">
-        <v>45017</v>
+        <v>43366</v>
       </c>
       <c r="N242" s="13"/>
       <c r="O242" s="7" t="s">
-        <v>56</v>
+        <v>869</v>
       </c>
       <c r="P242" s="13">
-        <v>26304011400776</v>
-      </c>
-      <c r="Q242" s="14"/>
+        <v>25809230101238</v>
+      </c>
+      <c r="Q242" s="14">
+        <v>1148141435</v>
+      </c>
       <c r="R242" s="15"/>
       <c r="S242" s="7" t="s">
-        <v>867</v>
+        <v>44</v>
       </c>
     </row>
     <row r="243" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23159,50 +23173,50 @@
         <v>241</v>
       </c>
       <c r="B243" s="7">
-        <v>20157</v>
+        <v>20265</v>
       </c>
       <c r="C243" s="8">
-        <v>93</v>
+        <v>208</v>
       </c>
       <c r="D243" s="9" t="s">
-        <v>868</v>
+        <v>870</v>
       </c>
       <c r="E243" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F243" s="7" t="s">
-        <v>21</v>
+        <v>871</v>
       </c>
       <c r="G243" s="7"/>
       <c r="H243" s="10">
-        <v>43832</v>
+        <v>45374</v>
       </c>
       <c r="I243" s="11">
-        <v>45384</v>
+        <v>45739</v>
       </c>
       <c r="J243" s="12">
-        <v>45809</v>
+        <v>45830</v>
       </c>
       <c r="K243" s="7"/>
       <c r="L243" s="11">
-        <v>21451</v>
+        <v>23408</v>
       </c>
       <c r="M243" s="11">
-        <v>43366</v>
+        <v>45323</v>
       </c>
       <c r="N243" s="13"/>
       <c r="O243" s="7" t="s">
-        <v>869</v>
+        <v>24</v>
       </c>
       <c r="P243" s="13">
-        <v>25809230101238</v>
+        <v>26402011701018</v>
       </c>
       <c r="Q243" s="14">
-        <v>1148141435</v>
+        <v>1202825386</v>
       </c>
       <c r="R243" s="15"/>
       <c r="S243" s="7" t="s">
-        <v>44</v>
+        <v>358</v>
       </c>
     </row>
     <row r="244" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23210,50 +23224,52 @@
         <v>242</v>
       </c>
       <c r="B244" s="7">
-        <v>20265</v>
+        <v>20034</v>
       </c>
       <c r="C244" s="8">
-        <v>208</v>
+        <v>38</v>
       </c>
       <c r="D244" s="9" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
       <c r="E244" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F244" s="7" t="s">
-        <v>871</v>
+        <v>27</v>
       </c>
       <c r="G244" s="7"/>
       <c r="H244" s="10">
-        <v>45374</v>
+        <v>43312</v>
       </c>
       <c r="I244" s="11">
-        <v>45739</v>
+        <v>45778</v>
       </c>
       <c r="J244" s="12">
-        <v>45830</v>
-      </c>
-      <c r="K244" s="7"/>
+        <v>45868</v>
+      </c>
+      <c r="K244" s="7" t="s">
+        <v>873</v>
+      </c>
       <c r="L244" s="11">
-        <v>23408</v>
+        <v>20084</v>
       </c>
       <c r="M244" s="11">
-        <v>45323</v>
+        <v>41999</v>
       </c>
       <c r="N244" s="13"/>
       <c r="O244" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P244" s="13">
-        <v>26402011701018</v>
+        <v>25412261300231</v>
       </c>
       <c r="Q244" s="14">
-        <v>1202825386</v>
+        <v>1220128618</v>
       </c>
       <c r="R244" s="15"/>
       <c r="S244" s="7" t="s">
-        <v>358</v>
+        <v>29</v>
       </c>
     </row>
     <row r="245" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23261,52 +23277,50 @@
         <v>243</v>
       </c>
       <c r="B245" s="7">
-        <v>20034</v>
+        <v>20179</v>
       </c>
       <c r="C245" s="8">
-        <v>38</v>
+        <v>115</v>
       </c>
       <c r="D245" s="9" t="s">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="E245" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F245" s="7" t="s">
-        <v>27</v>
+        <v>875</v>
       </c>
       <c r="G245" s="7"/>
       <c r="H245" s="10">
-        <v>43312</v>
+        <v>44333</v>
       </c>
       <c r="I245" s="11">
-        <v>45778</v>
+        <v>45613</v>
       </c>
       <c r="J245" s="12">
-        <v>45868</v>
+        <v>45977</v>
       </c>
       <c r="K245" s="7" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
       <c r="L245" s="11">
-        <v>20084</v>
+        <v>22364</v>
       </c>
       <c r="M245" s="11">
-        <v>41999</v>
+        <v>44279</v>
       </c>
       <c r="N245" s="13"/>
       <c r="O245" s="7" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="P245" s="13">
-        <v>25412261300231</v>
-      </c>
-      <c r="Q245" s="14">
-        <v>1220128618</v>
-      </c>
+        <v>26103240100659</v>
+      </c>
+      <c r="Q245" s="14"/>
       <c r="R245" s="15"/>
       <c r="S245" s="7" t="s">
-        <v>29</v>
+        <v>877</v>
       </c>
     </row>
     <row r="246" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23314,50 +23328,52 @@
         <v>244</v>
       </c>
       <c r="B246" s="7">
-        <v>20179</v>
+        <v>20109</v>
       </c>
       <c r="C246" s="8">
-        <v>115</v>
+        <v>25</v>
       </c>
       <c r="D246" s="9" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="E246" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F246" s="7" t="s">
-        <v>875</v>
+        <v>372</v>
       </c>
       <c r="G246" s="7"/>
       <c r="H246" s="10">
-        <v>44333</v>
+        <v>44454</v>
       </c>
       <c r="I246" s="11">
-        <v>45613</v>
+        <v>45731</v>
       </c>
       <c r="J246" s="12">
-        <v>45977</v>
+        <v>45822</v>
       </c>
       <c r="K246" s="7" t="s">
-        <v>876</v>
+        <v>879</v>
       </c>
       <c r="L246" s="11">
-        <v>22364</v>
+        <v>22503</v>
       </c>
       <c r="M246" s="11">
-        <v>44279</v>
+        <v>44418</v>
       </c>
       <c r="N246" s="13"/>
       <c r="O246" s="7" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="P246" s="13">
-        <v>26103240100659</v>
-      </c>
-      <c r="Q246" s="14"/>
+        <v>26108102200792</v>
+      </c>
+      <c r="Q246" s="14">
+        <v>1142996504</v>
+      </c>
       <c r="R246" s="15"/>
       <c r="S246" s="7" t="s">
-        <v>877</v>
+        <v>373</v>
       </c>
     </row>
     <row r="247" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23365,52 +23381,52 @@
         <v>245</v>
       </c>
       <c r="B247" s="7">
-        <v>20109</v>
+        <v>20113</v>
       </c>
       <c r="C247" s="8">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D247" s="9" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="E247" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F247" s="7" t="s">
-        <v>372</v>
+        <v>27</v>
       </c>
       <c r="G247" s="7"/>
       <c r="H247" s="10">
-        <v>44454</v>
+        <v>44376</v>
       </c>
       <c r="I247" s="11">
-        <v>45731</v>
+        <v>45745</v>
       </c>
       <c r="J247" s="12">
-        <v>45822</v>
+        <v>45836</v>
       </c>
       <c r="K247" s="7" t="s">
-        <v>879</v>
+        <v>881</v>
       </c>
       <c r="L247" s="11">
-        <v>22503</v>
+        <v>22394</v>
       </c>
       <c r="M247" s="11">
-        <v>44418</v>
+        <v>44309</v>
       </c>
       <c r="N247" s="13"/>
       <c r="O247" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P247" s="13">
-        <v>26108102200792</v>
+        <v>26104231600971</v>
       </c>
       <c r="Q247" s="14">
-        <v>1142996504</v>
+        <v>1270907591</v>
       </c>
       <c r="R247" s="15"/>
       <c r="S247" s="7" t="s">
-        <v>373</v>
+        <v>29</v>
       </c>
     </row>
     <row r="248" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23418,13 +23434,13 @@
         <v>246</v>
       </c>
       <c r="B248" s="7">
-        <v>20113</v>
+        <v>20124</v>
       </c>
       <c r="C248" s="8">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="D248" s="9" t="s">
-        <v>880</v>
+        <v>882</v>
       </c>
       <c r="E248" s="7" t="s">
         <v>20</v>
@@ -23434,33 +23450,31 @@
       </c>
       <c r="G248" s="7"/>
       <c r="H248" s="10">
-        <v>44376</v>
+        <v>44335</v>
       </c>
       <c r="I248" s="11">
-        <v>45745</v>
+        <v>45796</v>
       </c>
       <c r="J248" s="12">
-        <v>45836</v>
+        <v>45887</v>
       </c>
       <c r="K248" s="7" t="s">
-        <v>881</v>
+        <v>883</v>
       </c>
       <c r="L248" s="11">
-        <v>22394</v>
+        <v>22145</v>
       </c>
       <c r="M248" s="11">
-        <v>44309</v>
+        <v>44060</v>
       </c>
       <c r="N248" s="13"/>
       <c r="O248" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P248" s="13">
-        <v>26104231600971</v>
-      </c>
-      <c r="Q248" s="14">
-        <v>1270907591</v>
-      </c>
+        <v>26008170101595</v>
+      </c>
+      <c r="Q248" s="14"/>
       <c r="R248" s="15"/>
       <c r="S248" s="7" t="s">
         <v>29</v>
@@ -23471,50 +23485,44 @@
         <v>247</v>
       </c>
       <c r="B249" s="7">
-        <v>20124</v>
+        <v>20343</v>
       </c>
       <c r="C249" s="8">
-        <v>48</v>
+        <v>278</v>
       </c>
       <c r="D249" s="9" t="s">
-        <v>882</v>
+        <v>884</v>
       </c>
       <c r="E249" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F249" s="7" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="G249" s="7"/>
       <c r="H249" s="10">
-        <v>44335</v>
+        <v>45875</v>
       </c>
       <c r="I249" s="11">
-        <v>45796</v>
+        <v>45875</v>
       </c>
       <c r="J249" s="12">
-        <v>45887</v>
+        <v>45966</v>
       </c>
       <c r="K249" s="7" t="s">
-        <v>883</v>
-      </c>
-      <c r="L249" s="11">
-        <v>22145</v>
-      </c>
-      <c r="M249" s="11">
-        <v>44060</v>
-      </c>
+        <v>885</v>
+      </c>
+      <c r="L249" s="11"/>
+      <c r="M249" s="11"/>
       <c r="N249" s="13"/>
       <c r="O249" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="P249" s="13">
-        <v>26008170101595</v>
-      </c>
+      <c r="P249" s="13"/>
       <c r="Q249" s="14"/>
       <c r="R249" s="15"/>
       <c r="S249" s="7" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
     </row>
     <row r="250" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23522,44 +23530,52 @@
         <v>248</v>
       </c>
       <c r="B250" s="7">
-        <v>20343</v>
+        <v>20284</v>
       </c>
       <c r="C250" s="8">
-        <v>278</v>
+        <v>218</v>
       </c>
       <c r="D250" s="9" t="s">
-        <v>884</v>
+        <v>886</v>
       </c>
       <c r="E250" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F250" s="7" t="s">
-        <v>38</v>
+        <v>256</v>
       </c>
       <c r="G250" s="7"/>
       <c r="H250" s="10">
-        <v>45875</v>
+        <v>45752</v>
       </c>
       <c r="I250" s="11">
-        <v>45875</v>
+        <v>45752</v>
       </c>
       <c r="J250" s="12">
-        <v>45966</v>
+        <v>45842</v>
       </c>
       <c r="K250" s="7" t="s">
-        <v>885</v>
-      </c>
-      <c r="L250" s="11"/>
-      <c r="M250" s="11"/>
+        <v>887</v>
+      </c>
+      <c r="L250" s="11">
+        <v>23090</v>
+      </c>
+      <c r="M250" s="11">
+        <v>45005</v>
+      </c>
       <c r="N250" s="13"/>
       <c r="O250" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="P250" s="13"/>
-      <c r="Q250" s="14"/>
+      <c r="P250" s="13">
+        <v>26303201701016</v>
+      </c>
+      <c r="Q250" s="14">
+        <v>1002976808</v>
+      </c>
       <c r="R250" s="15"/>
       <c r="S250" s="7" t="s">
-        <v>39</v>
+        <v>385</v>
       </c>
     </row>
     <row r="251" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23567,48 +23583,48 @@
         <v>249</v>
       </c>
       <c r="B251" s="7">
-        <v>20284</v>
+        <v>20292</v>
       </c>
       <c r="C251" s="8">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="D251" s="9" t="s">
-        <v>886</v>
+        <v>888</v>
       </c>
       <c r="E251" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F251" s="7" t="s">
-        <v>256</v>
+        <v>68</v>
       </c>
       <c r="G251" s="7"/>
       <c r="H251" s="10">
-        <v>45752</v>
+        <v>45716</v>
       </c>
       <c r="I251" s="11">
-        <v>45752</v>
+        <v>45715</v>
       </c>
       <c r="J251" s="12">
-        <v>45842</v>
+        <v>45803</v>
       </c>
       <c r="K251" s="7" t="s">
-        <v>887</v>
+        <v>889</v>
       </c>
       <c r="L251" s="11">
-        <v>23090</v>
+        <v>23709</v>
       </c>
       <c r="M251" s="11">
-        <v>45005</v>
+        <v>45624</v>
       </c>
       <c r="N251" s="13"/>
       <c r="O251" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P251" s="13">
-        <v>26303201701016</v>
+        <v>26411281701094</v>
       </c>
       <c r="Q251" s="14">
-        <v>1002976808</v>
+        <v>1062830905</v>
       </c>
       <c r="R251" s="15"/>
       <c r="S251" s="7" t="s">
@@ -23620,52 +23636,52 @@
         <v>250</v>
       </c>
       <c r="B252" s="7">
-        <v>20292</v>
+        <v>20269</v>
       </c>
       <c r="C252" s="8">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="D252" s="9" t="s">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="E252" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F252" s="7" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="G252" s="7"/>
       <c r="H252" s="10">
-        <v>45716</v>
+        <v>45383</v>
       </c>
       <c r="I252" s="11">
-        <v>45715</v>
+        <v>45748</v>
       </c>
       <c r="J252" s="12">
-        <v>45803</v>
+        <v>45838</v>
       </c>
       <c r="K252" s="7" t="s">
-        <v>889</v>
+        <v>891</v>
       </c>
       <c r="L252" s="11">
-        <v>23709</v>
+        <v>23021</v>
       </c>
       <c r="M252" s="11">
-        <v>45624</v>
+        <v>44936</v>
       </c>
       <c r="N252" s="13"/>
       <c r="O252" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P252" s="13">
-        <v>26411281701094</v>
+        <v>26301100104472</v>
       </c>
       <c r="Q252" s="14">
-        <v>1062830905</v>
+        <v>1270115952</v>
       </c>
       <c r="R252" s="15"/>
       <c r="S252" s="7" t="s">
-        <v>385</v>
+        <v>29</v>
       </c>
     </row>
     <row r="253" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23673,13 +23689,13 @@
         <v>251</v>
       </c>
       <c r="B253" s="7">
-        <v>20269</v>
+        <v>20238</v>
       </c>
       <c r="C253" s="8">
-        <v>205</v>
+        <v>178</v>
       </c>
       <c r="D253" s="9" t="s">
-        <v>890</v>
+        <v>892</v>
       </c>
       <c r="E253" s="7" t="s">
         <v>20</v>
@@ -23689,33 +23705,31 @@
       </c>
       <c r="G253" s="7"/>
       <c r="H253" s="10">
-        <v>45383</v>
+        <v>44961</v>
       </c>
       <c r="I253" s="11">
-        <v>45748</v>
+        <v>45781</v>
       </c>
       <c r="J253" s="12">
-        <v>45838</v>
+        <v>45872</v>
       </c>
       <c r="K253" s="7" t="s">
-        <v>891</v>
+        <v>893</v>
       </c>
       <c r="L253" s="11">
-        <v>23021</v>
+        <v>22857</v>
       </c>
       <c r="M253" s="11">
-        <v>44936</v>
+        <v>44772</v>
       </c>
       <c r="N253" s="13"/>
       <c r="O253" s="7" t="s">
         <v>24</v>
       </c>
       <c r="P253" s="13">
-        <v>26301100104472</v>
-      </c>
-      <c r="Q253" s="14">
-        <v>1270115952</v>
-      </c>
+        <v>26207302100359</v>
+      </c>
+      <c r="Q253" s="14"/>
       <c r="R253" s="15"/>
       <c r="S253" s="7" t="s">
         <v>29</v>
@@ -23726,50 +23740,52 @@
         <v>252</v>
       </c>
       <c r="B254" s="7">
-        <v>20238</v>
+        <v>20221</v>
       </c>
       <c r="C254" s="8">
-        <v>178</v>
+        <v>161</v>
       </c>
       <c r="D254" s="9" t="s">
-        <v>892</v>
+        <v>894</v>
       </c>
       <c r="E254" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F254" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G254" s="7"/>
       <c r="H254" s="10">
-        <v>44961</v>
+        <v>44878</v>
       </c>
       <c r="I254" s="11">
-        <v>45781</v>
+        <v>45882</v>
       </c>
       <c r="J254" s="12">
-        <v>45872</v>
+        <v>45942</v>
       </c>
       <c r="K254" s="7" t="s">
-        <v>893</v>
+        <v>895</v>
       </c>
       <c r="L254" s="11">
-        <v>22857</v>
+        <v>22943</v>
       </c>
       <c r="M254" s="11">
-        <v>44772</v>
+        <v>44858</v>
       </c>
       <c r="N254" s="13"/>
       <c r="O254" s="7" t="s">
-        <v>24</v>
+        <v>767</v>
       </c>
       <c r="P254" s="13">
-        <v>26207302100359</v>
-      </c>
-      <c r="Q254" s="14"/>
+        <v>26210241400258</v>
+      </c>
+      <c r="Q254" s="14">
+        <v>1004279367</v>
+      </c>
       <c r="R254" s="15"/>
       <c r="S254" s="7" t="s">
-        <v>29</v>
+        <v>219</v>
       </c>
     </row>
     <row r="255" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23777,52 +23793,52 @@
         <v>253</v>
       </c>
       <c r="B255" s="7">
-        <v>20221</v>
+        <v>20285</v>
       </c>
       <c r="C255" s="8">
-        <v>161</v>
+        <v>219</v>
       </c>
       <c r="D255" s="9" t="s">
-        <v>894</v>
+        <v>896</v>
       </c>
       <c r="E255" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F255" s="7" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="G255" s="7"/>
       <c r="H255" s="10">
-        <v>44878</v>
+        <v>45715</v>
       </c>
       <c r="I255" s="11">
-        <v>45882</v>
+        <v>45715</v>
       </c>
       <c r="J255" s="12">
-        <v>45942</v>
+        <v>45803</v>
       </c>
       <c r="K255" s="7" t="s">
-        <v>895</v>
+        <v>897</v>
       </c>
       <c r="L255" s="11">
-        <v>22943</v>
+        <v>23740</v>
       </c>
       <c r="M255" s="11">
-        <v>44858</v>
+        <v>45655</v>
       </c>
       <c r="N255" s="13"/>
       <c r="O255" s="7" t="s">
-        <v>767</v>
+        <v>24</v>
       </c>
       <c r="P255" s="13">
-        <v>26210241400258</v>
+        <v>26412291402717</v>
       </c>
       <c r="Q255" s="14">
-        <v>1004279367</v>
+        <v>1004348133</v>
       </c>
       <c r="R255" s="15"/>
       <c r="S255" s="7" t="s">
-        <v>219</v>
+        <v>385</v>
       </c>
     </row>
     <row r="256" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23830,52 +23846,52 @@
         <v>254</v>
       </c>
       <c r="B256" s="7">
-        <v>20285</v>
+        <v>20126</v>
       </c>
       <c r="C256" s="8">
-        <v>219</v>
+        <v>50</v>
       </c>
       <c r="D256" s="9" t="s">
-        <v>896</v>
+        <v>898</v>
       </c>
       <c r="E256" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F256" s="7" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="G256" s="7"/>
       <c r="H256" s="10">
-        <v>45715</v>
+        <v>44555</v>
       </c>
       <c r="I256" s="11">
-        <v>45715</v>
+        <v>45741</v>
       </c>
       <c r="J256" s="12">
-        <v>45803</v>
+        <v>46015</v>
       </c>
       <c r="K256" s="7" t="s">
-        <v>897</v>
+        <v>899</v>
       </c>
       <c r="L256" s="11">
-        <v>23740</v>
+        <v>22465</v>
       </c>
       <c r="M256" s="11">
-        <v>45655</v>
+        <v>44380</v>
       </c>
       <c r="N256" s="13"/>
       <c r="O256" s="7" t="s">
-        <v>24</v>
+        <v>900</v>
       </c>
       <c r="P256" s="13">
-        <v>26412291402717</v>
+        <v>26107031300271</v>
       </c>
       <c r="Q256" s="14">
-        <v>1004348133</v>
+        <v>1063238105</v>
       </c>
       <c r="R256" s="15"/>
       <c r="S256" s="7" t="s">
-        <v>385</v>
+        <v>32</v>
       </c>
     </row>
     <row r="257" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23883,52 +23899,44 @@
         <v>255</v>
       </c>
       <c r="B257" s="7">
-        <v>20126</v>
+        <v>20377</v>
       </c>
       <c r="C257" s="8">
-        <v>50</v>
+        <v>312</v>
       </c>
       <c r="D257" s="9" t="s">
-        <v>898</v>
+        <v>901</v>
       </c>
       <c r="E257" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F257" s="7" t="s">
-        <v>27</v>
+        <v>109</v>
       </c>
       <c r="G257" s="7"/>
       <c r="H257" s="10">
-        <v>44555</v>
+        <v>45963</v>
       </c>
       <c r="I257" s="11">
-        <v>45741</v>
+        <v>45963</v>
       </c>
       <c r="J257" s="12">
-        <v>46015</v>
+        <v>46054</v>
       </c>
       <c r="K257" s="7" t="s">
-        <v>899</v>
-      </c>
-      <c r="L257" s="11">
-        <v>22465</v>
-      </c>
-      <c r="M257" s="11">
-        <v>44380</v>
-      </c>
+        <v>902</v>
+      </c>
+      <c r="L257" s="11"/>
+      <c r="M257" s="11"/>
       <c r="N257" s="13"/>
       <c r="O257" s="7" t="s">
-        <v>900</v>
-      </c>
-      <c r="P257" s="13">
-        <v>26107031300271</v>
-      </c>
-      <c r="Q257" s="14">
-        <v>1063238105</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="P257" s="13"/>
+      <c r="Q257" s="14"/>
       <c r="R257" s="15"/>
       <c r="S257" s="7" t="s">
-        <v>32</v>
+        <v>643</v>
       </c>
     </row>
     <row r="258" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23936,32 +23944,32 @@
         <v>256</v>
       </c>
       <c r="B258" s="7">
-        <v>20377</v>
-      </c>
-      <c r="C258" s="8">
-        <v>312</v>
+        <v>306</v>
+      </c>
+      <c r="C258" s="8" t="s">
+        <v>903</v>
       </c>
       <c r="D258" s="9" t="s">
-        <v>901</v>
+        <v>20</v>
       </c>
       <c r="E258" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F258" s="7" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="G258" s="7"/>
       <c r="H258" s="10">
-        <v>45963</v>
+        <v>45952</v>
       </c>
       <c r="I258" s="11">
-        <v>45963</v>
+        <v>45952</v>
       </c>
       <c r="J258" s="12">
-        <v>46054</v>
+        <v>46043</v>
       </c>
       <c r="K258" s="7" t="s">
-        <v>902</v>
+        <v>904</v>
       </c>
       <c r="L258" s="11"/>
       <c r="M258" s="11"/>
@@ -23973,7 +23981,7 @@
       <c r="Q258" s="14"/>
       <c r="R258" s="15"/>
       <c r="S258" s="7" t="s">
-        <v>643</v>
+        <v>153</v>
       </c>
     </row>
     <row r="259" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -23981,44 +23989,42 @@
         <v>257</v>
       </c>
       <c r="B259" s="7">
-        <v>306</v>
-      </c>
-      <c r="C259" s="8" t="s">
-        <v>903</v>
+        <v>20368</v>
+      </c>
+      <c r="C259" s="8">
+        <v>303</v>
       </c>
       <c r="D259" s="9" t="s">
-        <v>20</v>
+        <v>662</v>
       </c>
       <c r="E259" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F259" s="7" t="s">
-        <v>136</v>
+        <v>109</v>
       </c>
       <c r="G259" s="7"/>
       <c r="H259" s="10">
-        <v>45952</v>
+        <v>45931</v>
       </c>
       <c r="I259" s="11">
-        <v>45952</v>
+        <v>45931</v>
       </c>
       <c r="J259" s="12">
-        <v>46043</v>
+        <v>45931</v>
       </c>
       <c r="K259" s="7" t="s">
-        <v>904</v>
+        <v>106</v>
       </c>
       <c r="L259" s="11"/>
       <c r="M259" s="11"/>
       <c r="N259" s="13"/>
-      <c r="O259" s="7" t="s">
-        <v>24</v>
-      </c>
+      <c r="O259" s="7"/>
       <c r="P259" s="13"/>
       <c r="Q259" s="14"/>
       <c r="R259" s="15"/>
       <c r="S259" s="7" t="s">
-        <v>153</v>
+        <v>905</v>
       </c>
     </row>
     <row r="260" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -24026,32 +24032,26 @@
         <v>258</v>
       </c>
       <c r="B260" s="7">
-        <v>20368</v>
+        <v>20416</v>
       </c>
       <c r="C260" s="8">
-        <v>303</v>
+        <v>351</v>
       </c>
       <c r="D260" s="9" t="s">
-        <v>662</v>
+        <v>906</v>
       </c>
       <c r="E260" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F260" s="7" t="s">
-        <v>109</v>
+        <v>27</v>
       </c>
       <c r="G260" s="7"/>
-      <c r="H260" s="10">
-        <v>45931</v>
-      </c>
-      <c r="I260" s="11">
-        <v>45931</v>
-      </c>
-      <c r="J260" s="12">
-        <v>45931</v>
-      </c>
+      <c r="H260" s="10"/>
+      <c r="I260" s="11"/>
+      <c r="J260" s="12"/>
       <c r="K260" s="7" t="s">
-        <v>106</v>
+        <v>907</v>
       </c>
       <c r="L260" s="11"/>
       <c r="M260" s="11"/>
@@ -24060,35 +24060,39 @@
       <c r="P260" s="13"/>
       <c r="Q260" s="14"/>
       <c r="R260" s="15"/>
-      <c r="S260" s="7" t="s">
-        <v>905</v>
-      </c>
+      <c r="S260" s="7"/>
     </row>
     <row r="261" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A261" s="7">
         <v>259</v>
       </c>
       <c r="B261" s="7">
-        <v>20416</v>
+        <v>20411</v>
       </c>
       <c r="C261" s="8">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D261" s="9" t="s">
-        <v>906</v>
+        <v>694</v>
       </c>
       <c r="E261" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F261" s="7" t="s">
-        <v>27</v>
+        <v>68</v>
       </c>
       <c r="G261" s="7"/>
-      <c r="H261" s="10"/>
-      <c r="I261" s="11"/>
-      <c r="J261" s="12"/>
+      <c r="H261" s="10">
+        <v>46069</v>
+      </c>
+      <c r="I261" s="11">
+        <v>46069</v>
+      </c>
+      <c r="J261" s="12">
+        <v>46069</v>
+      </c>
       <c r="K261" s="7" t="s">
-        <v>907</v>
+        <v>695</v>
       </c>
       <c r="L261" s="11"/>
       <c r="M261" s="11"/>
@@ -24097,20 +24101,22 @@
       <c r="P261" s="13"/>
       <c r="Q261" s="14"/>
       <c r="R261" s="15"/>
-      <c r="S261" s="7"/>
+      <c r="S261" s="7" t="s">
+        <v>908</v>
+      </c>
     </row>
     <row r="262" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A262" s="7">
         <v>260</v>
       </c>
       <c r="B262" s="7">
-        <v>20411</v>
+        <v>20398</v>
       </c>
       <c r="C262" s="8">
-        <v>346</v>
+        <v>333</v>
       </c>
       <c r="D262" s="9" t="s">
-        <v>694</v>
+        <v>669</v>
       </c>
       <c r="E262" s="7" t="s">
         <v>20</v>
@@ -24120,16 +24126,16 @@
       </c>
       <c r="G262" s="7"/>
       <c r="H262" s="10">
-        <v>46069</v>
+        <v>46041</v>
       </c>
       <c r="I262" s="11">
-        <v>46069</v>
+        <v>46041</v>
       </c>
       <c r="J262" s="12">
-        <v>46069</v>
+        <v>46041</v>
       </c>
       <c r="K262" s="7" t="s">
-        <v>695</v>
+        <v>153</v>
       </c>
       <c r="L262" s="11"/>
       <c r="M262" s="11"/>
@@ -24139,7 +24145,7 @@
       <c r="Q262" s="14"/>
       <c r="R262" s="15"/>
       <c r="S262" s="7" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
     </row>
     <row r="263" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -24147,32 +24153,30 @@
         <v>261</v>
       </c>
       <c r="B263" s="7">
-        <v>20398</v>
-      </c>
-      <c r="C263" s="8">
-        <v>333</v>
-      </c>
+        <v>342</v>
+      </c>
+      <c r="C263" s="8"/>
       <c r="D263" s="9" t="s">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="E263" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F263" s="7" t="s">
-        <v>68</v>
+        <v>109</v>
       </c>
       <c r="G263" s="7"/>
       <c r="H263" s="10">
-        <v>46041</v>
+        <v>46057</v>
       </c>
       <c r="I263" s="11">
-        <v>46041</v>
+        <v>46057</v>
       </c>
       <c r="J263" s="12">
-        <v>46041</v>
+        <v>46057</v>
       </c>
       <c r="K263" s="7" t="s">
-        <v>153</v>
+        <v>409</v>
       </c>
       <c r="L263" s="11"/>
       <c r="M263" s="11"/>
@@ -24182,52 +24186,11 @@
       <c r="Q263" s="14"/>
       <c r="R263" s="15"/>
       <c r="S263" s="7" t="s">
-        <v>909</v>
-      </c>
-    </row>
-    <row r="264" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A264" s="7">
-        <v>262</v>
-      </c>
-      <c r="B264" s="7">
-        <v>342</v>
-      </c>
-      <c r="C264" s="8"/>
-      <c r="D264" s="9" t="s">
-        <v>677</v>
-      </c>
-      <c r="E264" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F264" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="G264" s="7"/>
-      <c r="H264" s="10">
-        <v>46057</v>
-      </c>
-      <c r="I264" s="11">
-        <v>46057</v>
-      </c>
-      <c r="J264" s="12">
-        <v>46057</v>
-      </c>
-      <c r="K264" s="7" t="s">
-        <v>409</v>
-      </c>
-      <c r="L264" s="11"/>
-      <c r="M264" s="11"/>
-      <c r="N264" s="13"/>
-      <c r="O264" s="7"/>
-      <c r="P264" s="13"/>
-      <c r="Q264" s="14"/>
-      <c r="R264" s="15"/>
-      <c r="S264" s="7" t="s">
         <v>910</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:S264"/>
+  <autoFilter ref="A2:S263"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
auto update (34 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3661,10 +3661,10 @@
         <v>29</v>
       </c>
       <c r="L8" s="11">
-        <v>21844</v>
+        <v>21845</v>
       </c>
       <c r="M8" s="11">
-        <v>43759</v>
+        <v>43760</v>
       </c>
       <c r="N8" s="13">
         <v>3500</v>
@@ -3889,7 +3889,7 @@
         <v>29</v>
       </c>
       <c r="L12" s="11">
-        <v>22291</v>
+        <v>22290</v>
       </c>
       <c r="M12" s="11">
         <v>44205</v>
@@ -4003,10 +4003,10 @@
         <v>64</v>
       </c>
       <c r="L14" s="11">
-        <v>22796</v>
+        <v>22797</v>
       </c>
       <c r="M14" s="11">
-        <v>44711</v>
+        <v>44712</v>
       </c>
       <c r="N14" s="13">
         <v>3000</v>
@@ -6505,10 +6505,10 @@
         <v>190</v>
       </c>
       <c r="L58" s="11">
-        <v>22638</v>
+        <v>22637</v>
       </c>
       <c r="M58" s="11">
-        <v>44553</v>
+        <v>44552</v>
       </c>
       <c r="N58" s="13">
         <v>3000</v>
@@ -6733,10 +6733,10 @@
         <v>201</v>
       </c>
       <c r="L62" s="11">
-        <v>24308</v>
+        <v>24026</v>
       </c>
       <c r="M62" s="11">
-        <v>46223</v>
+        <v>45941</v>
       </c>
       <c r="N62" s="13">
         <v>3000</v>
@@ -7244,10 +7244,10 @@
         <v>224</v>
       </c>
       <c r="L71" s="11">
-        <v>22933</v>
+        <v>22934</v>
       </c>
       <c r="M71" s="11">
-        <v>44848</v>
+        <v>44849</v>
       </c>
       <c r="N71" s="13">
         <v>2500</v>
@@ -8665,10 +8665,10 @@
         <v>106</v>
       </c>
       <c r="L96" s="11">
-        <v>24261</v>
+        <v>24062</v>
       </c>
       <c r="M96" s="11">
-        <v>46176</v>
+        <v>45977</v>
       </c>
       <c r="N96" s="13">
         <v>3000</v>
@@ -8893,7 +8893,7 @@
         <v>310</v>
       </c>
       <c r="L100" s="11">
-        <v>22859</v>
+        <v>19207</v>
       </c>
       <c r="M100" s="11">
         <v>41122</v>
@@ -9886,10 +9886,10 @@
         <v>237</v>
       </c>
       <c r="L119" s="11">
-        <v>24316</v>
+        <v>24366</v>
       </c>
       <c r="M119" s="11">
-        <v>46231</v>
+        <v>46281</v>
       </c>
       <c r="N119" s="13"/>
       <c r="O119" s="7" t="s">
@@ -10696,10 +10696,10 @@
         <v>373</v>
       </c>
       <c r="L10" s="11">
-        <v>20371</v>
+        <v>20381</v>
       </c>
       <c r="M10" s="11">
-        <v>42286</v>
+        <v>42296</v>
       </c>
       <c r="N10" s="13">
         <v>2500</v>
@@ -11858,10 +11858,10 @@
         <v>385</v>
       </c>
       <c r="L30" s="11">
-        <v>23472</v>
+        <v>23563</v>
       </c>
       <c r="M30" s="11">
-        <v>45387</v>
+        <v>45478</v>
       </c>
       <c r="N30" s="13">
         <v>3000</v>
@@ -14249,10 +14249,10 @@
         <v>358</v>
       </c>
       <c r="L71" s="11">
-        <v>20239</v>
+        <v>20179</v>
       </c>
       <c r="M71" s="11">
-        <v>42093</v>
+        <v>42094</v>
       </c>
       <c r="N71" s="13">
         <v>3000</v>
@@ -14955,10 +14955,10 @@
         <v>517</v>
       </c>
       <c r="L83" s="11">
-        <v>23610</v>
+        <v>23244</v>
       </c>
       <c r="M83" s="11">
-        <v>45525</v>
+        <v>45159</v>
       </c>
       <c r="N83" s="13">
         <v>3000</v>
@@ -15014,10 +15014,10 @@
         <v>44</v>
       </c>
       <c r="L84" s="11">
-        <v>23512</v>
+        <v>23513</v>
       </c>
       <c r="M84" s="11">
-        <v>45427</v>
+        <v>45428</v>
       </c>
       <c r="N84" s="13">
         <v>3000</v>
@@ -16874,10 +16874,10 @@
         <v>298</v>
       </c>
       <c r="L116" s="11">
-        <v>23791</v>
+        <v>23425</v>
       </c>
       <c r="M116" s="11">
-        <v>45706</v>
+        <v>45340</v>
       </c>
       <c r="N116" s="13">
         <v>3000</v>
@@ -18322,10 +18322,10 @@
         <v>657</v>
       </c>
       <c r="L142" s="11">
-        <v>23484</v>
+        <v>23575</v>
       </c>
       <c r="M142" s="11">
-        <v>45399</v>
+        <v>45490</v>
       </c>
       <c r="N142" s="13">
         <v>3000</v>
@@ -18550,10 +18550,10 @@
         <v>39</v>
       </c>
       <c r="L146" s="11">
-        <v>23886</v>
+        <v>23975</v>
       </c>
       <c r="M146" s="11">
-        <v>45801</v>
+        <v>45890</v>
       </c>
       <c r="N146" s="13">
         <v>2500</v>
@@ -20715,10 +20715,10 @@
         <v>44</v>
       </c>
       <c r="L185" s="11">
-        <v>23202</v>
+        <v>23203</v>
       </c>
       <c r="M185" s="11">
-        <v>45117</v>
+        <v>45118</v>
       </c>
       <c r="N185" s="13">
         <v>3000</v>

</xml_diff>

<commit_message>
auto update (48 cells, +8, -5)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3255,7 +3255,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S124"/>
+  <dimension ref="A1:S121"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -3283,7 +3283,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D122)</f>
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -3369,10 +3369,10 @@
         <v>44648</v>
       </c>
       <c r="I3" s="11">
-        <v>46293</v>
+        <v>46201</v>
       </c>
       <c r="J3" s="12">
-        <v>46383</v>
+        <v>46292</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>29</v>
@@ -3426,10 +3426,10 @@
         <v>44649</v>
       </c>
       <c r="I4" s="11">
-        <v>46294</v>
+        <v>46202</v>
       </c>
       <c r="J4" s="12">
-        <v>46384</v>
+        <v>46293</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>32</v>
@@ -3483,10 +3483,10 @@
         <v>41730</v>
       </c>
       <c r="I5" s="11">
-        <v>46316</v>
+        <v>46204</v>
       </c>
       <c r="J5" s="12">
-        <v>46407</v>
+        <v>46295</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>35</v>
@@ -3661,10 +3661,10 @@
         <v>29</v>
       </c>
       <c r="L8" s="11">
-        <v>21845</v>
+        <v>21844</v>
       </c>
       <c r="M8" s="11">
-        <v>43760</v>
+        <v>43759</v>
       </c>
       <c r="N8" s="13">
         <v>3500</v>
@@ -3889,7 +3889,7 @@
         <v>29</v>
       </c>
       <c r="L12" s="11">
-        <v>22290</v>
+        <v>22291</v>
       </c>
       <c r="M12" s="11">
         <v>44205</v>
@@ -4003,10 +4003,10 @@
         <v>64</v>
       </c>
       <c r="L14" s="11">
-        <v>22797</v>
+        <v>22796</v>
       </c>
       <c r="M14" s="11">
-        <v>44712</v>
+        <v>44711</v>
       </c>
       <c r="N14" s="13">
         <v>3000</v>
@@ -4735,7 +4735,7 @@
         <v>45740</v>
       </c>
       <c r="I27" s="11">
-        <v>45924</v>
+        <v>46289</v>
       </c>
       <c r="J27" s="12">
         <v>46379</v>
@@ -5985,7 +5985,7 @@
         <v>44014</v>
       </c>
       <c r="I49" s="11">
-        <v>46024</v>
+        <v>46297</v>
       </c>
       <c r="J49" s="12">
         <v>46388</v>
@@ -6505,10 +6505,10 @@
         <v>190</v>
       </c>
       <c r="L58" s="11">
-        <v>22637</v>
+        <v>22638</v>
       </c>
       <c r="M58" s="11">
-        <v>44552</v>
+        <v>44553</v>
       </c>
       <c r="N58" s="13">
         <v>3000</v>
@@ -6733,10 +6733,10 @@
         <v>201</v>
       </c>
       <c r="L62" s="11">
-        <v>24026</v>
+        <v>24308</v>
       </c>
       <c r="M62" s="11">
-        <v>45941</v>
+        <v>46223</v>
       </c>
       <c r="N62" s="13">
         <v>3000</v>
@@ -7244,10 +7244,10 @@
         <v>224</v>
       </c>
       <c r="L71" s="11">
-        <v>22934</v>
+        <v>22933</v>
       </c>
       <c r="M71" s="11">
-        <v>44849</v>
+        <v>44848</v>
       </c>
       <c r="N71" s="13">
         <v>2500</v>
@@ -8259,7 +8259,7 @@
         <v>45888</v>
       </c>
       <c r="I89" s="11">
-        <v>46253</v>
+        <v>46345</v>
       </c>
       <c r="J89" s="12">
         <v>46436</v>
@@ -8665,10 +8665,10 @@
         <v>106</v>
       </c>
       <c r="L96" s="11">
-        <v>24062</v>
+        <v>24261</v>
       </c>
       <c r="M96" s="11">
-        <v>45977</v>
+        <v>46176</v>
       </c>
       <c r="N96" s="13">
         <v>3000</v>
@@ -8773,7 +8773,7 @@
         <v>46104</v>
       </c>
       <c r="J98" s="12">
-        <v>46560</v>
+        <v>46468</v>
       </c>
       <c r="K98" s="7" t="s">
         <v>106</v>
@@ -8893,7 +8893,7 @@
         <v>310</v>
       </c>
       <c r="L100" s="11">
-        <v>19207</v>
+        <v>22859</v>
       </c>
       <c r="M100" s="11">
         <v>41122</v>
@@ -9001,7 +9001,7 @@
         <v>46143</v>
       </c>
       <c r="J102" s="12">
-        <v>46599</v>
+        <v>46507</v>
       </c>
       <c r="K102" s="7" t="s">
         <v>317</v>
@@ -9227,7 +9227,7 @@
         <v>46174</v>
       </c>
       <c r="J106" s="12">
-        <v>46630</v>
+        <v>46538</v>
       </c>
       <c r="K106" s="7" t="s">
         <v>29</v>
@@ -9886,14 +9886,16 @@
         <v>237</v>
       </c>
       <c r="L119" s="11">
-        <v>24366</v>
+        <v>24316</v>
       </c>
       <c r="M119" s="11">
-        <v>46281</v>
-      </c>
-      <c r="N119" s="13"/>
+        <v>46231</v>
+      </c>
+      <c r="N119" s="13">
+        <v>2500</v>
+      </c>
       <c r="O119" s="7" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
       <c r="P119" s="13">
         <v>26609161301038</v>
@@ -9928,25 +9930,17 @@
       <c r="G120" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="H120" s="10">
-        <v>45139</v>
-      </c>
+      <c r="H120" s="10"/>
       <c r="I120" s="11"/>
       <c r="J120" s="12"/>
       <c r="K120" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="L120" s="11">
-        <v>22510</v>
-      </c>
-      <c r="M120" s="11">
-        <v>45117</v>
-      </c>
+      <c r="L120" s="11"/>
+      <c r="M120" s="11"/>
       <c r="N120" s="13"/>
       <c r="O120" s="7"/>
-      <c r="P120" s="13">
-        <v>26108171301291</v>
-      </c>
+      <c r="P120" s="13"/>
       <c r="Q120" s="16"/>
       <c r="R120" s="15"/>
       <c r="S120" s="7"/>
@@ -9973,184 +9967,23 @@
       <c r="G121" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="H121" s="10">
-        <v>45263</v>
-      </c>
-      <c r="I121" s="11">
-        <v>45721</v>
-      </c>
-      <c r="J121" s="12">
-        <v>46085</v>
-      </c>
+      <c r="H121" s="10"/>
+      <c r="I121" s="11"/>
+      <c r="J121" s="12"/>
       <c r="K121" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="L121" s="11">
-        <v>21886</v>
-      </c>
-      <c r="M121" s="11">
-        <v>43801</v>
-      </c>
+      <c r="L121" s="11"/>
+      <c r="M121" s="11"/>
       <c r="N121" s="13"/>
-      <c r="O121" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="P121" s="13">
-        <v>25912021300059</v>
-      </c>
+      <c r="O121" s="7"/>
+      <c r="P121" s="13"/>
       <c r="Q121" s="16"/>
       <c r="R121" s="15"/>
       <c r="S121" s="7"/>
     </row>
-    <row r="122" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A122" s="7">
-        <v>127</v>
-      </c>
-      <c r="B122" s="7">
-        <v>20211</v>
-      </c>
-      <c r="C122" s="8">
-        <v>151</v>
-      </c>
-      <c r="D122" s="9" t="s">
-        <v>351</v>
-      </c>
-      <c r="E122" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F122" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G122" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H122" s="10">
-        <v>44805</v>
-      </c>
-      <c r="I122" s="11"/>
-      <c r="J122" s="12"/>
-      <c r="K122" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L122" s="11">
-        <v>22944</v>
-      </c>
-      <c r="M122" s="11">
-        <v>44859</v>
-      </c>
-      <c r="N122" s="13"/>
-      <c r="O122" s="7"/>
-      <c r="P122" s="13">
-        <v>26210251400258</v>
-      </c>
-      <c r="Q122" s="16"/>
-      <c r="R122" s="15"/>
-      <c r="S122" s="7"/>
-    </row>
-    <row r="123" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A123" s="7">
-        <v>128</v>
-      </c>
-      <c r="B123" s="7">
-        <v>20212</v>
-      </c>
-      <c r="C123" s="8">
-        <v>152</v>
-      </c>
-      <c r="D123" s="9" t="s">
-        <v>353</v>
-      </c>
-      <c r="E123" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F123" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G123" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H123" s="10">
-        <v>44814</v>
-      </c>
-      <c r="I123" s="11"/>
-      <c r="J123" s="12"/>
-      <c r="K123" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L123" s="11">
-        <v>21539</v>
-      </c>
-      <c r="M123" s="11">
-        <v>43454</v>
-      </c>
-      <c r="N123" s="13"/>
-      <c r="O123" s="7"/>
-      <c r="P123" s="13">
-        <v>25812208800538</v>
-      </c>
-      <c r="Q123" s="16"/>
-      <c r="R123" s="15"/>
-      <c r="S123" s="7"/>
-    </row>
-    <row r="124" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A124" s="7">
-        <v>129</v>
-      </c>
-      <c r="B124" s="7">
-        <v>20078</v>
-      </c>
-      <c r="C124" s="8">
-        <v>71</v>
-      </c>
-      <c r="D124" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E124" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F124" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G124" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H124" s="10">
-        <v>40063</v>
-      </c>
-      <c r="I124" s="11">
-        <v>46174</v>
-      </c>
-      <c r="J124" s="12">
-        <v>46265</v>
-      </c>
-      <c r="K124" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="L124" s="11">
-        <v>17467</v>
-      </c>
-      <c r="M124" s="11">
-        <v>35730</v>
-      </c>
-      <c r="N124" s="13">
-        <v>3500</v>
-      </c>
-      <c r="O124" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="P124" s="13">
-        <v>24710270101052</v>
-      </c>
-      <c r="Q124" s="16">
-        <v>1221545221</v>
-      </c>
-      <c r="R124" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="S124" s="7"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:S124"/>
+  <autoFilter ref="A2:S121"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>
@@ -10164,7 +9997,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S263"/>
+  <dimension ref="A1:S269"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -10192,7 +10025,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D189)</f>
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -10696,10 +10529,10 @@
         <v>373</v>
       </c>
       <c r="L10" s="11">
-        <v>20381</v>
+        <v>20371</v>
       </c>
       <c r="M10" s="11">
-        <v>42296</v>
+        <v>42286</v>
       </c>
       <c r="N10" s="13">
         <v>2500</v>
@@ -11858,10 +11691,10 @@
         <v>385</v>
       </c>
       <c r="L30" s="11">
-        <v>23563</v>
+        <v>23472</v>
       </c>
       <c r="M30" s="11">
-        <v>45478</v>
+        <v>45387</v>
       </c>
       <c r="N30" s="13">
         <v>3000</v>
@@ -14249,10 +14082,10 @@
         <v>358</v>
       </c>
       <c r="L71" s="11">
-        <v>20179</v>
+        <v>20239</v>
       </c>
       <c r="M71" s="11">
-        <v>42094</v>
+        <v>42093</v>
       </c>
       <c r="N71" s="13">
         <v>3000</v>
@@ -14955,10 +14788,10 @@
         <v>517</v>
       </c>
       <c r="L83" s="11">
-        <v>23244</v>
+        <v>23610</v>
       </c>
       <c r="M83" s="11">
-        <v>45159</v>
+        <v>45525</v>
       </c>
       <c r="N83" s="13">
         <v>3000</v>
@@ -15014,10 +14847,10 @@
         <v>44</v>
       </c>
       <c r="L84" s="11">
-        <v>23513</v>
+        <v>23512</v>
       </c>
       <c r="M84" s="11">
-        <v>45428</v>
+        <v>45427</v>
       </c>
       <c r="N84" s="13">
         <v>3000</v>
@@ -16874,10 +16707,10 @@
         <v>298</v>
       </c>
       <c r="L116" s="11">
-        <v>23425</v>
+        <v>23791</v>
       </c>
       <c r="M116" s="11">
-        <v>45340</v>
+        <v>45706</v>
       </c>
       <c r="N116" s="13">
         <v>3000</v>
@@ -18322,10 +18155,10 @@
         <v>657</v>
       </c>
       <c r="L142" s="11">
-        <v>23575</v>
+        <v>23484</v>
       </c>
       <c r="M142" s="11">
-        <v>45490</v>
+        <v>45399</v>
       </c>
       <c r="N142" s="13">
         <v>3000</v>
@@ -18550,10 +18383,10 @@
         <v>39</v>
       </c>
       <c r="L146" s="11">
-        <v>23975</v>
+        <v>23886</v>
       </c>
       <c r="M146" s="11">
-        <v>45890</v>
+        <v>45801</v>
       </c>
       <c r="N146" s="13">
         <v>2500</v>
@@ -20715,10 +20548,10 @@
         <v>44</v>
       </c>
       <c r="L185" s="11">
-        <v>23203</v>
+        <v>23202</v>
       </c>
       <c r="M185" s="11">
-        <v>45118</v>
+        <v>45117</v>
       </c>
       <c r="N185" s="13">
         <v>3000</v>
@@ -24189,8 +24022,300 @@
         <v>910</v>
       </c>
     </row>
+    <row r="264" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A264" s="7">
+        <v>262</v>
+      </c>
+      <c r="B264" s="7">
+        <v>20274</v>
+      </c>
+      <c r="C264" s="8">
+        <v>19</v>
+      </c>
+      <c r="D264" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="E264" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F264" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="G264" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H264" s="10">
+        <v>45139</v>
+      </c>
+      <c r="I264" s="11"/>
+      <c r="J264" s="12"/>
+      <c r="K264" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L264" s="11">
+        <v>22510</v>
+      </c>
+      <c r="M264" s="11">
+        <v>45117</v>
+      </c>
+      <c r="N264" s="13"/>
+      <c r="O264" s="7"/>
+      <c r="P264" s="13">
+        <v>26108171301291</v>
+      </c>
+      <c r="Q264" s="14"/>
+      <c r="R264" s="15"/>
+      <c r="S264" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="265" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A265" s="7">
+        <v>263</v>
+      </c>
+      <c r="B265" s="7">
+        <v>20276</v>
+      </c>
+      <c r="C265" s="8">
+        <v>56</v>
+      </c>
+      <c r="D265" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="E265" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F265" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G265" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H265" s="10">
+        <v>45263</v>
+      </c>
+      <c r="I265" s="11">
+        <v>45629</v>
+      </c>
+      <c r="J265" s="12">
+        <v>45720</v>
+      </c>
+      <c r="K265" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L265" s="11">
+        <v>21886</v>
+      </c>
+      <c r="M265" s="11">
+        <v>43801</v>
+      </c>
+      <c r="N265" s="13"/>
+      <c r="O265" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P265" s="13">
+        <v>25912021300059</v>
+      </c>
+      <c r="Q265" s="14"/>
+      <c r="R265" s="15"/>
+      <c r="S265" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="266" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A266" s="7">
+        <v>264</v>
+      </c>
+      <c r="B266" s="7">
+        <v>20211</v>
+      </c>
+      <c r="C266" s="8">
+        <v>151</v>
+      </c>
+      <c r="D266" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="E266" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F266" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G266" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H266" s="10">
+        <v>44805</v>
+      </c>
+      <c r="I266" s="11"/>
+      <c r="J266" s="12"/>
+      <c r="K266" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L266" s="11">
+        <v>22944</v>
+      </c>
+      <c r="M266" s="11">
+        <v>44859</v>
+      </c>
+      <c r="N266" s="13"/>
+      <c r="O266" s="7"/>
+      <c r="P266" s="13">
+        <v>26210251400258</v>
+      </c>
+      <c r="Q266" s="14"/>
+      <c r="R266" s="15"/>
+      <c r="S266" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="267" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A267" s="7">
+        <v>265</v>
+      </c>
+      <c r="B267" s="7">
+        <v>20212</v>
+      </c>
+      <c r="C267" s="8">
+        <v>152</v>
+      </c>
+      <c r="D267" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="E267" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F267" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G267" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H267" s="10">
+        <v>44814</v>
+      </c>
+      <c r="I267" s="11"/>
+      <c r="J267" s="12"/>
+      <c r="K267" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L267" s="11">
+        <v>21539</v>
+      </c>
+      <c r="M267" s="11">
+        <v>43454</v>
+      </c>
+      <c r="N267" s="13"/>
+      <c r="O267" s="7"/>
+      <c r="P267" s="13">
+        <v>25812208800538</v>
+      </c>
+      <c r="Q267" s="14"/>
+      <c r="R267" s="15"/>
+      <c r="S267" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="268" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A268" s="7">
+        <v>266</v>
+      </c>
+      <c r="B268" s="7">
+        <v>20078</v>
+      </c>
+      <c r="C268" s="8">
+        <v>71</v>
+      </c>
+      <c r="D268" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E268" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F268" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G268" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H268" s="10">
+        <v>40063</v>
+      </c>
+      <c r="I268" s="11">
+        <v>46174</v>
+      </c>
+      <c r="J268" s="12">
+        <v>46265</v>
+      </c>
+      <c r="K268" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="L268" s="11">
+        <v>17467</v>
+      </c>
+      <c r="M268" s="11">
+        <v>35730</v>
+      </c>
+      <c r="N268" s="13">
+        <v>3500</v>
+      </c>
+      <c r="O268" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P268" s="13">
+        <v>24710270101052</v>
+      </c>
+      <c r="Q268" s="14">
+        <v>1221545221</v>
+      </c>
+      <c r="R268" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="S268" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="269" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A269" s="7">
+        <v>267</v>
+      </c>
+      <c r="B269" s="7"/>
+      <c r="C269" s="8"/>
+      <c r="D269" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="E269" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F269" s="7" t="s">
+        <v>783</v>
+      </c>
+      <c r="G269" s="7"/>
+      <c r="H269" s="10">
+        <v>44827</v>
+      </c>
+      <c r="I269" s="11">
+        <v>45169</v>
+      </c>
+      <c r="J269" s="12">
+        <v>45169</v>
+      </c>
+      <c r="K269" s="7" t="s">
+        <v>784</v>
+      </c>
+      <c r="L269" s="11"/>
+      <c r="M269" s="11"/>
+      <c r="N269" s="13"/>
+      <c r="O269" s="7"/>
+      <c r="P269" s="13"/>
+      <c r="Q269" s="14"/>
+      <c r="R269" s="15"/>
+      <c r="S269" s="7" t="s">
+        <v>356</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S263"/>
+  <autoFilter ref="A2:S269"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
auto update (44 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3378,10 +3378,10 @@
         <v>44648</v>
       </c>
       <c r="I3" s="11">
-        <v>46293</v>
+        <v>46201</v>
       </c>
       <c r="J3" s="12">
-        <v>46383</v>
+        <v>46292</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>29</v>
@@ -3435,10 +3435,10 @@
         <v>44649</v>
       </c>
       <c r="I4" s="11">
-        <v>46294</v>
+        <v>46202</v>
       </c>
       <c r="J4" s="12">
-        <v>46384</v>
+        <v>46293</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>32</v>
@@ -3492,10 +3492,10 @@
         <v>41730</v>
       </c>
       <c r="I5" s="11">
-        <v>46296</v>
+        <v>46204</v>
       </c>
       <c r="J5" s="12">
-        <v>46387</v>
+        <v>46295</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>35</v>
@@ -3549,10 +3549,10 @@
         <v>45874</v>
       </c>
       <c r="I6" s="11">
-        <v>46331</v>
+        <v>46239</v>
       </c>
       <c r="J6" s="12">
-        <v>46422</v>
+        <v>46330</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>39</v>
@@ -3661,19 +3661,19 @@
         <v>43787</v>
       </c>
       <c r="I8" s="11">
-        <v>46252</v>
+        <v>46344</v>
       </c>
       <c r="J8" s="12">
-        <v>46343</v>
+        <v>46435</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>29</v>
       </c>
       <c r="L8" s="11">
-        <v>21845</v>
+        <v>21844</v>
       </c>
       <c r="M8" s="11">
-        <v>43760</v>
+        <v>43759</v>
       </c>
       <c r="N8" s="13">
         <v>3500</v>
@@ -3898,7 +3898,7 @@
         <v>29</v>
       </c>
       <c r="L12" s="11">
-        <v>22290</v>
+        <v>22291</v>
       </c>
       <c r="M12" s="11">
         <v>44205</v>
@@ -4012,10 +4012,10 @@
         <v>64</v>
       </c>
       <c r="L14" s="11">
-        <v>22797</v>
+        <v>22796</v>
       </c>
       <c r="M14" s="11">
-        <v>44712</v>
+        <v>44711</v>
       </c>
       <c r="N14" s="13">
         <v>3000</v>
@@ -4026,8 +4026,8 @@
       <c r="P14" s="13">
         <v>26205312101334</v>
       </c>
-      <c r="Q14" s="16">
-        <v>1225461250</v>
+      <c r="Q14" s="16" t="s">
+        <v>65</v>
       </c>
       <c r="R14" s="15" t="s">
         <v>66</v>
@@ -4744,7 +4744,7 @@
         <v>45740</v>
       </c>
       <c r="I27" s="11">
-        <v>45924</v>
+        <v>46289</v>
       </c>
       <c r="J27" s="12">
         <v>46379</v>
@@ -5994,7 +5994,7 @@
         <v>44014</v>
       </c>
       <c r="I49" s="11">
-        <v>46024</v>
+        <v>46297</v>
       </c>
       <c r="J49" s="12">
         <v>46388</v>
@@ -6188,8 +6188,8 @@
       <c r="P52" s="13">
         <v>26607280102199</v>
       </c>
-      <c r="Q52" s="16">
-        <v>1229037749</v>
+      <c r="Q52" s="16" t="s">
+        <v>174</v>
       </c>
       <c r="R52" s="15" t="s">
         <v>175</v>
@@ -6514,10 +6514,10 @@
         <v>190</v>
       </c>
       <c r="L58" s="11">
-        <v>22637</v>
+        <v>22638</v>
       </c>
       <c r="M58" s="11">
-        <v>44552</v>
+        <v>44553</v>
       </c>
       <c r="N58" s="13">
         <v>3000</v>
@@ -6742,10 +6742,10 @@
         <v>201</v>
       </c>
       <c r="L62" s="11">
-        <v>24026</v>
+        <v>24308</v>
       </c>
       <c r="M62" s="11">
-        <v>45941</v>
+        <v>46223</v>
       </c>
       <c r="N62" s="13">
         <v>3000</v>
@@ -7155,8 +7155,8 @@
       <c r="P69" s="13">
         <v>26201030103312</v>
       </c>
-      <c r="Q69" s="14" t="s">
-        <v>913</v>
+      <c r="Q69" s="14">
+        <v>12269601666</v>
       </c>
       <c r="R69" s="15" t="s">
         <v>217</v>
@@ -7253,10 +7253,10 @@
         <v>224</v>
       </c>
       <c r="L71" s="11">
-        <v>22934</v>
+        <v>22933</v>
       </c>
       <c r="M71" s="11">
-        <v>44849</v>
+        <v>44848</v>
       </c>
       <c r="N71" s="13">
         <v>2500</v>
@@ -7313,7 +7313,7 @@
         <v>24309</v>
       </c>
       <c r="M72" s="11">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="N72" s="13">
         <v>3000</v>
@@ -8048,7 +8048,7 @@
         <v>46425</v>
       </c>
       <c r="K85" s="7" t="s">
-        <v>306</v>
+        <v>265</v>
       </c>
       <c r="L85" s="11">
         <v>24123</v>
@@ -8268,7 +8268,7 @@
         <v>45888</v>
       </c>
       <c r="I89" s="11">
-        <v>46253</v>
+        <v>46345</v>
       </c>
       <c r="J89" s="12">
         <v>46436</v>
@@ -8451,7 +8451,7 @@
         <v>23476</v>
       </c>
       <c r="M92" s="11">
-        <v>45391</v>
+        <v>46121</v>
       </c>
       <c r="N92" s="13">
         <v>3000</v>
@@ -8674,10 +8674,10 @@
         <v>106</v>
       </c>
       <c r="L96" s="11">
-        <v>24062</v>
+        <v>24261</v>
       </c>
       <c r="M96" s="11">
-        <v>45977</v>
+        <v>46176</v>
       </c>
       <c r="N96" s="13">
         <v>3000</v>
@@ -8782,7 +8782,7 @@
         <v>46104</v>
       </c>
       <c r="J98" s="12">
-        <v>46560</v>
+        <v>46468</v>
       </c>
       <c r="K98" s="7" t="s">
         <v>106</v>
@@ -8791,7 +8791,7 @@
         <v>24188</v>
       </c>
       <c r="M98" s="11">
-        <v>46103</v>
+        <v>60713</v>
       </c>
       <c r="N98" s="13">
         <v>10000</v>
@@ -8902,7 +8902,7 @@
         <v>310</v>
       </c>
       <c r="L100" s="11">
-        <v>19207</v>
+        <v>22859</v>
       </c>
       <c r="M100" s="11">
         <v>41122</v>
@@ -9010,7 +9010,7 @@
         <v>46143</v>
       </c>
       <c r="J102" s="12">
-        <v>46599</v>
+        <v>46507</v>
       </c>
       <c r="K102" s="7" t="s">
         <v>317</v>
@@ -9019,7 +9019,7 @@
         <v>22964</v>
       </c>
       <c r="M102" s="11">
-        <v>44879</v>
+        <v>44909</v>
       </c>
       <c r="N102" s="13">
         <v>10000</v>
@@ -9236,7 +9236,7 @@
         <v>46174</v>
       </c>
       <c r="J106" s="12">
-        <v>46630</v>
+        <v>46538</v>
       </c>
       <c r="K106" s="7" t="s">
         <v>29</v>
@@ -9260,7 +9260,7 @@
         <v>1281771400</v>
       </c>
       <c r="R106" s="15" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="S106" s="7"/>
     </row>
@@ -9895,14 +9895,16 @@
         <v>237</v>
       </c>
       <c r="L119" s="11">
-        <v>24366</v>
+        <v>24316</v>
       </c>
       <c r="M119" s="11">
-        <v>46281</v>
-      </c>
-      <c r="N119" s="13"/>
+        <v>46231</v>
+      </c>
+      <c r="N119" s="13">
+        <v>2500</v>
+      </c>
       <c r="O119" s="7" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
       <c r="P119" s="13">
         <v>26609161301038</v>
@@ -9911,7 +9913,7 @@
         <v>1223226004</v>
       </c>
       <c r="R119" s="15" t="s">
-        <v>915</v>
+        <v>912</v>
       </c>
       <c r="S119" s="7"/>
     </row>

</xml_diff>

<commit_message>
auto update (23 cells, +5, -8)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2504" uniqueCount="913">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="915">
   <si>
     <t xml:space="preserve">الاجمالى </t>
   </si>
@@ -2751,6 +2751,12 @@
   </si>
   <si>
     <t xml:space="preserve">عزرة عادل حجازي -تل بني تميم - عرب السلام شبين القناطر - القليوبيه</t>
+  </si>
+  <si>
+    <t xml:space="preserve">377.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">محت فوكيه ناشد سلمون</t>
   </si>
 </sst>
 </file>
@@ -3255,7 +3261,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S121"/>
+  <dimension ref="A1:S126"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -3283,7 +3289,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D122)</f>
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -3369,10 +3375,10 @@
         <v>44648</v>
       </c>
       <c r="I3" s="11">
-        <v>46201</v>
+        <v>46293</v>
       </c>
       <c r="J3" s="12">
-        <v>46292</v>
+        <v>46383</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>29</v>
@@ -3426,10 +3432,10 @@
         <v>44649</v>
       </c>
       <c r="I4" s="11">
-        <v>46202</v>
+        <v>46294</v>
       </c>
       <c r="J4" s="12">
-        <v>46293</v>
+        <v>46384</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>32</v>
@@ -3483,10 +3489,10 @@
         <v>41730</v>
       </c>
       <c r="I5" s="11">
-        <v>46204</v>
+        <v>46296</v>
       </c>
       <c r="J5" s="12">
-        <v>46295</v>
+        <v>46387</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>35</v>
@@ -3540,10 +3546,10 @@
         <v>45874</v>
       </c>
       <c r="I6" s="11">
-        <v>46239</v>
+        <v>46331</v>
       </c>
       <c r="J6" s="12">
-        <v>46330</v>
+        <v>46422</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>39</v>
@@ -3709,10 +3715,10 @@
         <v>44343</v>
       </c>
       <c r="I9" s="11">
-        <v>46261</v>
+        <v>46353</v>
       </c>
       <c r="J9" s="12">
-        <v>46352</v>
+        <v>46444</v>
       </c>
       <c r="K9" s="7" t="s">
         <v>29</v>
@@ -3766,10 +3772,10 @@
         <v>43339</v>
       </c>
       <c r="I10" s="11">
-        <v>46261</v>
+        <v>46353</v>
       </c>
       <c r="J10" s="12">
-        <v>46352</v>
+        <v>46444</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>29</v>
@@ -4735,7 +4741,7 @@
         <v>45740</v>
       </c>
       <c r="I27" s="11">
-        <v>46289</v>
+        <v>45924</v>
       </c>
       <c r="J27" s="12">
         <v>46379</v>
@@ -5985,10 +5991,10 @@
         <v>44014</v>
       </c>
       <c r="I49" s="11">
-        <v>46297</v>
+        <v>46328</v>
       </c>
       <c r="J49" s="12">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="K49" s="7" t="s">
         <v>29</v>
@@ -8259,7 +8265,7 @@
         <v>45888</v>
       </c>
       <c r="I89" s="11">
-        <v>46345</v>
+        <v>46253</v>
       </c>
       <c r="J89" s="12">
         <v>46436</v>
@@ -8773,7 +8779,7 @@
         <v>46104</v>
       </c>
       <c r="J98" s="12">
-        <v>46468</v>
+        <v>46560</v>
       </c>
       <c r="K98" s="7" t="s">
         <v>106</v>
@@ -9001,7 +9007,7 @@
         <v>46143</v>
       </c>
       <c r="J102" s="12">
-        <v>46507</v>
+        <v>46599</v>
       </c>
       <c r="K102" s="7" t="s">
         <v>317</v>
@@ -9227,7 +9233,7 @@
         <v>46174</v>
       </c>
       <c r="J106" s="12">
-        <v>46538</v>
+        <v>46630</v>
       </c>
       <c r="K106" s="7" t="s">
         <v>29</v>
@@ -9891,11 +9897,9 @@
       <c r="M119" s="11">
         <v>46231</v>
       </c>
-      <c r="N119" s="13">
-        <v>2500</v>
-      </c>
+      <c r="N119" s="13"/>
       <c r="O119" s="7" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="P119" s="13">
         <v>26609161301038</v>
@@ -9982,8 +9986,229 @@
       <c r="R121" s="15"/>
       <c r="S121" s="7"/>
     </row>
+    <row r="122" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A122" s="7">
+        <v>127</v>
+      </c>
+      <c r="B122" s="7">
+        <v>20276</v>
+      </c>
+      <c r="C122" s="8">
+        <v>56</v>
+      </c>
+      <c r="D122" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="E122" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F122" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G122" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H122" s="10">
+        <v>45263</v>
+      </c>
+      <c r="I122" s="11">
+        <v>46086</v>
+      </c>
+      <c r="J122" s="12">
+        <v>46450</v>
+      </c>
+      <c r="K122" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L122" s="11">
+        <v>21886</v>
+      </c>
+      <c r="M122" s="11">
+        <v>43801</v>
+      </c>
+      <c r="N122" s="13"/>
+      <c r="O122" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P122" s="13">
+        <v>25912021300059</v>
+      </c>
+      <c r="Q122" s="16"/>
+      <c r="R122" s="15"/>
+      <c r="S122" s="7"/>
+    </row>
+    <row r="123" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A123" s="7">
+        <v>128</v>
+      </c>
+      <c r="B123" s="7">
+        <v>20274</v>
+      </c>
+      <c r="C123" s="8">
+        <v>19</v>
+      </c>
+      <c r="D123" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="E123" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F123" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="G123" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H123" s="10">
+        <v>45139</v>
+      </c>
+      <c r="I123" s="11"/>
+      <c r="J123" s="12"/>
+      <c r="K123" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L123" s="11">
+        <v>22510</v>
+      </c>
+      <c r="M123" s="11">
+        <v>45117</v>
+      </c>
+      <c r="N123" s="13"/>
+      <c r="O123" s="7"/>
+      <c r="P123" s="13">
+        <v>26108171301291</v>
+      </c>
+      <c r="Q123" s="16"/>
+      <c r="R123" s="15"/>
+      <c r="S123" s="7"/>
+    </row>
+    <row r="124" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A124" s="7">
+        <v>129</v>
+      </c>
+      <c r="B124" s="7">
+        <v>20211</v>
+      </c>
+      <c r="C124" s="8">
+        <v>151</v>
+      </c>
+      <c r="D124" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="E124" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F124" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G124" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H124" s="10">
+        <v>44805</v>
+      </c>
+      <c r="I124" s="11"/>
+      <c r="J124" s="12"/>
+      <c r="K124" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L124" s="11">
+        <v>22944</v>
+      </c>
+      <c r="M124" s="11">
+        <v>44859</v>
+      </c>
+      <c r="N124" s="13"/>
+      <c r="O124" s="7"/>
+      <c r="P124" s="13">
+        <v>26210251400258</v>
+      </c>
+      <c r="Q124" s="16"/>
+      <c r="R124" s="15"/>
+      <c r="S124" s="7"/>
+    </row>
+    <row r="125" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A125" s="7">
+        <v>130</v>
+      </c>
+      <c r="B125" s="7">
+        <v>20212</v>
+      </c>
+      <c r="C125" s="8">
+        <v>152</v>
+      </c>
+      <c r="D125" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="E125" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F125" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G125" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H125" s="10">
+        <v>44814</v>
+      </c>
+      <c r="I125" s="11"/>
+      <c r="J125" s="12"/>
+      <c r="K125" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L125" s="11">
+        <v>21539</v>
+      </c>
+      <c r="M125" s="11">
+        <v>43454</v>
+      </c>
+      <c r="N125" s="13"/>
+      <c r="O125" s="7"/>
+      <c r="P125" s="13">
+        <v>25812208800538</v>
+      </c>
+      <c r="Q125" s="16"/>
+      <c r="R125" s="15"/>
+      <c r="S125" s="7"/>
+    </row>
+    <row r="126" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A126" s="7">
+        <v>131</v>
+      </c>
+      <c r="B126" s="7">
+        <v>20441</v>
+      </c>
+      <c r="C126" s="8" t="s">
+        <v>913</v>
+      </c>
+      <c r="D126" s="9" t="s">
+        <v>914</v>
+      </c>
+      <c r="E126" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F126" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G126" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H126" s="10"/>
+      <c r="I126" s="11"/>
+      <c r="J126" s="12"/>
+      <c r="K126" s="7"/>
+      <c r="L126" s="11"/>
+      <c r="M126" s="11"/>
+      <c r="N126" s="13"/>
+      <c r="O126" s="7"/>
+      <c r="P126" s="13"/>
+      <c r="Q126" s="16"/>
+      <c r="R126" s="15"/>
+      <c r="S126" s="7"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S121"/>
+  <autoFilter ref="A2:S126"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>
@@ -9997,7 +10222,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S269"/>
+  <dimension ref="A1:S261"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -10025,7 +10250,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D189)</f>
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -10170,10 +10395,10 @@
         <v>45323</v>
       </c>
       <c r="I4" s="11">
-        <v>45413</v>
+        <v>45505</v>
       </c>
       <c r="J4" s="12">
-        <v>45504</v>
+        <v>45596</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>358</v>
@@ -23822,32 +24047,26 @@
         <v>257</v>
       </c>
       <c r="B259" s="7">
-        <v>20368</v>
+        <v>20416</v>
       </c>
       <c r="C259" s="8">
-        <v>303</v>
+        <v>351</v>
       </c>
       <c r="D259" s="9" t="s">
-        <v>662</v>
+        <v>906</v>
       </c>
       <c r="E259" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F259" s="7" t="s">
-        <v>109</v>
+        <v>27</v>
       </c>
       <c r="G259" s="7"/>
-      <c r="H259" s="10">
-        <v>45931</v>
-      </c>
-      <c r="I259" s="11">
-        <v>45931</v>
-      </c>
-      <c r="J259" s="12">
-        <v>45931</v>
-      </c>
+      <c r="H259" s="10"/>
+      <c r="I259" s="11"/>
+      <c r="J259" s="12"/>
       <c r="K259" s="7" t="s">
-        <v>106</v>
+        <v>907</v>
       </c>
       <c r="L259" s="11"/>
       <c r="M259" s="11"/>
@@ -23856,76 +24075,92 @@
       <c r="P259" s="13"/>
       <c r="Q259" s="14"/>
       <c r="R259" s="15"/>
-      <c r="S259" s="7" t="s">
-        <v>905</v>
-      </c>
+      <c r="S259" s="7"/>
     </row>
     <row r="260" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A260" s="7">
         <v>258</v>
       </c>
       <c r="B260" s="7">
-        <v>20416</v>
+        <v>20078</v>
       </c>
       <c r="C260" s="8">
-        <v>351</v>
+        <v>71</v>
       </c>
       <c r="D260" s="9" t="s">
-        <v>906</v>
+        <v>19</v>
       </c>
       <c r="E260" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F260" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G260" s="7"/>
-      <c r="H260" s="10"/>
-      <c r="I260" s="11"/>
-      <c r="J260" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="G260" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H260" s="10">
+        <v>40063</v>
+      </c>
+      <c r="I260" s="11">
+        <v>46174</v>
+      </c>
+      <c r="J260" s="12">
+        <v>46265</v>
+      </c>
       <c r="K260" s="7" t="s">
-        <v>907</v>
-      </c>
-      <c r="L260" s="11"/>
-      <c r="M260" s="11"/>
-      <c r="N260" s="13"/>
-      <c r="O260" s="7"/>
-      <c r="P260" s="13"/>
-      <c r="Q260" s="14"/>
-      <c r="R260" s="15"/>
+        <v>23</v>
+      </c>
+      <c r="L260" s="11">
+        <v>17467</v>
+      </c>
+      <c r="M260" s="11">
+        <v>35730</v>
+      </c>
+      <c r="N260" s="13">
+        <v>3500</v>
+      </c>
+      <c r="O260" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P260" s="13">
+        <v>24710270101052</v>
+      </c>
+      <c r="Q260" s="14">
+        <v>1221545221</v>
+      </c>
+      <c r="R260" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="S260" s="7"/>
     </row>
     <row r="261" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A261" s="7">
         <v>259</v>
       </c>
-      <c r="B261" s="7">
-        <v>20411</v>
-      </c>
-      <c r="C261" s="8">
-        <v>346</v>
-      </c>
+      <c r="B261" s="7"/>
+      <c r="C261" s="8"/>
       <c r="D261" s="9" t="s">
-        <v>694</v>
+        <v>305</v>
       </c>
       <c r="E261" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F261" s="7" t="s">
-        <v>68</v>
+        <v>783</v>
       </c>
       <c r="G261" s="7"/>
       <c r="H261" s="10">
-        <v>46069</v>
+        <v>44827</v>
       </c>
       <c r="I261" s="11">
-        <v>46069</v>
+        <v>45169</v>
       </c>
       <c r="J261" s="12">
-        <v>46069</v>
+        <v>45169</v>
       </c>
       <c r="K261" s="7" t="s">
-        <v>695</v>
+        <v>784</v>
       </c>
       <c r="L261" s="11"/>
       <c r="M261" s="11"/>
@@ -23934,384 +24169,10 @@
       <c r="P261" s="13"/>
       <c r="Q261" s="14"/>
       <c r="R261" s="15"/>
-      <c r="S261" s="7" t="s">
-        <v>908</v>
-      </c>
-    </row>
-    <row r="262" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A262" s="7">
-        <v>260</v>
-      </c>
-      <c r="B262" s="7">
-        <v>20398</v>
-      </c>
-      <c r="C262" s="8">
-        <v>333</v>
-      </c>
-      <c r="D262" s="9" t="s">
-        <v>669</v>
-      </c>
-      <c r="E262" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F262" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="G262" s="7"/>
-      <c r="H262" s="10">
-        <v>46041</v>
-      </c>
-      <c r="I262" s="11">
-        <v>46041</v>
-      </c>
-      <c r="J262" s="12">
-        <v>46041</v>
-      </c>
-      <c r="K262" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="L262" s="11"/>
-      <c r="M262" s="11"/>
-      <c r="N262" s="13"/>
-      <c r="O262" s="7"/>
-      <c r="P262" s="13"/>
-      <c r="Q262" s="14"/>
-      <c r="R262" s="15"/>
-      <c r="S262" s="7" t="s">
-        <v>909</v>
-      </c>
-    </row>
-    <row r="263" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A263" s="7">
-        <v>261</v>
-      </c>
-      <c r="B263" s="7">
-        <v>342</v>
-      </c>
-      <c r="C263" s="8"/>
-      <c r="D263" s="9" t="s">
-        <v>677</v>
-      </c>
-      <c r="E263" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F263" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="G263" s="7"/>
-      <c r="H263" s="10">
-        <v>46057</v>
-      </c>
-      <c r="I263" s="11">
-        <v>46057</v>
-      </c>
-      <c r="J263" s="12">
-        <v>46057</v>
-      </c>
-      <c r="K263" s="7" t="s">
-        <v>409</v>
-      </c>
-      <c r="L263" s="11"/>
-      <c r="M263" s="11"/>
-      <c r="N263" s="13"/>
-      <c r="O263" s="7"/>
-      <c r="P263" s="13"/>
-      <c r="Q263" s="14"/>
-      <c r="R263" s="15"/>
-      <c r="S263" s="7" t="s">
-        <v>910</v>
-      </c>
-    </row>
-    <row r="264" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A264" s="7">
-        <v>262</v>
-      </c>
-      <c r="B264" s="7">
-        <v>20274</v>
-      </c>
-      <c r="C264" s="8">
-        <v>19</v>
-      </c>
-      <c r="D264" s="9" t="s">
-        <v>348</v>
-      </c>
-      <c r="E264" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F264" s="7" t="s">
-        <v>347</v>
-      </c>
-      <c r="G264" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H264" s="10">
-        <v>45139</v>
-      </c>
-      <c r="I264" s="11"/>
-      <c r="J264" s="12"/>
-      <c r="K264" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L264" s="11">
-        <v>22510</v>
-      </c>
-      <c r="M264" s="11">
-        <v>45117</v>
-      </c>
-      <c r="N264" s="13"/>
-      <c r="O264" s="7"/>
-      <c r="P264" s="13">
-        <v>26108171301291</v>
-      </c>
-      <c r="Q264" s="14"/>
-      <c r="R264" s="15"/>
-      <c r="S264" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="265" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A265" s="7">
-        <v>263</v>
-      </c>
-      <c r="B265" s="7">
-        <v>20276</v>
-      </c>
-      <c r="C265" s="8">
-        <v>56</v>
-      </c>
-      <c r="D265" s="9" t="s">
-        <v>350</v>
-      </c>
-      <c r="E265" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F265" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G265" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H265" s="10">
-        <v>45263</v>
-      </c>
-      <c r="I265" s="11">
-        <v>45629</v>
-      </c>
-      <c r="J265" s="12">
-        <v>45720</v>
-      </c>
-      <c r="K265" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L265" s="11">
-        <v>21886</v>
-      </c>
-      <c r="M265" s="11">
-        <v>43801</v>
-      </c>
-      <c r="N265" s="13"/>
-      <c r="O265" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="P265" s="13">
-        <v>25912021300059</v>
-      </c>
-      <c r="Q265" s="14"/>
-      <c r="R265" s="15"/>
-      <c r="S265" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="266" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A266" s="7">
-        <v>264</v>
-      </c>
-      <c r="B266" s="7">
-        <v>20211</v>
-      </c>
-      <c r="C266" s="8">
-        <v>151</v>
-      </c>
-      <c r="D266" s="9" t="s">
-        <v>351</v>
-      </c>
-      <c r="E266" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F266" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G266" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H266" s="10">
-        <v>44805</v>
-      </c>
-      <c r="I266" s="11"/>
-      <c r="J266" s="12"/>
-      <c r="K266" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L266" s="11">
-        <v>22944</v>
-      </c>
-      <c r="M266" s="11">
-        <v>44859</v>
-      </c>
-      <c r="N266" s="13"/>
-      <c r="O266" s="7"/>
-      <c r="P266" s="13">
-        <v>26210251400258</v>
-      </c>
-      <c r="Q266" s="14"/>
-      <c r="R266" s="15"/>
-      <c r="S266" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="267" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A267" s="7">
-        <v>265</v>
-      </c>
-      <c r="B267" s="7">
-        <v>20212</v>
-      </c>
-      <c r="C267" s="8">
-        <v>152</v>
-      </c>
-      <c r="D267" s="9" t="s">
-        <v>353</v>
-      </c>
-      <c r="E267" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F267" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G267" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H267" s="10">
-        <v>44814</v>
-      </c>
-      <c r="I267" s="11"/>
-      <c r="J267" s="12"/>
-      <c r="K267" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L267" s="11">
-        <v>21539</v>
-      </c>
-      <c r="M267" s="11">
-        <v>43454</v>
-      </c>
-      <c r="N267" s="13"/>
-      <c r="O267" s="7"/>
-      <c r="P267" s="13">
-        <v>25812208800538</v>
-      </c>
-      <c r="Q267" s="14"/>
-      <c r="R267" s="15"/>
-      <c r="S267" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="268" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A268" s="7">
-        <v>266</v>
-      </c>
-      <c r="B268" s="7">
-        <v>20078</v>
-      </c>
-      <c r="C268" s="8">
-        <v>71</v>
-      </c>
-      <c r="D268" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E268" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F268" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G268" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H268" s="10">
-        <v>40063</v>
-      </c>
-      <c r="I268" s="11">
-        <v>46174</v>
-      </c>
-      <c r="J268" s="12">
-        <v>46265</v>
-      </c>
-      <c r="K268" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="L268" s="11">
-        <v>17467</v>
-      </c>
-      <c r="M268" s="11">
-        <v>35730</v>
-      </c>
-      <c r="N268" s="13">
-        <v>3500</v>
-      </c>
-      <c r="O268" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="P268" s="13">
-        <v>24710270101052</v>
-      </c>
-      <c r="Q268" s="14">
-        <v>1221545221</v>
-      </c>
-      <c r="R268" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="S268" s="7"/>
-    </row>
-    <row r="269" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A269" s="7">
-        <v>267</v>
-      </c>
-      <c r="B269" s="7"/>
-      <c r="C269" s="8"/>
-      <c r="D269" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="E269" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F269" s="7" t="s">
-        <v>783</v>
-      </c>
-      <c r="G269" s="7"/>
-      <c r="H269" s="10">
-        <v>44827</v>
-      </c>
-      <c r="I269" s="11">
-        <v>45169</v>
-      </c>
-      <c r="J269" s="12">
-        <v>45169</v>
-      </c>
-      <c r="K269" s="7" t="s">
-        <v>784</v>
-      </c>
-      <c r="L269" s="11"/>
-      <c r="M269" s="11"/>
-      <c r="N269" s="13"/>
-      <c r="O269" s="7"/>
-      <c r="P269" s="13"/>
-      <c r="Q269" s="14"/>
-      <c r="R269" s="15"/>
-      <c r="S269" s="7"/>
+      <c r="S261" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:S269"/>
+  <autoFilter ref="A2:S261"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
auto update (0 cells, +4, -4)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3261,7 +3261,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S126"/>
+  <dimension ref="A1:S122"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -3289,7 +3289,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D122)</f>
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -9988,227 +9988,41 @@
     </row>
     <row r="122" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A122" s="7">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B122" s="7">
-        <v>20276</v>
-      </c>
-      <c r="C122" s="8">
-        <v>56</v>
+        <v>20441</v>
+      </c>
+      <c r="C122" s="8" t="s">
+        <v>913</v>
       </c>
       <c r="D122" s="9" t="s">
-        <v>350</v>
+        <v>914</v>
       </c>
       <c r="E122" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F122" s="7" t="s">
-        <v>180</v>
+        <v>68</v>
       </c>
       <c r="G122" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H122" s="10">
-        <v>45263</v>
-      </c>
-      <c r="I122" s="11">
-        <v>46086</v>
-      </c>
-      <c r="J122" s="12">
-        <v>46450</v>
-      </c>
-      <c r="K122" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L122" s="11">
-        <v>21886</v>
-      </c>
-      <c r="M122" s="11">
-        <v>43801</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="H122" s="10"/>
+      <c r="I122" s="11"/>
+      <c r="J122" s="12"/>
+      <c r="K122" s="7"/>
+      <c r="L122" s="11"/>
+      <c r="M122" s="11"/>
       <c r="N122" s="13"/>
-      <c r="O122" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="P122" s="13">
-        <v>25912021300059</v>
-      </c>
+      <c r="O122" s="7"/>
+      <c r="P122" s="13"/>
       <c r="Q122" s="16"/>
       <c r="R122" s="15"/>
       <c r="S122" s="7"/>
     </row>
-    <row r="123" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A123" s="7">
-        <v>128</v>
-      </c>
-      <c r="B123" s="7">
-        <v>20274</v>
-      </c>
-      <c r="C123" s="8">
-        <v>19</v>
-      </c>
-      <c r="D123" s="9" t="s">
-        <v>348</v>
-      </c>
-      <c r="E123" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F123" s="7" t="s">
-        <v>347</v>
-      </c>
-      <c r="G123" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H123" s="10">
-        <v>45139</v>
-      </c>
-      <c r="I123" s="11"/>
-      <c r="J123" s="12"/>
-      <c r="K123" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L123" s="11">
-        <v>22510</v>
-      </c>
-      <c r="M123" s="11">
-        <v>45117</v>
-      </c>
-      <c r="N123" s="13"/>
-      <c r="O123" s="7"/>
-      <c r="P123" s="13">
-        <v>26108171301291</v>
-      </c>
-      <c r="Q123" s="16"/>
-      <c r="R123" s="15"/>
-      <c r="S123" s="7"/>
-    </row>
-    <row r="124" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A124" s="7">
-        <v>129</v>
-      </c>
-      <c r="B124" s="7">
-        <v>20211</v>
-      </c>
-      <c r="C124" s="8">
-        <v>151</v>
-      </c>
-      <c r="D124" s="9" t="s">
-        <v>351</v>
-      </c>
-      <c r="E124" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F124" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G124" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H124" s="10">
-        <v>44805</v>
-      </c>
-      <c r="I124" s="11"/>
-      <c r="J124" s="12"/>
-      <c r="K124" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L124" s="11">
-        <v>22944</v>
-      </c>
-      <c r="M124" s="11">
-        <v>44859</v>
-      </c>
-      <c r="N124" s="13"/>
-      <c r="O124" s="7"/>
-      <c r="P124" s="13">
-        <v>26210251400258</v>
-      </c>
-      <c r="Q124" s="16"/>
-      <c r="R124" s="15"/>
-      <c r="S124" s="7"/>
-    </row>
-    <row r="125" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A125" s="7">
-        <v>130</v>
-      </c>
-      <c r="B125" s="7">
-        <v>20212</v>
-      </c>
-      <c r="C125" s="8">
-        <v>152</v>
-      </c>
-      <c r="D125" s="9" t="s">
-        <v>353</v>
-      </c>
-      <c r="E125" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F125" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G125" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H125" s="10">
-        <v>44814</v>
-      </c>
-      <c r="I125" s="11"/>
-      <c r="J125" s="12"/>
-      <c r="K125" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L125" s="11">
-        <v>21539</v>
-      </c>
-      <c r="M125" s="11">
-        <v>43454</v>
-      </c>
-      <c r="N125" s="13"/>
-      <c r="O125" s="7"/>
-      <c r="P125" s="13">
-        <v>25812208800538</v>
-      </c>
-      <c r="Q125" s="16"/>
-      <c r="R125" s="15"/>
-      <c r="S125" s="7"/>
-    </row>
-    <row r="126" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A126" s="7">
-        <v>131</v>
-      </c>
-      <c r="B126" s="7">
-        <v>20441</v>
-      </c>
-      <c r="C126" s="8" t="s">
-        <v>913</v>
-      </c>
-      <c r="D126" s="9" t="s">
-        <v>914</v>
-      </c>
-      <c r="E126" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F126" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="G126" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H126" s="10"/>
-      <c r="I126" s="11"/>
-      <c r="J126" s="12"/>
-      <c r="K126" s="7"/>
-      <c r="L126" s="11"/>
-      <c r="M126" s="11"/>
-      <c r="N126" s="13"/>
-      <c r="O126" s="7"/>
-      <c r="P126" s="13"/>
-      <c r="Q126" s="16"/>
-      <c r="R126" s="15"/>
-      <c r="S126" s="7"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:S126"/>
+  <autoFilter ref="A2:S122"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>
@@ -10222,7 +10036,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S261"/>
+  <dimension ref="A1:S265"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -10250,7 +10064,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D189)</f>
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -24171,8 +23985,202 @@
       <c r="R261" s="15"/>
       <c r="S261" s="7"/>
     </row>
+    <row r="262" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A262" s="7">
+        <v>260</v>
+      </c>
+      <c r="B262" s="7">
+        <v>20276</v>
+      </c>
+      <c r="C262" s="8">
+        <v>56</v>
+      </c>
+      <c r="D262" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="E262" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F262" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G262" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H262" s="10">
+        <v>45263</v>
+      </c>
+      <c r="I262" s="11">
+        <v>46086</v>
+      </c>
+      <c r="J262" s="12">
+        <v>46450</v>
+      </c>
+      <c r="K262" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L262" s="11">
+        <v>21886</v>
+      </c>
+      <c r="M262" s="11">
+        <v>43801</v>
+      </c>
+      <c r="N262" s="13"/>
+      <c r="O262" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P262" s="13">
+        <v>25912021300059</v>
+      </c>
+      <c r="Q262" s="14"/>
+      <c r="R262" s="15"/>
+      <c r="S262" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="263" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A263" s="7">
+        <v>261</v>
+      </c>
+      <c r="B263" s="7">
+        <v>20274</v>
+      </c>
+      <c r="C263" s="8">
+        <v>19</v>
+      </c>
+      <c r="D263" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="E263" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F263" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="G263" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H263" s="10">
+        <v>45139</v>
+      </c>
+      <c r="I263" s="11"/>
+      <c r="J263" s="12"/>
+      <c r="K263" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L263" s="11">
+        <v>22510</v>
+      </c>
+      <c r="M263" s="11">
+        <v>45117</v>
+      </c>
+      <c r="N263" s="13"/>
+      <c r="O263" s="7"/>
+      <c r="P263" s="13">
+        <v>26108171301291</v>
+      </c>
+      <c r="Q263" s="14"/>
+      <c r="R263" s="15"/>
+      <c r="S263" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="264" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A264" s="7">
+        <v>262</v>
+      </c>
+      <c r="B264" s="7">
+        <v>20211</v>
+      </c>
+      <c r="C264" s="8">
+        <v>151</v>
+      </c>
+      <c r="D264" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="E264" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F264" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G264" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H264" s="10">
+        <v>44805</v>
+      </c>
+      <c r="I264" s="11"/>
+      <c r="J264" s="12"/>
+      <c r="K264" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L264" s="11">
+        <v>22944</v>
+      </c>
+      <c r="M264" s="11">
+        <v>44859</v>
+      </c>
+      <c r="N264" s="13"/>
+      <c r="O264" s="7"/>
+      <c r="P264" s="13">
+        <v>26210251400258</v>
+      </c>
+      <c r="Q264" s="14"/>
+      <c r="R264" s="15"/>
+      <c r="S264" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="265" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A265" s="7">
+        <v>263</v>
+      </c>
+      <c r="B265" s="7">
+        <v>20212</v>
+      </c>
+      <c r="C265" s="8">
+        <v>152</v>
+      </c>
+      <c r="D265" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="E265" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F265" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G265" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H265" s="10">
+        <v>44814</v>
+      </c>
+      <c r="I265" s="11"/>
+      <c r="J265" s="12"/>
+      <c r="K265" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="L265" s="11">
+        <v>21539</v>
+      </c>
+      <c r="M265" s="11">
+        <v>43454</v>
+      </c>
+      <c r="N265" s="13"/>
+      <c r="O265" s="7"/>
+      <c r="P265" s="13">
+        <v>25812208800538</v>
+      </c>
+      <c r="Q265" s="14"/>
+      <c r="R265" s="15"/>
+      <c r="S265" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S261"/>
+  <autoFilter ref="A2:S265"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
auto update (23 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3667,10 +3667,10 @@
         <v>29</v>
       </c>
       <c r="L8" s="11">
-        <v>21845</v>
+        <v>21844</v>
       </c>
       <c r="M8" s="11">
-        <v>43760</v>
+        <v>43759</v>
       </c>
       <c r="N8" s="13">
         <v>3500</v>
@@ -3895,7 +3895,7 @@
         <v>29</v>
       </c>
       <c r="L12" s="11">
-        <v>22290</v>
+        <v>22291</v>
       </c>
       <c r="M12" s="11">
         <v>44205</v>
@@ -9892,10 +9892,10 @@
         <v>237</v>
       </c>
       <c r="L119" s="11">
-        <v>24366</v>
+        <v>24316</v>
       </c>
       <c r="M119" s="11">
-        <v>46281</v>
+        <v>46231</v>
       </c>
       <c r="N119" s="13"/>
       <c r="O119" s="7" t="s">
@@ -10568,10 +10568,10 @@
         <v>373</v>
       </c>
       <c r="L10" s="11">
-        <v>20381</v>
+        <v>20371</v>
       </c>
       <c r="M10" s="11">
-        <v>42296</v>
+        <v>42286</v>
       </c>
       <c r="N10" s="13">
         <v>2500</v>
@@ -11730,10 +11730,10 @@
         <v>385</v>
       </c>
       <c r="L30" s="11">
-        <v>23563</v>
+        <v>23472</v>
       </c>
       <c r="M30" s="11">
-        <v>45478</v>
+        <v>45387</v>
       </c>
       <c r="N30" s="13">
         <v>3000</v>
@@ -14121,10 +14121,10 @@
         <v>358</v>
       </c>
       <c r="L71" s="11">
-        <v>20179</v>
+        <v>20239</v>
       </c>
       <c r="M71" s="11">
-        <v>42094</v>
+        <v>42093</v>
       </c>
       <c r="N71" s="13">
         <v>3000</v>
@@ -14827,10 +14827,10 @@
         <v>517</v>
       </c>
       <c r="L83" s="11">
-        <v>23244</v>
+        <v>23610</v>
       </c>
       <c r="M83" s="11">
-        <v>45159</v>
+        <v>45525</v>
       </c>
       <c r="N83" s="13">
         <v>3000</v>
@@ -14886,10 +14886,10 @@
         <v>44</v>
       </c>
       <c r="L84" s="11">
-        <v>23513</v>
+        <v>23512</v>
       </c>
       <c r="M84" s="11">
-        <v>45428</v>
+        <v>45427</v>
       </c>
       <c r="N84" s="13">
         <v>3000</v>
@@ -16746,10 +16746,10 @@
         <v>298</v>
       </c>
       <c r="L116" s="11">
-        <v>23425</v>
+        <v>23791</v>
       </c>
       <c r="M116" s="11">
-        <v>45340</v>
+        <v>45706</v>
       </c>
       <c r="N116" s="13">
         <v>3000</v>
@@ -18194,10 +18194,10 @@
         <v>657</v>
       </c>
       <c r="L142" s="11">
-        <v>23575</v>
+        <v>23484</v>
       </c>
       <c r="M142" s="11">
-        <v>45490</v>
+        <v>45399</v>
       </c>
       <c r="N142" s="13">
         <v>3000</v>
@@ -18422,10 +18422,10 @@
         <v>39</v>
       </c>
       <c r="L146" s="11">
-        <v>23975</v>
+        <v>23886</v>
       </c>
       <c r="M146" s="11">
-        <v>45890</v>
+        <v>45801</v>
       </c>
       <c r="N146" s="13">
         <v>2500</v>
@@ -20587,10 +20587,10 @@
         <v>44</v>
       </c>
       <c r="L185" s="11">
-        <v>23203</v>
+        <v>23202</v>
       </c>
       <c r="M185" s="11">
-        <v>45118</v>
+        <v>45117</v>
       </c>
       <c r="N185" s="13">
         <v>3000</v>

</xml_diff>

<commit_message>
auto update (29 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -4009,10 +4009,10 @@
         <v>64</v>
       </c>
       <c r="L14" s="11">
-        <v>22797</v>
+        <v>22796</v>
       </c>
       <c r="M14" s="11">
-        <v>44712</v>
+        <v>44711</v>
       </c>
       <c r="N14" s="13">
         <v>3000</v>
@@ -4063,7 +4063,7 @@
         <v>46361</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="L15" s="11">
         <v>23115</v>
@@ -4177,7 +4177,7 @@
         <v>46363</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>75</v>
+        <v>137</v>
       </c>
       <c r="L17" s="11">
         <v>23832</v>
@@ -4348,7 +4348,7 @@
         <v>46365</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>83</v>
+        <v>35</v>
       </c>
       <c r="L20" s="11">
         <v>23559</v>
@@ -4519,7 +4519,7 @@
         <v>46371</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L23" s="11">
         <v>24277</v>
@@ -4741,13 +4741,13 @@
         <v>45740</v>
       </c>
       <c r="I27" s="11">
-        <v>45924</v>
+        <v>46289</v>
       </c>
       <c r="J27" s="12">
         <v>46379</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="L27" s="11">
         <v>23112</v>
@@ -6508,13 +6508,13 @@
         <v>46399</v>
       </c>
       <c r="K58" s="7" t="s">
-        <v>190</v>
+        <v>35</v>
       </c>
       <c r="L58" s="11">
-        <v>22637</v>
+        <v>22638</v>
       </c>
       <c r="M58" s="11">
-        <v>44552</v>
+        <v>44553</v>
       </c>
       <c r="N58" s="13">
         <v>3000</v>
@@ -6739,10 +6739,10 @@
         <v>201</v>
       </c>
       <c r="L62" s="11">
-        <v>24026</v>
+        <v>24308</v>
       </c>
       <c r="M62" s="11">
-        <v>45941</v>
+        <v>46223</v>
       </c>
       <c r="N62" s="13">
         <v>3000</v>
@@ -7250,10 +7250,10 @@
         <v>224</v>
       </c>
       <c r="L71" s="11">
-        <v>22934</v>
+        <v>22933</v>
       </c>
       <c r="M71" s="11">
-        <v>44849</v>
+        <v>44848</v>
       </c>
       <c r="N71" s="13">
         <v>2500</v>
@@ -7931,7 +7931,7 @@
         <v>46425</v>
       </c>
       <c r="K83" s="7" t="s">
-        <v>259</v>
+        <v>159</v>
       </c>
       <c r="L83" s="11">
         <v>23503</v>
@@ -7988,7 +7988,7 @@
         <v>46425</v>
       </c>
       <c r="K84" s="7" t="s">
-        <v>262</v>
+        <v>244</v>
       </c>
       <c r="L84" s="11">
         <v>23053</v>
@@ -8045,7 +8045,7 @@
         <v>46425</v>
       </c>
       <c r="K85" s="7" t="s">
-        <v>265</v>
+        <v>95</v>
       </c>
       <c r="L85" s="11">
         <v>24123</v>
@@ -8265,7 +8265,7 @@
         <v>45888</v>
       </c>
       <c r="I89" s="11">
-        <v>46253</v>
+        <v>46345</v>
       </c>
       <c r="J89" s="12">
         <v>46436</v>
@@ -8328,7 +8328,7 @@
         <v>46437</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>280</v>
+        <v>219</v>
       </c>
       <c r="L90" s="11">
         <v>23955</v>
@@ -8499,7 +8499,7 @@
         <v>46439</v>
       </c>
       <c r="K93" s="7" t="s">
-        <v>288</v>
+        <v>129</v>
       </c>
       <c r="L93" s="11">
         <v>22479</v>
@@ -8554,7 +8554,7 @@
         <v>46439</v>
       </c>
       <c r="K94" s="7" t="s">
-        <v>291</v>
+        <v>146</v>
       </c>
       <c r="L94" s="11">
         <v>24056</v>
@@ -8671,10 +8671,10 @@
         <v>106</v>
       </c>
       <c r="L96" s="11">
-        <v>24062</v>
+        <v>24261</v>
       </c>
       <c r="M96" s="11">
-        <v>45977</v>
+        <v>46176</v>
       </c>
       <c r="N96" s="13">
         <v>3000</v>
@@ -8779,7 +8779,7 @@
         <v>46104</v>
       </c>
       <c r="J98" s="12">
-        <v>46560</v>
+        <v>46468</v>
       </c>
       <c r="K98" s="7" t="s">
         <v>106</v>
@@ -8839,7 +8839,7 @@
         <v>46568</v>
       </c>
       <c r="K99" s="7" t="s">
-        <v>306</v>
+        <v>95</v>
       </c>
       <c r="L99" s="11">
         <v>22912</v>
@@ -8899,7 +8899,7 @@
         <v>310</v>
       </c>
       <c r="L100" s="11">
-        <v>19207</v>
+        <v>22859</v>
       </c>
       <c r="M100" s="11">
         <v>41122</v>
@@ -9007,7 +9007,7 @@
         <v>46143</v>
       </c>
       <c r="J102" s="12">
-        <v>46599</v>
+        <v>46507</v>
       </c>
       <c r="K102" s="7" t="s">
         <v>317</v>
@@ -9293,7 +9293,7 @@
         <v>46630</v>
       </c>
       <c r="K107" s="7" t="s">
-        <v>330</v>
+        <v>153</v>
       </c>
       <c r="L107" s="11">
         <v>24348</v>

</xml_diff>

<commit_message>
auto update (52 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3667,10 +3667,10 @@
         <v>29</v>
       </c>
       <c r="L8" s="11">
-        <v>21845</v>
+        <v>21844</v>
       </c>
       <c r="M8" s="11">
-        <v>43760</v>
+        <v>43759</v>
       </c>
       <c r="N8" s="13">
         <v>3500</v>
@@ -3895,7 +3895,7 @@
         <v>29</v>
       </c>
       <c r="L12" s="11">
-        <v>22290</v>
+        <v>22291</v>
       </c>
       <c r="M12" s="11">
         <v>44205</v>
@@ -4009,10 +4009,10 @@
         <v>64</v>
       </c>
       <c r="L14" s="11">
-        <v>22797</v>
+        <v>22796</v>
       </c>
       <c r="M14" s="11">
-        <v>44712</v>
+        <v>44711</v>
       </c>
       <c r="N14" s="13">
         <v>3000</v>
@@ -4063,7 +4063,7 @@
         <v>46361</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="L15" s="11">
         <v>23115</v>
@@ -4177,7 +4177,7 @@
         <v>46363</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>75</v>
+        <v>137</v>
       </c>
       <c r="L17" s="11">
         <v>23832</v>
@@ -4348,7 +4348,7 @@
         <v>46365</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>83</v>
+        <v>35</v>
       </c>
       <c r="L20" s="11">
         <v>23559</v>
@@ -4519,7 +4519,7 @@
         <v>46371</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L23" s="11">
         <v>24277</v>
@@ -4741,13 +4741,13 @@
         <v>45740</v>
       </c>
       <c r="I27" s="11">
-        <v>45924</v>
+        <v>46289</v>
       </c>
       <c r="J27" s="12">
         <v>46379</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="L27" s="11">
         <v>23112</v>
@@ -6508,13 +6508,13 @@
         <v>46399</v>
       </c>
       <c r="K58" s="7" t="s">
-        <v>190</v>
+        <v>35</v>
       </c>
       <c r="L58" s="11">
-        <v>22637</v>
+        <v>22638</v>
       </c>
       <c r="M58" s="11">
-        <v>44552</v>
+        <v>44553</v>
       </c>
       <c r="N58" s="13">
         <v>3000</v>
@@ -6739,10 +6739,10 @@
         <v>201</v>
       </c>
       <c r="L62" s="11">
-        <v>24026</v>
+        <v>24308</v>
       </c>
       <c r="M62" s="11">
-        <v>45941</v>
+        <v>46223</v>
       </c>
       <c r="N62" s="13">
         <v>3000</v>
@@ -7250,10 +7250,10 @@
         <v>224</v>
       </c>
       <c r="L71" s="11">
-        <v>22934</v>
+        <v>22933</v>
       </c>
       <c r="M71" s="11">
-        <v>44849</v>
+        <v>44848</v>
       </c>
       <c r="N71" s="13">
         <v>2500</v>
@@ -7931,7 +7931,7 @@
         <v>46425</v>
       </c>
       <c r="K83" s="7" t="s">
-        <v>259</v>
+        <v>159</v>
       </c>
       <c r="L83" s="11">
         <v>23503</v>
@@ -7988,7 +7988,7 @@
         <v>46425</v>
       </c>
       <c r="K84" s="7" t="s">
-        <v>262</v>
+        <v>244</v>
       </c>
       <c r="L84" s="11">
         <v>23053</v>
@@ -8045,7 +8045,7 @@
         <v>46425</v>
       </c>
       <c r="K85" s="7" t="s">
-        <v>265</v>
+        <v>95</v>
       </c>
       <c r="L85" s="11">
         <v>24123</v>
@@ -8265,7 +8265,7 @@
         <v>45888</v>
       </c>
       <c r="I89" s="11">
-        <v>46253</v>
+        <v>46345</v>
       </c>
       <c r="J89" s="12">
         <v>46436</v>
@@ -8328,7 +8328,7 @@
         <v>46437</v>
       </c>
       <c r="K90" s="7" t="s">
-        <v>280</v>
+        <v>219</v>
       </c>
       <c r="L90" s="11">
         <v>23955</v>
@@ -8499,7 +8499,7 @@
         <v>46439</v>
       </c>
       <c r="K93" s="7" t="s">
-        <v>288</v>
+        <v>129</v>
       </c>
       <c r="L93" s="11">
         <v>22479</v>
@@ -8554,7 +8554,7 @@
         <v>46439</v>
       </c>
       <c r="K94" s="7" t="s">
-        <v>291</v>
+        <v>146</v>
       </c>
       <c r="L94" s="11">
         <v>24056</v>
@@ -8671,10 +8671,10 @@
         <v>106</v>
       </c>
       <c r="L96" s="11">
-        <v>24062</v>
+        <v>24261</v>
       </c>
       <c r="M96" s="11">
-        <v>45977</v>
+        <v>46176</v>
       </c>
       <c r="N96" s="13">
         <v>3000</v>
@@ -8779,7 +8779,7 @@
         <v>46104</v>
       </c>
       <c r="J98" s="12">
-        <v>46560</v>
+        <v>46468</v>
       </c>
       <c r="K98" s="7" t="s">
         <v>106</v>
@@ -8839,7 +8839,7 @@
         <v>46568</v>
       </c>
       <c r="K99" s="7" t="s">
-        <v>306</v>
+        <v>95</v>
       </c>
       <c r="L99" s="11">
         <v>22912</v>
@@ -8899,7 +8899,7 @@
         <v>310</v>
       </c>
       <c r="L100" s="11">
-        <v>19207</v>
+        <v>22859</v>
       </c>
       <c r="M100" s="11">
         <v>41122</v>
@@ -9007,7 +9007,7 @@
         <v>46143</v>
       </c>
       <c r="J102" s="12">
-        <v>46599</v>
+        <v>46507</v>
       </c>
       <c r="K102" s="7" t="s">
         <v>317</v>
@@ -9293,7 +9293,7 @@
         <v>46630</v>
       </c>
       <c r="K107" s="7" t="s">
-        <v>330</v>
+        <v>153</v>
       </c>
       <c r="L107" s="11">
         <v>24348</v>
@@ -9892,10 +9892,10 @@
         <v>237</v>
       </c>
       <c r="L119" s="11">
-        <v>24366</v>
+        <v>24316</v>
       </c>
       <c r="M119" s="11">
-        <v>46281</v>
+        <v>46231</v>
       </c>
       <c r="N119" s="13"/>
       <c r="O119" s="7" t="s">
@@ -10568,10 +10568,10 @@
         <v>373</v>
       </c>
       <c r="L10" s="11">
-        <v>20381</v>
+        <v>20371</v>
       </c>
       <c r="M10" s="11">
-        <v>42296</v>
+        <v>42286</v>
       </c>
       <c r="N10" s="13">
         <v>2500</v>
@@ -11730,10 +11730,10 @@
         <v>385</v>
       </c>
       <c r="L30" s="11">
-        <v>23563</v>
+        <v>23472</v>
       </c>
       <c r="M30" s="11">
-        <v>45478</v>
+        <v>45387</v>
       </c>
       <c r="N30" s="13">
         <v>3000</v>
@@ -14121,10 +14121,10 @@
         <v>358</v>
       </c>
       <c r="L71" s="11">
-        <v>20179</v>
+        <v>20239</v>
       </c>
       <c r="M71" s="11">
-        <v>42094</v>
+        <v>42093</v>
       </c>
       <c r="N71" s="13">
         <v>3000</v>
@@ -14827,10 +14827,10 @@
         <v>517</v>
       </c>
       <c r="L83" s="11">
-        <v>23244</v>
+        <v>23610</v>
       </c>
       <c r="M83" s="11">
-        <v>45159</v>
+        <v>45525</v>
       </c>
       <c r="N83" s="13">
         <v>3000</v>
@@ -14886,10 +14886,10 @@
         <v>44</v>
       </c>
       <c r="L84" s="11">
-        <v>23513</v>
+        <v>23512</v>
       </c>
       <c r="M84" s="11">
-        <v>45428</v>
+        <v>45427</v>
       </c>
       <c r="N84" s="13">
         <v>3000</v>
@@ -16746,10 +16746,10 @@
         <v>298</v>
       </c>
       <c r="L116" s="11">
-        <v>23425</v>
+        <v>23791</v>
       </c>
       <c r="M116" s="11">
-        <v>45340</v>
+        <v>45706</v>
       </c>
       <c r="N116" s="13">
         <v>3000</v>
@@ -18194,10 +18194,10 @@
         <v>657</v>
       </c>
       <c r="L142" s="11">
-        <v>23575</v>
+        <v>23484</v>
       </c>
       <c r="M142" s="11">
-        <v>45490</v>
+        <v>45399</v>
       </c>
       <c r="N142" s="13">
         <v>3000</v>
@@ -18422,10 +18422,10 @@
         <v>39</v>
       </c>
       <c r="L146" s="11">
-        <v>23975</v>
+        <v>23886</v>
       </c>
       <c r="M146" s="11">
-        <v>45890</v>
+        <v>45801</v>
       </c>
       <c r="N146" s="13">
         <v>2500</v>
@@ -20587,10 +20587,10 @@
         <v>44</v>
       </c>
       <c r="L185" s="11">
-        <v>23203</v>
+        <v>23202</v>
       </c>
       <c r="M185" s="11">
-        <v>45118</v>
+        <v>45117</v>
       </c>
       <c r="N185" s="13">
         <v>3000</v>

</xml_diff>

<commit_message>
auto update (19 cells, +0, -5)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3375,10 +3375,10 @@
         <v>44648</v>
       </c>
       <c r="I3" s="11">
-        <v>46293</v>
+        <v>46201</v>
       </c>
       <c r="J3" s="12">
-        <v>46383</v>
+        <v>46292</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>29</v>
@@ -3432,10 +3432,10 @@
         <v>44649</v>
       </c>
       <c r="I4" s="11">
-        <v>46294</v>
+        <v>46202</v>
       </c>
       <c r="J4" s="12">
-        <v>46384</v>
+        <v>46293</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>32</v>
@@ -3489,10 +3489,10 @@
         <v>41730</v>
       </c>
       <c r="I5" s="11">
-        <v>46296</v>
+        <v>46204</v>
       </c>
       <c r="J5" s="12">
-        <v>46387</v>
+        <v>46295</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>35</v>
@@ -3546,10 +3546,10 @@
         <v>45874</v>
       </c>
       <c r="I6" s="11">
-        <v>46331</v>
+        <v>46239</v>
       </c>
       <c r="J6" s="12">
-        <v>46422</v>
+        <v>46330</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>39</v>
@@ -4741,7 +4741,7 @@
         <v>45740</v>
       </c>
       <c r="I27" s="11">
-        <v>45924</v>
+        <v>46289</v>
       </c>
       <c r="J27" s="12">
         <v>46379</v>
@@ -5991,10 +5991,10 @@
         <v>44014</v>
       </c>
       <c r="I49" s="11">
-        <v>46328</v>
+        <v>46297</v>
       </c>
       <c r="J49" s="12">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="K49" s="7" t="s">
         <v>29</v>
@@ -8265,7 +8265,7 @@
         <v>45888</v>
       </c>
       <c r="I89" s="11">
-        <v>46253</v>
+        <v>46345</v>
       </c>
       <c r="J89" s="12">
         <v>46436</v>
@@ -8779,7 +8779,7 @@
         <v>46104</v>
       </c>
       <c r="J98" s="12">
-        <v>46560</v>
+        <v>46468</v>
       </c>
       <c r="K98" s="7" t="s">
         <v>106</v>
@@ -9007,7 +9007,7 @@
         <v>46143</v>
       </c>
       <c r="J102" s="12">
-        <v>46599</v>
+        <v>46507</v>
       </c>
       <c r="K102" s="7" t="s">
         <v>317</v>
@@ -9233,7 +9233,7 @@
         <v>46174</v>
       </c>
       <c r="J106" s="12">
-        <v>46630</v>
+        <v>46538</v>
       </c>
       <c r="K106" s="7" t="s">
         <v>29</v>
@@ -9897,9 +9897,11 @@
       <c r="M119" s="11">
         <v>46281</v>
       </c>
-      <c r="N119" s="13"/>
+      <c r="N119" s="13">
+        <v>2500</v>
+      </c>
       <c r="O119" s="7" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
       <c r="P119" s="13">
         <v>26609161301038</v>
@@ -10036,7 +10038,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S265"/>
+  <dimension ref="A1:S260"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -10064,7 +10066,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D189)</f>
-        <v>263</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -10209,10 +10211,10 @@
         <v>45323</v>
       </c>
       <c r="I4" s="11">
-        <v>45505</v>
+        <v>45413</v>
       </c>
       <c r="J4" s="12">
-        <v>45596</v>
+        <v>45504</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>358</v>
@@ -23948,239 +23950,8 @@
       </c>
       <c r="S260" s="7"/>
     </row>
-    <row r="261" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A261" s="7">
-        <v>259</v>
-      </c>
-      <c r="B261" s="7"/>
-      <c r="C261" s="8"/>
-      <c r="D261" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="E261" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F261" s="7" t="s">
-        <v>783</v>
-      </c>
-      <c r="G261" s="7"/>
-      <c r="H261" s="10">
-        <v>44827</v>
-      </c>
-      <c r="I261" s="11">
-        <v>45169</v>
-      </c>
-      <c r="J261" s="12">
-        <v>45169</v>
-      </c>
-      <c r="K261" s="7" t="s">
-        <v>784</v>
-      </c>
-      <c r="L261" s="11"/>
-      <c r="M261" s="11"/>
-      <c r="N261" s="13"/>
-      <c r="O261" s="7"/>
-      <c r="P261" s="13"/>
-      <c r="Q261" s="14"/>
-      <c r="R261" s="15"/>
-      <c r="S261" s="7"/>
-    </row>
-    <row r="262" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A262" s="7">
-        <v>260</v>
-      </c>
-      <c r="B262" s="7">
-        <v>20276</v>
-      </c>
-      <c r="C262" s="8">
-        <v>56</v>
-      </c>
-      <c r="D262" s="9" t="s">
-        <v>350</v>
-      </c>
-      <c r="E262" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F262" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G262" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H262" s="10">
-        <v>45263</v>
-      </c>
-      <c r="I262" s="11">
-        <v>46086</v>
-      </c>
-      <c r="J262" s="12">
-        <v>46450</v>
-      </c>
-      <c r="K262" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L262" s="11">
-        <v>21886</v>
-      </c>
-      <c r="M262" s="11">
-        <v>43801</v>
-      </c>
-      <c r="N262" s="13"/>
-      <c r="O262" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="P262" s="13">
-        <v>25912021300059</v>
-      </c>
-      <c r="Q262" s="14"/>
-      <c r="R262" s="15"/>
-      <c r="S262" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="263" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A263" s="7">
-        <v>261</v>
-      </c>
-      <c r="B263" s="7">
-        <v>20274</v>
-      </c>
-      <c r="C263" s="8">
-        <v>19</v>
-      </c>
-      <c r="D263" s="9" t="s">
-        <v>348</v>
-      </c>
-      <c r="E263" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F263" s="7" t="s">
-        <v>347</v>
-      </c>
-      <c r="G263" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H263" s="10">
-        <v>45139</v>
-      </c>
-      <c r="I263" s="11"/>
-      <c r="J263" s="12"/>
-      <c r="K263" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L263" s="11">
-        <v>22510</v>
-      </c>
-      <c r="M263" s="11">
-        <v>45117</v>
-      </c>
-      <c r="N263" s="13"/>
-      <c r="O263" s="7"/>
-      <c r="P263" s="13">
-        <v>26108171301291</v>
-      </c>
-      <c r="Q263" s="14"/>
-      <c r="R263" s="15"/>
-      <c r="S263" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="264" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A264" s="7">
-        <v>262</v>
-      </c>
-      <c r="B264" s="7">
-        <v>20211</v>
-      </c>
-      <c r="C264" s="8">
-        <v>151</v>
-      </c>
-      <c r="D264" s="9" t="s">
-        <v>351</v>
-      </c>
-      <c r="E264" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F264" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G264" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H264" s="10">
-        <v>44805</v>
-      </c>
-      <c r="I264" s="11"/>
-      <c r="J264" s="12"/>
-      <c r="K264" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L264" s="11">
-        <v>22944</v>
-      </c>
-      <c r="M264" s="11">
-        <v>44859</v>
-      </c>
-      <c r="N264" s="13"/>
-      <c r="O264" s="7"/>
-      <c r="P264" s="13">
-        <v>26210251400258</v>
-      </c>
-      <c r="Q264" s="14"/>
-      <c r="R264" s="15"/>
-      <c r="S264" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="265" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A265" s="7">
-        <v>263</v>
-      </c>
-      <c r="B265" s="7">
-        <v>20212</v>
-      </c>
-      <c r="C265" s="8">
-        <v>152</v>
-      </c>
-      <c r="D265" s="9" t="s">
-        <v>353</v>
-      </c>
-      <c r="E265" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F265" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G265" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H265" s="10">
-        <v>44814</v>
-      </c>
-      <c r="I265" s="11"/>
-      <c r="J265" s="12"/>
-      <c r="K265" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="L265" s="11">
-        <v>21539</v>
-      </c>
-      <c r="M265" s="11">
-        <v>43454</v>
-      </c>
-      <c r="N265" s="13"/>
-      <c r="O265" s="7"/>
-      <c r="P265" s="13">
-        <v>25812208800538</v>
-      </c>
-      <c r="Q265" s="14"/>
-      <c r="R265" s="15"/>
-      <c r="S265" s="7" t="s">
-        <v>349</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:S265"/>
+  <autoFilter ref="A2:S260"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
auto update (6 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -3375,10 +3375,10 @@
         <v>44648</v>
       </c>
       <c r="I3" s="11">
-        <v>46201</v>
+        <v>46293</v>
       </c>
       <c r="J3" s="12">
-        <v>46292</v>
+        <v>46383</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>29</v>
@@ -3432,10 +3432,10 @@
         <v>44649</v>
       </c>
       <c r="I4" s="11">
-        <v>46202</v>
+        <v>46294</v>
       </c>
       <c r="J4" s="12">
-        <v>46293</v>
+        <v>46384</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>32</v>
@@ -3489,10 +3489,10 @@
         <v>41730</v>
       </c>
       <c r="I5" s="11">
-        <v>46204</v>
+        <v>46296</v>
       </c>
       <c r="J5" s="12">
-        <v>46295</v>
+        <v>46387</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
auto update (23 cells, +4, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -6508,7 +6508,7 @@
         <v>46399</v>
       </c>
       <c r="K58" s="7" t="s">
-        <v>190</v>
+        <v>35</v>
       </c>
       <c r="L58" s="11">
         <v>22637</v>
@@ -7310,7 +7310,7 @@
         <v>24309</v>
       </c>
       <c r="M72" s="11">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="N72" s="13">
         <v>3000</v>
@@ -8448,7 +8448,7 @@
         <v>23476</v>
       </c>
       <c r="M92" s="11">
-        <v>46121</v>
+        <v>45391</v>
       </c>
       <c r="N92" s="13">
         <v>3000</v>
@@ -8788,7 +8788,7 @@
         <v>24188</v>
       </c>
       <c r="M98" s="11">
-        <v>60713</v>
+        <v>46103</v>
       </c>
       <c r="N98" s="13">
         <v>10000</v>
@@ -9016,7 +9016,7 @@
         <v>22964</v>
       </c>
       <c r="M102" s="11">
-        <v>44909</v>
+        <v>44879</v>
       </c>
       <c r="N102" s="13">
         <v>10000</v>
@@ -10038,7 +10038,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S260"/>
+  <dimension ref="A1:S264"/>
   <sheetFormatPr defaultRowHeight="35.1" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.57" customWidth="1"/>
@@ -10066,7 +10066,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2">
         <f>COUNTA(D3:D189)</f>
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" ht="36.75" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -10570,10 +10570,10 @@
         <v>373</v>
       </c>
       <c r="L10" s="11">
-        <v>20381</v>
+        <v>20371</v>
       </c>
       <c r="M10" s="11">
-        <v>42296</v>
+        <v>42286</v>
       </c>
       <c r="N10" s="13">
         <v>2500</v>
@@ -11732,10 +11732,10 @@
         <v>385</v>
       </c>
       <c r="L30" s="11">
-        <v>23563</v>
+        <v>23472</v>
       </c>
       <c r="M30" s="11">
-        <v>45478</v>
+        <v>45387</v>
       </c>
       <c r="N30" s="13">
         <v>3000</v>
@@ -14123,10 +14123,10 @@
         <v>358</v>
       </c>
       <c r="L71" s="11">
-        <v>20179</v>
+        <v>20239</v>
       </c>
       <c r="M71" s="11">
-        <v>42094</v>
+        <v>42093</v>
       </c>
       <c r="N71" s="13">
         <v>3000</v>
@@ -14829,10 +14829,10 @@
         <v>517</v>
       </c>
       <c r="L83" s="11">
-        <v>23244</v>
+        <v>23610</v>
       </c>
       <c r="M83" s="11">
-        <v>45159</v>
+        <v>45525</v>
       </c>
       <c r="N83" s="13">
         <v>3000</v>
@@ -14888,10 +14888,10 @@
         <v>44</v>
       </c>
       <c r="L84" s="11">
-        <v>23513</v>
+        <v>23512</v>
       </c>
       <c r="M84" s="11">
-        <v>45428</v>
+        <v>45427</v>
       </c>
       <c r="N84" s="13">
         <v>3000</v>
@@ -16748,10 +16748,10 @@
         <v>298</v>
       </c>
       <c r="L116" s="11">
-        <v>23425</v>
+        <v>23791</v>
       </c>
       <c r="M116" s="11">
-        <v>45340</v>
+        <v>45706</v>
       </c>
       <c r="N116" s="13">
         <v>3000</v>
@@ -18196,10 +18196,10 @@
         <v>657</v>
       </c>
       <c r="L142" s="11">
-        <v>23575</v>
+        <v>23484</v>
       </c>
       <c r="M142" s="11">
-        <v>45490</v>
+        <v>45399</v>
       </c>
       <c r="N142" s="13">
         <v>3000</v>
@@ -18424,10 +18424,10 @@
         <v>39</v>
       </c>
       <c r="L146" s="11">
-        <v>23975</v>
+        <v>23886</v>
       </c>
       <c r="M146" s="11">
-        <v>45890</v>
+        <v>45801</v>
       </c>
       <c r="N146" s="13">
         <v>2500</v>
@@ -20589,10 +20589,10 @@
         <v>44</v>
       </c>
       <c r="L185" s="11">
-        <v>23203</v>
+        <v>23202</v>
       </c>
       <c r="M185" s="11">
-        <v>45118</v>
+        <v>45117</v>
       </c>
       <c r="N185" s="13">
         <v>3000</v>
@@ -23950,8 +23950,178 @@
       </c>
       <c r="S260" s="7"/>
     </row>
+    <row r="261" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A261" s="7">
+        <v>259</v>
+      </c>
+      <c r="B261" s="7">
+        <v>20368</v>
+      </c>
+      <c r="C261" s="8">
+        <v>303</v>
+      </c>
+      <c r="D261" s="9" t="s">
+        <v>662</v>
+      </c>
+      <c r="E261" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F261" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G261" s="7"/>
+      <c r="H261" s="10">
+        <v>45931</v>
+      </c>
+      <c r="I261" s="11">
+        <v>45931</v>
+      </c>
+      <c r="J261" s="12">
+        <v>45931</v>
+      </c>
+      <c r="K261" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="L261" s="11"/>
+      <c r="M261" s="11"/>
+      <c r="N261" s="13"/>
+      <c r="O261" s="7"/>
+      <c r="P261" s="13"/>
+      <c r="Q261" s="14"/>
+      <c r="R261" s="15"/>
+      <c r="S261" s="7" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="262" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A262" s="7">
+        <v>260</v>
+      </c>
+      <c r="B262" s="7">
+        <v>20398</v>
+      </c>
+      <c r="C262" s="8">
+        <v>333</v>
+      </c>
+      <c r="D262" s="9" t="s">
+        <v>669</v>
+      </c>
+      <c r="E262" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F262" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G262" s="7"/>
+      <c r="H262" s="10">
+        <v>46041</v>
+      </c>
+      <c r="I262" s="11">
+        <v>46041</v>
+      </c>
+      <c r="J262" s="12">
+        <v>46041</v>
+      </c>
+      <c r="K262" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="L262" s="11"/>
+      <c r="M262" s="11"/>
+      <c r="N262" s="13"/>
+      <c r="O262" s="7"/>
+      <c r="P262" s="13"/>
+      <c r="Q262" s="14"/>
+      <c r="R262" s="15"/>
+      <c r="S262" s="7" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="263" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A263" s="7">
+        <v>261</v>
+      </c>
+      <c r="B263" s="7">
+        <v>342</v>
+      </c>
+      <c r="C263" s="8"/>
+      <c r="D263" s="9" t="s">
+        <v>677</v>
+      </c>
+      <c r="E263" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F263" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G263" s="7"/>
+      <c r="H263" s="10">
+        <v>46057</v>
+      </c>
+      <c r="I263" s="11">
+        <v>46057</v>
+      </c>
+      <c r="J263" s="12">
+        <v>46057</v>
+      </c>
+      <c r="K263" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="L263" s="11"/>
+      <c r="M263" s="11"/>
+      <c r="N263" s="13"/>
+      <c r="O263" s="7"/>
+      <c r="P263" s="13"/>
+      <c r="Q263" s="14"/>
+      <c r="R263" s="15"/>
+      <c r="S263" s="7" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="264" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A264" s="7">
+        <v>262</v>
+      </c>
+      <c r="B264" s="7">
+        <v>20411</v>
+      </c>
+      <c r="C264" s="8">
+        <v>346</v>
+      </c>
+      <c r="D264" s="9" t="s">
+        <v>694</v>
+      </c>
+      <c r="E264" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F264" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G264" s="7"/>
+      <c r="H264" s="10">
+        <v>46069</v>
+      </c>
+      <c r="I264" s="11">
+        <v>46069</v>
+      </c>
+      <c r="J264" s="12">
+        <v>46069</v>
+      </c>
+      <c r="K264" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="L264" s="11"/>
+      <c r="M264" s="11"/>
+      <c r="N264" s="13"/>
+      <c r="O264" s="7"/>
+      <c r="P264" s="13"/>
+      <c r="Q264" s="14"/>
+      <c r="R264" s="15"/>
+      <c r="S264" s="7" t="s">
+        <v>908</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S260"/>
+  <autoFilter ref="A2:S264"/>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>

</xml_diff>

<commit_message>
auto update (18 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -10570,10 +10570,10 @@
         <v>373</v>
       </c>
       <c r="L10" s="11">
-        <v>20371</v>
+        <v>20381</v>
       </c>
       <c r="M10" s="11">
-        <v>42286</v>
+        <v>42296</v>
       </c>
       <c r="N10" s="13">
         <v>2500</v>
@@ -11732,10 +11732,10 @@
         <v>385</v>
       </c>
       <c r="L30" s="11">
-        <v>23472</v>
+        <v>23563</v>
       </c>
       <c r="M30" s="11">
-        <v>45387</v>
+        <v>45478</v>
       </c>
       <c r="N30" s="13">
         <v>3000</v>
@@ -14123,10 +14123,10 @@
         <v>358</v>
       </c>
       <c r="L71" s="11">
-        <v>20239</v>
+        <v>20179</v>
       </c>
       <c r="M71" s="11">
-        <v>42093</v>
+        <v>42094</v>
       </c>
       <c r="N71" s="13">
         <v>3000</v>
@@ -14829,10 +14829,10 @@
         <v>517</v>
       </c>
       <c r="L83" s="11">
-        <v>23610</v>
+        <v>23244</v>
       </c>
       <c r="M83" s="11">
-        <v>45525</v>
+        <v>45159</v>
       </c>
       <c r="N83" s="13">
         <v>3000</v>
@@ -14888,10 +14888,10 @@
         <v>44</v>
       </c>
       <c r="L84" s="11">
-        <v>23512</v>
+        <v>23513</v>
       </c>
       <c r="M84" s="11">
-        <v>45427</v>
+        <v>45428</v>
       </c>
       <c r="N84" s="13">
         <v>3000</v>
@@ -16748,10 +16748,10 @@
         <v>298</v>
       </c>
       <c r="L116" s="11">
-        <v>23791</v>
+        <v>23425</v>
       </c>
       <c r="M116" s="11">
-        <v>45706</v>
+        <v>45340</v>
       </c>
       <c r="N116" s="13">
         <v>3000</v>
@@ -18196,10 +18196,10 @@
         <v>657</v>
       </c>
       <c r="L142" s="11">
-        <v>23484</v>
+        <v>23575</v>
       </c>
       <c r="M142" s="11">
-        <v>45399</v>
+        <v>45490</v>
       </c>
       <c r="N142" s="13">
         <v>3000</v>
@@ -18424,10 +18424,10 @@
         <v>39</v>
       </c>
       <c r="L146" s="11">
-        <v>23886</v>
+        <v>23975</v>
       </c>
       <c r="M146" s="11">
-        <v>45801</v>
+        <v>45890</v>
       </c>
       <c r="N146" s="13">
         <v>2500</v>
@@ -20589,10 +20589,10 @@
         <v>44</v>
       </c>
       <c r="L185" s="11">
-        <v>23202</v>
+        <v>23203</v>
       </c>
       <c r="M185" s="11">
-        <v>45117</v>
+        <v>45118</v>
       </c>
       <c r="N185" s="13">
         <v>3000</v>

</xml_diff>

<commit_message>
auto update (18 cells, +1, -1)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="915">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2507" uniqueCount="916">
   <si>
     <t xml:space="preserve">الاجمالى </t>
   </si>
@@ -2757,6 +2757,9 @@
   </si>
   <si>
     <t xml:space="preserve">محت فوكيه ناشد سلمون</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مدحت فوكيه ناشد سلمون</t>
   </si>
 </sst>
 </file>
@@ -9990,7 +9993,7 @@
     </row>
     <row r="122" ht="35.1" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A122" s="7">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B122" s="7">
         <v>20441</v>
@@ -9999,7 +10002,7 @@
         <v>913</v>
       </c>
       <c r="D122" s="9" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="E122" s="7" t="s">
         <v>20</v>
@@ -10570,10 +10573,10 @@
         <v>373</v>
       </c>
       <c r="L10" s="11">
-        <v>20381</v>
+        <v>20371</v>
       </c>
       <c r="M10" s="11">
-        <v>42296</v>
+        <v>42286</v>
       </c>
       <c r="N10" s="13">
         <v>2500</v>
@@ -11732,10 +11735,10 @@
         <v>385</v>
       </c>
       <c r="L30" s="11">
-        <v>23563</v>
+        <v>23472</v>
       </c>
       <c r="M30" s="11">
-        <v>45478</v>
+        <v>45387</v>
       </c>
       <c r="N30" s="13">
         <v>3000</v>
@@ -14123,10 +14126,10 @@
         <v>358</v>
       </c>
       <c r="L71" s="11">
-        <v>20179</v>
+        <v>20239</v>
       </c>
       <c r="M71" s="11">
-        <v>42094</v>
+        <v>42093</v>
       </c>
       <c r="N71" s="13">
         <v>3000</v>
@@ -14829,10 +14832,10 @@
         <v>517</v>
       </c>
       <c r="L83" s="11">
-        <v>23244</v>
+        <v>23610</v>
       </c>
       <c r="M83" s="11">
-        <v>45159</v>
+        <v>45525</v>
       </c>
       <c r="N83" s="13">
         <v>3000</v>
@@ -14888,10 +14891,10 @@
         <v>44</v>
       </c>
       <c r="L84" s="11">
-        <v>23513</v>
+        <v>23512</v>
       </c>
       <c r="M84" s="11">
-        <v>45428</v>
+        <v>45427</v>
       </c>
       <c r="N84" s="13">
         <v>3000</v>
@@ -16748,10 +16751,10 @@
         <v>298</v>
       </c>
       <c r="L116" s="11">
-        <v>23425</v>
+        <v>23791</v>
       </c>
       <c r="M116" s="11">
-        <v>45340</v>
+        <v>45706</v>
       </c>
       <c r="N116" s="13">
         <v>3000</v>
@@ -18196,10 +18199,10 @@
         <v>657</v>
       </c>
       <c r="L142" s="11">
-        <v>23575</v>
+        <v>23484</v>
       </c>
       <c r="M142" s="11">
-        <v>45490</v>
+        <v>45399</v>
       </c>
       <c r="N142" s="13">
         <v>3000</v>
@@ -18424,10 +18427,10 @@
         <v>39</v>
       </c>
       <c r="L146" s="11">
-        <v>23975</v>
+        <v>23886</v>
       </c>
       <c r="M146" s="11">
-        <v>45890</v>
+        <v>45801</v>
       </c>
       <c r="N146" s="13">
         <v>2500</v>
@@ -20589,10 +20592,10 @@
         <v>44</v>
       </c>
       <c r="L185" s="11">
-        <v>23203</v>
+        <v>23202</v>
       </c>
       <c r="M185" s="11">
-        <v>45118</v>
+        <v>45117</v>
       </c>
       <c r="N185" s="13">
         <v>3000</v>

</xml_diff>

<commit_message>
auto update (20 cells, +0, -0)
</commit_message>
<xml_diff>
--- a/metro-contact.xlsx
+++ b/metro-contact.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2507" uniqueCount="916">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2509" uniqueCount="918">
   <si>
     <t xml:space="preserve">الاجمالى </t>
   </si>
@@ -2760,6 +2760,12 @@
   </si>
   <si>
     <t xml:space="preserve">مدحت فوكيه ناشد سلمون</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الإشارات الخط الاول</t>
+  </si>
+  <si>
+    <t xml:space="preserve">٣٣ش ترعة الجلاد _بجوار مستشفي شبرا شبرا _ القاهرة</t>
   </si>
 </sst>
 </file>
@@ -10016,14 +10022,18 @@
       <c r="H122" s="10"/>
       <c r="I122" s="11"/>
       <c r="J122" s="12"/>
-      <c r="K122" s="7"/>
+      <c r="K122" s="7" t="s">
+        <v>916</v>
+      </c>
       <c r="L122" s="11"/>
       <c r="M122" s="11"/>
       <c r="N122" s="13"/>
       <c r="O122" s="7"/>
       <c r="P122" s="13"/>
       <c r="Q122" s="16"/>
-      <c r="R122" s="15"/>
+      <c r="R122" s="15" t="s">
+        <v>917</v>
+      </c>
       <c r="S122" s="7"/>
     </row>
   </sheetData>
@@ -10573,10 +10583,10 @@
         <v>373</v>
       </c>
       <c r="L10" s="11">
-        <v>20381</v>
+        <v>20371</v>
       </c>
       <c r="M10" s="11">
-        <v>42296</v>
+        <v>42286</v>
       </c>
       <c r="N10" s="13">
         <v>2500</v>
@@ -11735,10 +11745,10 @@
         <v>385</v>
       </c>
       <c r="L30" s="11">
-        <v>23563</v>
+        <v>23472</v>
       </c>
       <c r="M30" s="11">
-        <v>45478</v>
+        <v>45387</v>
       </c>
       <c r="N30" s="13">
         <v>3000</v>
@@ -14126,10 +14136,10 @@
         <v>358</v>
       </c>
       <c r="L71" s="11">
-        <v>20179</v>
+        <v>20239</v>
       </c>
       <c r="M71" s="11">
-        <v>42094</v>
+        <v>42093</v>
       </c>
       <c r="N71" s="13">
         <v>3000</v>
@@ -14832,10 +14842,10 @@
         <v>517</v>
       </c>
       <c r="L83" s="11">
-        <v>23244</v>
+        <v>23610</v>
       </c>
       <c r="M83" s="11">
-        <v>45159</v>
+        <v>45525</v>
       </c>
       <c r="N83" s="13">
         <v>3000</v>
@@ -14891,10 +14901,10 @@
         <v>44</v>
       </c>
       <c r="L84" s="11">
-        <v>23513</v>
+        <v>23512</v>
       </c>
       <c r="M84" s="11">
-        <v>45428</v>
+        <v>45427</v>
       </c>
       <c r="N84" s="13">
         <v>3000</v>
@@ -16751,10 +16761,10 @@
         <v>298</v>
       </c>
       <c r="L116" s="11">
-        <v>23425</v>
+        <v>23791</v>
       </c>
       <c r="M116" s="11">
-        <v>45340</v>
+        <v>45706</v>
       </c>
       <c r="N116" s="13">
         <v>3000</v>
@@ -18199,10 +18209,10 @@
         <v>657</v>
       </c>
       <c r="L142" s="11">
-        <v>23575</v>
+        <v>23484</v>
       </c>
       <c r="M142" s="11">
-        <v>45490</v>
+        <v>45399</v>
       </c>
       <c r="N142" s="13">
         <v>3000</v>
@@ -18427,10 +18437,10 @@
         <v>39</v>
       </c>
       <c r="L146" s="11">
-        <v>23975</v>
+        <v>23886</v>
       </c>
       <c r="M146" s="11">
-        <v>45890</v>
+        <v>45801</v>
       </c>
       <c r="N146" s="13">
         <v>2500</v>
@@ -20592,10 +20602,10 @@
         <v>44</v>
       </c>
       <c r="L185" s="11">
-        <v>23203</v>
+        <v>23202</v>
       </c>
       <c r="M185" s="11">
-        <v>45118</v>
+        <v>45117</v>
       </c>
       <c r="N185" s="13">
         <v>3000</v>

</xml_diff>